<commit_message>
Full backup 09/06/2026 10:36:57
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -835,7 +835,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="24"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="24"/>
   </cellStyleXfs>
-  <cellXfs count="312">
+  <cellXfs count="318">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1650,6 +1650,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="12" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="12" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="12" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="13" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="13" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="13" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2785,9 +2803,7 @@
         <f>IF(G13=0,"-",H13/G13)</f>
         <v/>
       </c>
-      <c r="K13" s="304" t="n">
-        <v>90048</v>
-      </c>
+      <c r="K13" s="304" t="n"/>
       <c r="L13" s="306" t="inlineStr">
         <is>
           <t>120k Order, 89k Advance Production</t>
@@ -2973,22 +2989,23 @@
       </c>
       <c r="C16" s="300" t="inlineStr">
         <is>
-          <t>Habib Hanif Inc</t>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
       <c r="D16" s="301" t="inlineStr">
         <is>
-          <t>S-45</t>
+          <t>HELLO HAIR COLOR</t>
         </is>
       </c>
       <c r="E16" s="302" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F16" s="303" t="n">
-        <v>5389</v>
-      </c>
-      <c r="G16" s="303" t="n">
-        <v>0</v>
+        <v>6206</v>
+      </c>
+      <c r="G16" s="303">
+        <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F16,MRP!$D$3:$D$9,0)),0)</f>
+        <v/>
       </c>
       <c r="H16" s="304">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F16)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
@@ -3002,10 +3019,12 @@
         <f>IF(G16=0,"-",H16/G16)</f>
         <v/>
       </c>
-      <c r="K16" s="304" t="n">
-        <v>44352</v>
-      </c>
-      <c r="L16" s="306" t="n"/>
+      <c r="K16" s="304" t="n"/>
+      <c r="L16" s="306" t="inlineStr">
+        <is>
+          <t>Advance Production</t>
+        </is>
+      </c>
       <c r="M16" s="151" t="n"/>
       <c r="N16" s="151" t="n"/>
       <c r="O16" s="151" t="n"/>
@@ -3043,19 +3062,19 @@
       </c>
       <c r="C17" s="300" t="inlineStr">
         <is>
-          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+          <t>Mablay Beauty PVT LTD.</t>
         </is>
       </c>
       <c r="D17" s="301" t="inlineStr">
         <is>
-          <t>HELLO HAIR COLOR</t>
+          <t>VINCE NURTURAL</t>
         </is>
       </c>
       <c r="E17" s="302" t="n">
         <v>30</v>
       </c>
       <c r="F17" s="303" t="n">
-        <v>6206</v>
+        <v>5814</v>
       </c>
       <c r="G17" s="303">
         <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F17,MRP!$D$3:$D$9,0)),0)</f>
@@ -3074,11 +3093,7 @@
         <v/>
       </c>
       <c r="K17" s="304" t="n"/>
-      <c r="L17" s="306" t="inlineStr">
-        <is>
-          <t>Advance Production</t>
-        </is>
-      </c>
+      <c r="L17" s="306" t="n"/>
       <c r="P17" s="151" t="n"/>
       <c r="Q17" s="151" t="n"/>
       <c r="R17" s="151" t="n"/>
@@ -3103,19 +3118,19 @@
       </c>
       <c r="C18" s="300" t="inlineStr">
         <is>
-          <t>Mablay Beauty PVT LTD.</t>
+          <t>Adore</t>
         </is>
       </c>
       <c r="D18" s="301" t="inlineStr">
         <is>
-          <t>VINCE NURTURAL</t>
+          <t>V- HC BROWN</t>
         </is>
       </c>
       <c r="E18" s="302" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F18" s="303" t="n">
-        <v>5814</v>
+        <v>6530</v>
       </c>
       <c r="G18" s="303">
         <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F18,MRP!$D$3:$D$9,0)),0)</f>
@@ -3134,7 +3149,11 @@
         <v/>
       </c>
       <c r="K18" s="304" t="n"/>
-      <c r="L18" s="306" t="n"/>
+      <c r="L18" s="306" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hold </t>
+        </is>
+      </c>
       <c r="P18" s="151" t="n"/>
       <c r="Q18" s="151" t="n"/>
       <c r="R18" s="151" t="n"/>
@@ -3162,49 +3181,33 @@
     </row>
     <row r="19" ht="16.5" customHeight="1" s="254">
       <c r="A19" s="151" t="n"/>
-      <c r="B19" s="299" t="inlineStr">
-        <is>
-          <t>TUBE</t>
-        </is>
-      </c>
-      <c r="C19" s="300" t="inlineStr">
-        <is>
-          <t>Adore</t>
-        </is>
-      </c>
-      <c r="D19" s="301" t="inlineStr">
-        <is>
-          <t>V- HC BROWN</t>
-        </is>
-      </c>
-      <c r="E19" s="302" t="n">
-        <v>35</v>
-      </c>
-      <c r="F19" s="303" t="n">
-        <v>6530</v>
-      </c>
-      <c r="G19" s="303">
-        <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F19,MRP!$D$3:$D$9,0)),0)</f>
-        <v/>
-      </c>
-      <c r="H19" s="304">
-        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F19)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
-        <v/>
-      </c>
-      <c r="I19" s="303">
-        <f>G19-H19</f>
-        <v/>
-      </c>
-      <c r="J19" s="305">
-        <f>IF(G19=0,"-",H19/G19)</f>
-        <v/>
-      </c>
-      <c r="K19" s="304" t="n"/>
-      <c r="L19" s="306" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hold </t>
-        </is>
-      </c>
+      <c r="B19" s="307" t="n"/>
+      <c r="C19" s="308" t="n"/>
+      <c r="D19" s="309" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E19" s="307" t="n"/>
+      <c r="F19" s="308" t="n"/>
+      <c r="G19" s="310">
+        <f>SUM(G11:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="310">
+        <f>SUM(H11:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="310">
+        <f>SUMIF(I11:I18,"&gt;"&amp;0)</f>
+        <v/>
+      </c>
+      <c r="J19" s="310" t="n"/>
+      <c r="K19" s="310">
+        <f>SUM(K11:K18)</f>
+        <v/>
+      </c>
+      <c r="L19" s="310" t="n"/>
       <c r="M19" s="151" t="n"/>
       <c r="N19" s="151" t="n"/>
       <c r="O19" s="151" t="n"/>
@@ -3235,33 +3238,46 @@
     </row>
     <row r="20" ht="16.5" customHeight="1" s="254">
       <c r="A20" s="151" t="n"/>
-      <c r="B20" s="307" t="n"/>
-      <c r="C20" s="308" t="n"/>
-      <c r="D20" s="309" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E20" s="307" t="n"/>
-      <c r="F20" s="308" t="n"/>
-      <c r="G20" s="310">
-        <f>SUM(G11:G19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="310">
-        <f>SUM(H11:H19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="310">
-        <f>SUMIF(I11:I19,"&gt;"&amp;0)</f>
-        <v/>
-      </c>
-      <c r="J20" s="310" t="n"/>
-      <c r="K20" s="310">
-        <f>SUM(K11:K19)</f>
-        <v/>
-      </c>
-      <c r="L20" s="310" t="n"/>
+      <c r="B20" s="299" t="inlineStr">
+        <is>
+          <t>PET</t>
+        </is>
+      </c>
+      <c r="C20" s="300" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D20" s="301" t="inlineStr">
+        <is>
+          <t>PET BOTTLE SMALL (120ML) YELLOW</t>
+        </is>
+      </c>
+      <c r="E20" s="302" t="inlineStr">
+        <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="F20" s="303" t="n">
+        <v>8005</v>
+      </c>
+      <c r="G20" s="303" t="n">
+        <v>19840</v>
+      </c>
+      <c r="H20" s="304">
+        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F20)*Production_Log!$H$3:$H$8963)</f>
+        <v/>
+      </c>
+      <c r="I20" s="303">
+        <f>G20-H20</f>
+        <v/>
+      </c>
+      <c r="J20" s="305">
+        <f>IF(G20=0,"-",H20/G20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="304" t="n"/>
+      <c r="L20" s="306" t="n"/>
       <c r="M20" s="151" t="n"/>
       <c r="N20" s="151" t="n"/>
       <c r="O20" s="151" t="n"/>
@@ -3287,24 +3303,24 @@
       </c>
       <c r="C21" s="300" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
       <c r="D21" s="301" t="inlineStr">
         <is>
-          <t>PET BOTTLE SMALL (120ML) YELLOW</t>
+          <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
       <c r="E21" s="302" t="inlineStr">
         <is>
-          <t>120 ml</t>
+          <t>150 ml</t>
         </is>
       </c>
       <c r="F21" s="303" t="n">
-        <v>8005</v>
+        <v>8001</v>
       </c>
       <c r="G21" s="303" t="n">
-        <v>19840</v>
+        <v>249997</v>
       </c>
       <c r="H21" s="304">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F21)*Production_Log!$H$3:$H$8963)</f>
@@ -3345,24 +3361,24 @@
       </c>
       <c r="C22" s="300" t="inlineStr">
         <is>
-          <t>Alpha Labs PVT LTD</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D22" s="301" t="inlineStr">
         <is>
-          <t>TRANSPARENT BOTTLE 150ML</t>
+          <t>PET BOTTLE LARGE 200ML WHITE</t>
         </is>
       </c>
       <c r="E22" s="302" t="inlineStr">
         <is>
-          <t>150 ml</t>
+          <t>200 ml</t>
         </is>
       </c>
       <c r="F22" s="303" t="n">
-        <v>8001</v>
+        <v>8007</v>
       </c>
       <c r="G22" s="303" t="n">
-        <v>249997</v>
+        <v>10000</v>
       </c>
       <c r="H22" s="304">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F22)*Production_Log!$H$3:$H$8963)</f>
@@ -3376,9 +3392,7 @@
         <f>IF(G22=0,"-",H22/G22)</f>
         <v/>
       </c>
-      <c r="K22" s="304" t="n">
-        <v>32200</v>
-      </c>
+      <c r="K22" s="304" t="n"/>
       <c r="L22" s="306" t="n"/>
       <c r="M22" s="151" t="n"/>
       <c r="N22" s="151" t="n"/>
@@ -3410,7 +3424,7 @@
       </c>
       <c r="D23" s="301" t="inlineStr">
         <is>
-          <t>PET BOTTLE LARGE 200ML WHITE</t>
+          <t>BT-200 ML YELLOW</t>
         </is>
       </c>
       <c r="E23" s="302" t="inlineStr">
@@ -3419,10 +3433,10 @@
         </is>
       </c>
       <c r="F23" s="303" t="n">
-        <v>8007</v>
+        <v>8006</v>
       </c>
       <c r="G23" s="303" t="n">
-        <v>10000</v>
+        <v>42400</v>
       </c>
       <c r="H23" s="304">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F23)*Production_Log!$H$3:$H$8963)</f>
@@ -3468,7 +3482,7 @@
       </c>
       <c r="D24" s="301" t="inlineStr">
         <is>
-          <t>BT-200 ML YELLOW</t>
+          <t>BT-200ML MUSTARD OIL (TRANSPARENT)</t>
         </is>
       </c>
       <c r="E24" s="302" t="inlineStr">
@@ -3477,10 +3491,10 @@
         </is>
       </c>
       <c r="F24" s="303" t="n">
-        <v>8006</v>
+        <v>8014</v>
       </c>
       <c r="G24" s="303" t="n">
-        <v>42400</v>
+        <v>10000</v>
       </c>
       <c r="H24" s="304">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F24)*Production_Log!$H$3:$H$8963)</f>
@@ -3516,46 +3530,33 @@
     </row>
     <row r="25" ht="16.5" customHeight="1" s="254">
       <c r="A25" s="151" t="n"/>
-      <c r="B25" s="299" t="inlineStr">
-        <is>
-          <t>PET</t>
-        </is>
-      </c>
-      <c r="C25" s="300" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D25" s="301" t="inlineStr">
-        <is>
-          <t>BT-200ML MUSTARD OIL (TRANSPARENT)</t>
-        </is>
-      </c>
-      <c r="E25" s="302" t="inlineStr">
-        <is>
-          <t>200 ml</t>
-        </is>
-      </c>
-      <c r="F25" s="303" t="n">
-        <v>8014</v>
-      </c>
-      <c r="G25" s="303" t="n">
-        <v>10000</v>
-      </c>
-      <c r="H25" s="304">
-        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F25)*Production_Log!$H$3:$H$8963)</f>
-        <v/>
-      </c>
-      <c r="I25" s="303">
-        <f>G25-H25</f>
-        <v/>
-      </c>
-      <c r="J25" s="305">
-        <f>IF(G25=0,"-",H25/G25)</f>
-        <v/>
-      </c>
-      <c r="K25" s="304" t="n"/>
-      <c r="L25" s="306" t="n"/>
+      <c r="B25" s="307" t="n"/>
+      <c r="C25" s="308" t="n"/>
+      <c r="D25" s="309" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E25" s="307" t="n"/>
+      <c r="F25" s="308" t="n"/>
+      <c r="G25" s="310">
+        <f>SUM(G20:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="310">
+        <f>SUM(H20:H24)</f>
+        <v/>
+      </c>
+      <c r="I25" s="310">
+        <f>SUMIF(I20:I24,"&gt;"&amp;0)</f>
+        <v/>
+      </c>
+      <c r="J25" s="310" t="n"/>
+      <c r="K25" s="310">
+        <f>SUM(K20:K24)</f>
+        <v/>
+      </c>
+      <c r="L25" s="310" t="n"/>
       <c r="M25" s="151" t="n"/>
       <c r="N25" s="151" t="n"/>
       <c r="O25" s="151" t="n"/>
@@ -3576,33 +3577,44 @@
     </row>
     <row r="26" ht="16.5" customHeight="1" s="254">
       <c r="A26" s="151" t="n"/>
-      <c r="B26" s="307" t="n"/>
-      <c r="C26" s="308" t="n"/>
-      <c r="D26" s="309" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E26" s="307" t="n"/>
-      <c r="F26" s="308" t="n"/>
-      <c r="G26" s="310">
-        <f>SUM(G21:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="310">
-        <f>SUM(H21:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="310">
-        <f>SUMIF(I21:I25,"&gt;"&amp;0)</f>
-        <v/>
-      </c>
-      <c r="J26" s="310" t="n"/>
-      <c r="K26" s="310">
-        <f>SUM(K21:K25)</f>
-        <v/>
-      </c>
-      <c r="L26" s="310" t="n"/>
+      <c r="B26" s="299" t="inlineStr">
+        <is>
+          <t>TUBE</t>
+        </is>
+      </c>
+      <c r="C26" s="300" t="inlineStr">
+        <is>
+          <t>Bahadur</t>
+        </is>
+      </c>
+      <c r="D26" s="301" t="inlineStr">
+        <is>
+          <t>BAHADUR TUBE 12.5MM</t>
+        </is>
+      </c>
+      <c r="E26" s="302" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F26" s="303" t="n">
+        <v>9004</v>
+      </c>
+      <c r="G26" s="303" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="304">
+        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F26)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
+        <v/>
+      </c>
+      <c r="I26" s="303">
+        <f>G26-H26</f>
+        <v/>
+      </c>
+      <c r="J26" s="305">
+        <f>IF(G26=0,"-",H26/G26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="304" t="n"/>
+      <c r="L26" s="306" t="n"/>
       <c r="M26" s="151" t="n"/>
       <c r="N26" s="151" t="n"/>
       <c r="O26" s="151" t="n"/>
@@ -3630,19 +3642,19 @@
       </c>
       <c r="C27" s="300" t="inlineStr">
         <is>
-          <t>Bahadur</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D27" s="301" t="inlineStr">
         <is>
-          <t>BAHADUR TUBE 12.5MM</t>
+          <t>S-45 DIA 19MM</t>
         </is>
       </c>
       <c r="E27" s="302" t="n">
-        <v>12.5</v>
+        <v>19</v>
       </c>
       <c r="F27" s="303" t="n">
-        <v>9004</v>
+        <v>6624</v>
       </c>
       <c r="G27" s="303" t="n">
         <v>0</v>
@@ -3693,14 +3705,14 @@
       </c>
       <c r="D28" s="301" t="inlineStr">
         <is>
-          <t>S-45 DIA 19MM</t>
+          <t>S-43 DIA 19MM</t>
         </is>
       </c>
       <c r="E28" s="302" t="n">
         <v>19</v>
       </c>
       <c r="F28" s="303" t="n">
-        <v>6624</v>
+        <v>6623</v>
       </c>
       <c r="G28" s="303" t="n">
         <v>0</v>
@@ -3744,19 +3756,19 @@
       </c>
       <c r="C29" s="300" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Brookes Pharma Private Limited</t>
         </is>
       </c>
       <c r="D29" s="301" t="inlineStr">
         <is>
-          <t>S-43 DIA 19MM</t>
+          <t>PHLOGIN GEL 20G</t>
         </is>
       </c>
       <c r="E29" s="302" t="n">
         <v>19</v>
       </c>
       <c r="F29" s="303" t="n">
-        <v>6623</v>
+        <v>6559</v>
       </c>
       <c r="G29" s="303" t="n">
         <v>0</v>
@@ -3805,14 +3817,14 @@
       </c>
       <c r="D30" s="301" t="inlineStr">
         <is>
-          <t>PHLOGIN GEL 20G</t>
+          <t>PYODINE GEL 20GM</t>
         </is>
       </c>
       <c r="E30" s="302" t="n">
         <v>19</v>
       </c>
       <c r="F30" s="303" t="n">
-        <v>6559</v>
+        <v>1085</v>
       </c>
       <c r="G30" s="303" t="n">
         <v>0</v>
@@ -3863,14 +3875,14 @@
       </c>
       <c r="D31" s="301" t="inlineStr">
         <is>
-          <t>PYODINE GEL 20GM</t>
+          <t>CONTRATUBEX GEL 20G</t>
         </is>
       </c>
       <c r="E31" s="302" t="n">
         <v>19</v>
       </c>
       <c r="F31" s="303" t="n">
-        <v>1085</v>
+        <v>6560</v>
       </c>
       <c r="G31" s="303" t="n">
         <v>0</v>
@@ -3916,19 +3928,19 @@
       </c>
       <c r="C32" s="300" t="inlineStr">
         <is>
-          <t>Brookes Pharma Private Limited</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D32" s="301" t="inlineStr">
         <is>
-          <t>CONTRATUBEX GEL 20G</t>
+          <t>S-43 DIA 20.5</t>
         </is>
       </c>
       <c r="E32" s="302" t="n">
-        <v>19</v>
+        <v>20.5</v>
       </c>
       <c r="F32" s="303" t="n">
-        <v>6560</v>
+        <v>5699</v>
       </c>
       <c r="G32" s="303" t="n">
         <v>0</v>
@@ -3974,19 +3986,19 @@
       </c>
       <c r="C33" s="300" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Mablay Beauty PVT LTD.</t>
         </is>
       </c>
       <c r="D33" s="301" t="inlineStr">
         <is>
-          <t>S-43 DIA 20.5</t>
+          <t>VINCE HIS ONLY BEARD &amp; MUSTACHE COLOR CREAM</t>
         </is>
       </c>
       <c r="E33" s="302" t="n">
         <v>20.5</v>
       </c>
       <c r="F33" s="303" t="n">
-        <v>5699</v>
+        <v>6077</v>
       </c>
       <c r="G33" s="303" t="n">
         <v>0</v>
@@ -4030,19 +4042,19 @@
       </c>
       <c r="C34" s="300" t="inlineStr">
         <is>
-          <t>Mablay Beauty PVT LTD.</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D34" s="301" t="inlineStr">
         <is>
-          <t>VINCE HIS ONLY BEARD &amp; MUSTACHE COLOR CREAM</t>
+          <t>S-45 DIA 20.5</t>
         </is>
       </c>
       <c r="E34" s="302" t="n">
         <v>20.5</v>
       </c>
       <c r="F34" s="303" t="n">
-        <v>6077</v>
+        <v>5698</v>
       </c>
       <c r="G34" s="303" t="n">
         <v>0</v>
@@ -4091,14 +4103,14 @@
       </c>
       <c r="D35" s="301" t="inlineStr">
         <is>
-          <t>S-45 DIA 20.5</t>
+          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
       <c r="E35" s="302" t="n">
         <v>20.5</v>
       </c>
       <c r="F35" s="303" t="n">
-        <v>5698</v>
+        <v>5731</v>
       </c>
       <c r="G35" s="303" t="n">
         <v>0</v>
@@ -4147,14 +4159,14 @@
       </c>
       <c r="D36" s="301" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
+          <t>SAMSOL HAIR COLOR 43 DIA 20.5 MM</t>
         </is>
       </c>
       <c r="E36" s="302" t="n">
         <v>20.5</v>
       </c>
       <c r="F36" s="303" t="n">
-        <v>5731</v>
+        <v>5732</v>
       </c>
       <c r="G36" s="303" t="n">
         <v>0</v>
@@ -4212,14 +4224,14 @@
       </c>
       <c r="D37" s="301" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 43 DIA 20.5 MM</t>
+          <t>SAMSOL HAIR COLOR 39 SMALL PURPLE</t>
         </is>
       </c>
       <c r="E37" s="302" t="n">
         <v>20.5</v>
       </c>
       <c r="F37" s="303" t="n">
-        <v>5732</v>
+        <v>6556</v>
       </c>
       <c r="G37" s="303" t="n">
         <v>0</v>
@@ -4270,14 +4282,14 @@
       </c>
       <c r="D38" s="301" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 39 SMALL PURPLE</t>
+          <t>SAMSOL HAIR COLOR 41 SMALL PURPLE</t>
         </is>
       </c>
       <c r="E38" s="302" t="n">
         <v>20.5</v>
       </c>
       <c r="F38" s="303" t="n">
-        <v>6556</v>
+        <v>6557</v>
       </c>
       <c r="G38" s="303" t="n">
         <v>0</v>
@@ -4323,19 +4335,19 @@
       </c>
       <c r="C39" s="300" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Habib Hanif Inc</t>
         </is>
       </c>
       <c r="D39" s="301" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 41 SMALL PURPLE</t>
+          <t>S-45</t>
         </is>
       </c>
       <c r="E39" s="302" t="n">
-        <v>20.5</v>
+        <v>25</v>
       </c>
       <c r="F39" s="303" t="n">
-        <v>6557</v>
+        <v>5389</v>
       </c>
       <c r="G39" s="303" t="n">
         <v>0</v>
@@ -32554,13 +32566,15 @@
         <v>0</v>
       </c>
       <c r="G7" s="52" t="n">
-        <v>0</v>
+        <v>525</v>
       </c>
       <c r="H7" s="53">
         <f>E7+F7-G7</f>
         <v/>
       </c>
-      <c r="I7" s="52" t="n"/>
+      <c r="I7" s="52" t="n">
+        <v>75</v>
+      </c>
       <c r="J7" s="52">
         <f>IFERROR(IF(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])=0,"-",ROUND((H7+I7)/(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])/1000),0)),"-")</f>
         <v/>
@@ -34001,10 +34015,10 @@
         <v>0</v>
       </c>
       <c r="F44" s="52" t="n">
-        <v>38000</v>
+        <v>23000</v>
       </c>
       <c r="G44" s="52" t="n">
-        <v>38000</v>
+        <v>0</v>
       </c>
       <c r="H44" s="53">
         <f>E44+F44-G44</f>
@@ -34794,7 +34808,7 @@
         <v>0</v>
       </c>
       <c r="G62" s="52" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H62" s="53">
         <f>E62+F62-G62</f>
@@ -34838,7 +34852,7 @@
         <v>0</v>
       </c>
       <c r="G63" s="52" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H63" s="53">
         <f>E63+F63-G63</f>
@@ -34926,7 +34940,7 @@
         <v>0</v>
       </c>
       <c r="G65" s="52" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H65" s="53">
         <f>E65+F65-G65</f>
@@ -35497,7 +35511,7 @@
         <v>4</v>
       </c>
       <c r="F78" s="52" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G78" s="52" t="n">
         <v>0</v>
@@ -35667,10 +35681,10 @@
         <v>0</v>
       </c>
       <c r="F82" s="52" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G82" s="52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H82" s="53">
         <f>E82+F82-G82</f>
@@ -35702,13 +35716,13 @@
         </is>
       </c>
       <c r="E83" s="52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F83" s="52" t="n">
+        <v>2</v>
+      </c>
+      <c r="G83" s="52" t="n">
         <v>0</v>
-      </c>
-      <c r="G83" s="52" t="n">
-        <v>1</v>
       </c>
       <c r="H83" s="53">
         <f>E83+F83-G83</f>
@@ -36225,7 +36239,7 @@
         <v>0</v>
       </c>
       <c r="G98" s="52" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="H98" s="53">
         <f>E98+F98-G98</f>
@@ -36815,7 +36829,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="52" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H113" s="53">
         <f>E113+F113-G113</f>
@@ -42161,172 +42175,348 @@
       <c r="S42" s="276" t="n"/>
     </row>
     <row r="43" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A43" s="191" t="n"/>
-      <c r="B43" s="192" t="n"/>
-      <c r="C43" s="192" t="n"/>
-      <c r="D43" s="192" t="n"/>
-      <c r="E43" s="192" t="n"/>
-      <c r="F43" s="192" t="n"/>
-      <c r="G43" s="193" t="n"/>
-      <c r="H43" s="193" t="n"/>
-      <c r="I43" s="193" t="n"/>
-      <c r="J43" s="194" t="n"/>
-      <c r="K43" s="192" t="n"/>
-      <c r="L43" s="192" t="n"/>
-      <c r="M43" s="192" t="n"/>
-      <c r="N43" s="192" t="n"/>
-      <c r="O43" s="192" t="n"/>
-      <c r="P43" s="192" t="n"/>
-      <c r="Q43" s="192" t="n"/>
-      <c r="R43" s="192" t="n"/>
-      <c r="S43" s="192" t="n"/>
+      <c r="A43" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B43" s="276" t="inlineStr">
+        <is>
+          <t>Lacquer-02</t>
+        </is>
+      </c>
+      <c r="C43" s="276" t="inlineStr"/>
+      <c r="D43" s="276" t="inlineStr"/>
+      <c r="E43" s="276" t="inlineStr"/>
+      <c r="F43" s="276" t="n"/>
+      <c r="G43" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="278">
+        <f>IFERROR(I43/(H43+I43),"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="276" t="n"/>
+      <c r="L43" s="276" t="n"/>
+      <c r="M43" s="276" t="n"/>
+      <c r="N43" s="276" t="n"/>
+      <c r="O43" s="276" t="n"/>
+      <c r="P43" s="276" t="n"/>
+      <c r="Q43" s="276" t="n"/>
+      <c r="R43" s="276" t="n"/>
+      <c r="S43" s="276" t="n"/>
     </row>
     <row r="44" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A44" s="191" t="n"/>
-      <c r="B44" s="192" t="n"/>
-      <c r="C44" s="192" t="n"/>
-      <c r="D44" s="192" t="n"/>
-      <c r="E44" s="192" t="n"/>
-      <c r="F44" s="192" t="n"/>
-      <c r="G44" s="193" t="n"/>
-      <c r="H44" s="193" t="n"/>
-      <c r="I44" s="193" t="n"/>
-      <c r="J44" s="194" t="n"/>
-      <c r="K44" s="192" t="n"/>
-      <c r="L44" s="192" t="n"/>
-      <c r="M44" s="192" t="n"/>
-      <c r="N44" s="192" t="n"/>
-      <c r="O44" s="192" t="n"/>
-      <c r="P44" s="192" t="n"/>
-      <c r="Q44" s="192" t="n"/>
-      <c r="R44" s="192" t="n"/>
-      <c r="S44" s="192" t="n"/>
+      <c r="A44" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B44" s="276" t="inlineStr">
+        <is>
+          <t>Lacquer-04</t>
+        </is>
+      </c>
+      <c r="C44" s="276" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D44" s="276" t="inlineStr">
+        <is>
+          <t>TUBES COMMON RED</t>
+        </is>
+      </c>
+      <c r="E44" s="276" t="n">
+        <v>25</v>
+      </c>
+      <c r="F44" s="276" t="n">
+        <v>6470</v>
+      </c>
+      <c r="G44" s="277" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H44" s="277" t="n">
+        <v>20735</v>
+      </c>
+      <c r="I44" s="277" t="n">
+        <v>265</v>
+      </c>
+      <c r="J44" s="278">
+        <f>IFERROR(I44/(H44+I44),"")</f>
+        <v/>
+      </c>
+      <c r="K44" s="276" t="n"/>
+      <c r="L44" s="276" t="n"/>
+      <c r="M44" s="276" t="n"/>
+      <c r="N44" s="276" t="n"/>
+      <c r="O44" s="276" t="n"/>
+      <c r="P44" s="276" t="n"/>
+      <c r="Q44" s="276" t="n"/>
+      <c r="R44" s="276" t="n"/>
+      <c r="S44" s="276" t="n"/>
     </row>
     <row r="45" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A45" s="191" t="n"/>
-      <c r="B45" s="192" t="n"/>
-      <c r="C45" s="192" t="n"/>
-      <c r="D45" s="192" t="n"/>
-      <c r="E45" s="192" t="n"/>
-      <c r="F45" s="192" t="n"/>
-      <c r="G45" s="193" t="n"/>
-      <c r="H45" s="193" t="n"/>
-      <c r="I45" s="193" t="n"/>
-      <c r="J45" s="194" t="n"/>
-      <c r="K45" s="192" t="n"/>
-      <c r="L45" s="192" t="n"/>
-      <c r="M45" s="192" t="n"/>
-      <c r="N45" s="192" t="n"/>
-      <c r="O45" s="192" t="n"/>
-      <c r="P45" s="192" t="n"/>
-      <c r="Q45" s="192" t="n"/>
-      <c r="R45" s="192" t="n"/>
-      <c r="S45" s="192" t="n"/>
+      <c r="A45" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B45" s="276" t="inlineStr">
+        <is>
+          <t>Latex-01</t>
+        </is>
+      </c>
+      <c r="C45" s="276" t="inlineStr"/>
+      <c r="D45" s="276" t="inlineStr"/>
+      <c r="E45" s="276" t="inlineStr"/>
+      <c r="F45" s="276" t="n"/>
+      <c r="G45" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="278">
+        <f>IFERROR(I45/(H45+I45),"")</f>
+        <v/>
+      </c>
+      <c r="K45" s="276" t="n"/>
+      <c r="L45" s="276" t="n"/>
+      <c r="M45" s="276" t="n"/>
+      <c r="N45" s="276" t="n"/>
+      <c r="O45" s="276" t="n"/>
+      <c r="P45" s="276" t="n"/>
+      <c r="Q45" s="276" t="n"/>
+      <c r="R45" s="276" t="n"/>
+      <c r="S45" s="276" t="n"/>
     </row>
     <row r="46" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A46" s="191" t="n"/>
-      <c r="B46" s="192" t="n"/>
-      <c r="C46" s="192" t="n"/>
-      <c r="D46" s="192" t="n"/>
-      <c r="E46" s="192" t="n"/>
-      <c r="F46" s="192" t="n"/>
-      <c r="G46" s="193" t="n"/>
-      <c r="H46" s="193" t="n"/>
-      <c r="I46" s="193" t="n"/>
-      <c r="J46" s="194" t="n"/>
-      <c r="K46" s="192" t="n"/>
-      <c r="L46" s="192" t="n"/>
-      <c r="M46" s="192" t="n"/>
-      <c r="N46" s="192" t="n"/>
-      <c r="O46" s="192" t="n"/>
-      <c r="P46" s="192" t="n"/>
-      <c r="Q46" s="192" t="n"/>
-      <c r="R46" s="192" t="n"/>
-      <c r="S46" s="192" t="n"/>
+      <c r="A46" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B46" s="276" t="inlineStr">
+        <is>
+          <t>PF Machine</t>
+        </is>
+      </c>
+      <c r="C46" s="276" t="inlineStr">
+        <is>
+          <t>Alpha Labs PVT LTD</t>
+        </is>
+      </c>
+      <c r="D46" s="276" t="inlineStr">
+        <is>
+          <t>TRANSPARENT BOTTLE 150ML</t>
+        </is>
+      </c>
+      <c r="E46" s="276" t="inlineStr">
+        <is>
+          <t>150 ml</t>
+        </is>
+      </c>
+      <c r="F46" s="276" t="n">
+        <v>8001</v>
+      </c>
+      <c r="G46" s="277" t="n">
+        <v>4080</v>
+      </c>
+      <c r="H46" s="277" t="n">
+        <v>3680</v>
+      </c>
+      <c r="I46" s="277" t="n">
+        <v>400</v>
+      </c>
+      <c r="J46" s="278">
+        <f>IFERROR(I46/(H46+I46),"")</f>
+        <v/>
+      </c>
+      <c r="K46" s="276" t="n">
+        <v>150</v>
+      </c>
+      <c r="L46" s="276" t="n">
+        <v>210</v>
+      </c>
+      <c r="M46" s="276" t="n"/>
+      <c r="N46" s="276" t="n"/>
+      <c r="O46" s="276" t="n"/>
+      <c r="P46" s="276" t="n"/>
+      <c r="Q46" s="276" t="n"/>
+      <c r="R46" s="276" t="n"/>
+      <c r="S46" s="276" t="n"/>
     </row>
     <row r="47" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A47" s="191" t="n"/>
-      <c r="B47" s="192" t="n"/>
-      <c r="C47" s="192" t="n"/>
-      <c r="D47" s="192" t="n"/>
-      <c r="E47" s="192" t="n"/>
-      <c r="F47" s="192" t="n"/>
-      <c r="G47" s="193" t="n"/>
-      <c r="H47" s="193" t="n"/>
-      <c r="I47" s="193" t="n"/>
-      <c r="J47" s="194" t="n"/>
-      <c r="K47" s="192" t="n"/>
-      <c r="L47" s="192" t="n"/>
-      <c r="M47" s="192" t="n"/>
-      <c r="N47" s="192" t="n"/>
-      <c r="O47" s="192" t="n"/>
-      <c r="P47" s="192" t="n"/>
-      <c r="Q47" s="192" t="n"/>
-      <c r="R47" s="192" t="n"/>
-      <c r="S47" s="192" t="n"/>
+      <c r="A47" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B47" s="276" t="inlineStr">
+        <is>
+          <t>Press-04</t>
+        </is>
+      </c>
+      <c r="C47" s="276" t="inlineStr"/>
+      <c r="D47" s="276" t="inlineStr"/>
+      <c r="E47" s="276" t="inlineStr"/>
+      <c r="F47" s="276" t="n"/>
+      <c r="G47" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="278">
+        <f>IFERROR(I47/(H47+I47),"")</f>
+        <v/>
+      </c>
+      <c r="K47" s="276" t="n"/>
+      <c r="L47" s="276" t="n"/>
+      <c r="M47" s="276" t="n"/>
+      <c r="N47" s="276" t="n"/>
+      <c r="O47" s="276" t="n"/>
+      <c r="P47" s="276" t="n"/>
+      <c r="Q47" s="276" t="n"/>
+      <c r="R47" s="276" t="n"/>
+      <c r="S47" s="276" t="n"/>
     </row>
     <row r="48" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A48" s="191" t="n"/>
-      <c r="B48" s="192" t="n"/>
-      <c r="C48" s="192" t="n"/>
-      <c r="D48" s="192" t="n"/>
-      <c r="E48" s="192" t="n"/>
-      <c r="F48" s="192" t="n"/>
-      <c r="G48" s="193" t="n"/>
-      <c r="H48" s="193" t="n"/>
-      <c r="I48" s="193" t="n"/>
-      <c r="J48" s="194" t="n"/>
-      <c r="K48" s="192" t="n"/>
-      <c r="L48" s="192" t="n"/>
-      <c r="M48" s="192" t="n"/>
-      <c r="N48" s="192" t="n"/>
-      <c r="O48" s="192" t="n"/>
-      <c r="P48" s="192" t="n"/>
-      <c r="Q48" s="192" t="n"/>
-      <c r="R48" s="192" t="n"/>
-      <c r="S48" s="192" t="n"/>
+      <c r="A48" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B48" s="276" t="inlineStr">
+        <is>
+          <t>Press-06</t>
+        </is>
+      </c>
+      <c r="C48" s="276" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D48" s="276" t="inlineStr">
+        <is>
+          <t>TUBES COMMON RED</t>
+        </is>
+      </c>
+      <c r="E48" s="276" t="n">
+        <v>25</v>
+      </c>
+      <c r="F48" s="276" t="n">
+        <v>6470</v>
+      </c>
+      <c r="G48" s="277" t="n">
+        <v>24000</v>
+      </c>
+      <c r="H48" s="277" t="n">
+        <v>23850</v>
+      </c>
+      <c r="I48" s="277" t="n">
+        <v>150</v>
+      </c>
+      <c r="J48" s="278">
+        <f>IFERROR(I48/(H48+I48),"")</f>
+        <v/>
+      </c>
+      <c r="K48" s="276" t="n"/>
+      <c r="L48" s="276" t="n"/>
+      <c r="M48" s="276" t="n"/>
+      <c r="N48" s="276" t="n"/>
+      <c r="O48" s="276" t="n"/>
+      <c r="P48" s="276" t="n"/>
+      <c r="Q48" s="276" t="n"/>
+      <c r="R48" s="276" t="n"/>
+      <c r="S48" s="276" t="n"/>
     </row>
     <row r="49" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A49" s="191" t="n"/>
-      <c r="B49" s="192" t="n"/>
-      <c r="C49" s="192" t="n"/>
-      <c r="D49" s="192" t="n"/>
-      <c r="E49" s="192" t="n"/>
-      <c r="F49" s="192" t="n"/>
-      <c r="G49" s="193" t="n"/>
-      <c r="H49" s="193" t="n"/>
-      <c r="I49" s="193" t="n"/>
-      <c r="J49" s="194" t="n"/>
-      <c r="K49" s="192" t="n"/>
-      <c r="L49" s="192" t="n"/>
-      <c r="M49" s="192" t="n"/>
-      <c r="N49" s="192" t="n"/>
-      <c r="O49" s="192" t="n"/>
-      <c r="P49" s="192" t="n"/>
-      <c r="Q49" s="192" t="n"/>
-      <c r="R49" s="192" t="n"/>
-      <c r="S49" s="192" t="n"/>
+      <c r="A49" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B49" s="276" t="inlineStr">
+        <is>
+          <t>Printing-03</t>
+        </is>
+      </c>
+      <c r="C49" s="276" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D49" s="276" t="inlineStr">
+        <is>
+          <t>TUBES COMMON RED</t>
+        </is>
+      </c>
+      <c r="E49" s="276" t="n">
+        <v>25</v>
+      </c>
+      <c r="F49" s="276" t="n">
+        <v>6470</v>
+      </c>
+      <c r="G49" s="277" t="n">
+        <v>15816</v>
+      </c>
+      <c r="H49" s="277" t="n">
+        <v>15456</v>
+      </c>
+      <c r="I49" s="277" t="n">
+        <v>360</v>
+      </c>
+      <c r="J49" s="278">
+        <f>IFERROR(I49/(H49+I49),"")</f>
+        <v/>
+      </c>
+      <c r="K49" s="276" t="n"/>
+      <c r="L49" s="276" t="n"/>
+      <c r="M49" s="276" t="n">
+        <v>120</v>
+      </c>
+      <c r="N49" s="276" t="n"/>
+      <c r="O49" s="276" t="n"/>
+      <c r="P49" s="276" t="n"/>
+      <c r="Q49" s="276" t="n"/>
+      <c r="R49" s="276" t="n"/>
+      <c r="S49" s="276" t="n"/>
     </row>
     <row r="50" hidden="1" ht="15" customHeight="1" s="254">
-      <c r="A50" s="191" t="n"/>
-      <c r="B50" s="192" t="n"/>
-      <c r="C50" s="192" t="n"/>
-      <c r="D50" s="192" t="n"/>
-      <c r="E50" s="192" t="n"/>
-      <c r="F50" s="192" t="n"/>
-      <c r="G50" s="193" t="n"/>
-      <c r="H50" s="193" t="n"/>
-      <c r="I50" s="193" t="n"/>
-      <c r="J50" s="194" t="n"/>
-      <c r="K50" s="192" t="n"/>
-      <c r="L50" s="192" t="n"/>
-      <c r="M50" s="192" t="n"/>
-      <c r="N50" s="192" t="n"/>
-      <c r="O50" s="192" t="n"/>
-      <c r="P50" s="192" t="n"/>
-      <c r="Q50" s="192" t="n"/>
-      <c r="R50" s="192" t="n"/>
-      <c r="S50" s="192" t="n"/>
+      <c r="A50" s="285" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B50" s="276" t="inlineStr">
+        <is>
+          <t>Printing-04</t>
+        </is>
+      </c>
+      <c r="C50" s="276" t="inlineStr"/>
+      <c r="D50" s="276" t="inlineStr"/>
+      <c r="E50" s="276" t="inlineStr"/>
+      <c r="F50" s="276" t="n"/>
+      <c r="G50" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="278">
+        <f>IFERROR(I50/(H50+I50),"")</f>
+        <v/>
+      </c>
+      <c r="K50" s="276" t="n"/>
+      <c r="L50" s="276" t="n"/>
+      <c r="M50" s="276" t="n"/>
+      <c r="N50" s="276" t="n"/>
+      <c r="O50" s="276" t="n"/>
+      <c r="P50" s="276" t="n"/>
+      <c r="Q50" s="276" t="n"/>
+      <c r="R50" s="276" t="n"/>
+      <c r="S50" s="276" t="n"/>
     </row>
     <row r="51" hidden="1" ht="15" customHeight="1" s="254">
       <c r="A51" s="191" t="n"/>
@@ -49820,7 +50010,7 @@
     <row r="1" ht="30" customHeight="1" s="254">
       <c r="A1" s="280" t="inlineStr">
         <is>
-          <t>FG STOCK IN HAND — Last Updated: 08-Jun-2026</t>
+          <t>FG STOCK IN HAND — Last Updated: 09-Jun-2026</t>
         </is>
       </c>
     </row>
@@ -49879,31 +50069,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="254">
-      <c r="A4" s="286" t="n">
+      <c r="A4" s="312" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="286" t="n">
+      <c r="B4" s="312" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="287" t="inlineStr">
+      <c r="C4" s="313" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="287" t="inlineStr">
+      <c r="D4" s="313" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="286" t="inlineStr">
+      <c r="E4" s="312" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="288" t="n">
-        <v>28060</v>
-      </c>
-      <c r="G4" s="286" t="inlineStr">
+      <c r="F4" s="314" t="n">
+        <v>31740</v>
+      </c>
+      <c r="G4" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49919,31 +50109,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="254">
-      <c r="A5" s="286" t="n">
+      <c r="A5" s="312" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="286" t="n">
+      <c r="B5" s="312" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="287" t="inlineStr">
+      <c r="C5" s="313" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="287" t="inlineStr">
+      <c r="D5" s="313" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="286" t="inlineStr">
+      <c r="E5" s="312" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="288" t="n">
+      <c r="F5" s="314" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="286" t="inlineStr">
+      <c r="G5" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49959,31 +50149,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="254">
-      <c r="A6" s="286" t="n">
+      <c r="A6" s="312" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="286" t="n">
+      <c r="B6" s="312" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="287" t="inlineStr">
+      <c r="C6" s="313" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="287" t="inlineStr">
+      <c r="D6" s="313" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="286" t="inlineStr">
+      <c r="E6" s="312" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="288" t="n">
+      <c r="F6" s="314" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="286" t="inlineStr">
+      <c r="G6" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49999,31 +50189,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="254">
-      <c r="A7" s="286" t="n">
+      <c r="A7" s="312" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="286" t="n">
-        <v>4050</v>
-      </c>
-      <c r="C7" s="287" t="inlineStr">
-        <is>
-          <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
-        </is>
-      </c>
-      <c r="D7" s="287" t="inlineStr">
-        <is>
-          <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
-        </is>
-      </c>
-      <c r="E7" s="286" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="F7" s="288" t="n">
-        <v>9450</v>
-      </c>
-      <c r="G7" s="286" t="inlineStr">
+      <c r="B7" s="312" t="n">
+        <v>6470</v>
+      </c>
+      <c r="C7" s="313" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D7" s="313" t="inlineStr">
+        <is>
+          <t>TUBES COMMON RED</t>
+        </is>
+      </c>
+      <c r="E7" s="312" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F7" s="314" t="n">
+        <v>15456</v>
+      </c>
+      <c r="G7" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50039,31 +50229,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="254">
-      <c r="A8" s="286" t="n">
+      <c r="A8" s="312" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="286" t="n">
-        <v>6337</v>
-      </c>
-      <c r="C8" s="287" t="inlineStr">
-        <is>
-          <t>Al-Rehman Group</t>
-        </is>
-      </c>
-      <c r="D8" s="287" t="inlineStr">
-        <is>
-          <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
-        </is>
-      </c>
-      <c r="E8" s="286" t="inlineStr">
+      <c r="B8" s="312" t="n">
+        <v>4050</v>
+      </c>
+      <c r="C8" s="313" t="inlineStr">
+        <is>
+          <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
+        </is>
+      </c>
+      <c r="D8" s="313" t="inlineStr">
+        <is>
+          <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
+        </is>
+      </c>
+      <c r="E8" s="312" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="288" t="n">
-        <v>15680</v>
-      </c>
-      <c r="G8" s="286" t="inlineStr">
+      <c r="F8" s="314" t="n">
+        <v>9450</v>
+      </c>
+      <c r="G8" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50079,31 +50269,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="254">
-      <c r="A9" s="286" t="n">
+      <c r="A9" s="312" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="286" t="n">
-        <v>6416</v>
-      </c>
-      <c r="C9" s="287" t="inlineStr">
+      <c r="B9" s="312" t="n">
+        <v>6337</v>
+      </c>
+      <c r="C9" s="313" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="287" t="inlineStr">
-        <is>
-          <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
-        </is>
-      </c>
-      <c r="E9" s="286" t="inlineStr">
+      <c r="D9" s="313" t="inlineStr">
+        <is>
+          <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
+        </is>
+      </c>
+      <c r="E9" s="312" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="288" t="n">
-        <v>15435</v>
-      </c>
-      <c r="G9" s="286" t="inlineStr">
+      <c r="F9" s="314" t="n">
+        <v>15680</v>
+      </c>
+      <c r="G9" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50119,31 +50309,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="254">
-      <c r="A10" s="286" t="n">
+      <c r="A10" s="312" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="286" t="n">
-        <v>5782</v>
-      </c>
-      <c r="C10" s="287" t="inlineStr">
-        <is>
-          <t>Mega Grey</t>
-        </is>
-      </c>
-      <c r="D10" s="287" t="inlineStr">
-        <is>
-          <t>M.G</t>
-        </is>
-      </c>
-      <c r="E10" s="286" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F10" s="288" t="n">
-        <v>63648</v>
-      </c>
-      <c r="G10" s="286" t="inlineStr">
+      <c r="B10" s="312" t="n">
+        <v>6416</v>
+      </c>
+      <c r="C10" s="313" t="inlineStr">
+        <is>
+          <t>Al-Rehman Group</t>
+        </is>
+      </c>
+      <c r="D10" s="313" t="inlineStr">
+        <is>
+          <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
+        </is>
+      </c>
+      <c r="E10" s="312" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F10" s="314" t="n">
+        <v>15435</v>
+      </c>
+      <c r="G10" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50159,31 +50349,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="254">
-      <c r="A11" s="286" t="n">
+      <c r="A11" s="312" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="286" t="n">
-        <v>6531</v>
-      </c>
-      <c r="C11" s="287" t="inlineStr">
-        <is>
-          <t>Adore</t>
-        </is>
-      </c>
-      <c r="D11" s="287" t="inlineStr">
-        <is>
-          <t>V-HC BLACK</t>
-        </is>
-      </c>
-      <c r="E11" s="286" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F11" s="288" t="n">
-        <v>4380</v>
-      </c>
-      <c r="G11" s="286" t="inlineStr">
+      <c r="B11" s="312" t="n">
+        <v>5782</v>
+      </c>
+      <c r="C11" s="313" t="inlineStr">
+        <is>
+          <t>Mega Grey</t>
+        </is>
+      </c>
+      <c r="D11" s="313" t="inlineStr">
+        <is>
+          <t>M.G</t>
+        </is>
+      </c>
+      <c r="E11" s="312" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F11" s="314" t="n">
+        <v>63648</v>
+      </c>
+      <c r="G11" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50199,38 +50389,38 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="254">
-      <c r="A12" s="286" t="n">
+      <c r="A12" s="312" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="286" t="n">
-        <v>6206</v>
-      </c>
-      <c r="C12" s="287" t="inlineStr">
-        <is>
-          <t>Golden Pearl Cosmetics (PVT) LTD</t>
-        </is>
-      </c>
-      <c r="D12" s="287" t="inlineStr">
-        <is>
-          <t>HELLO HAIR COLOR</t>
-        </is>
-      </c>
-      <c r="E12" s="286" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="F12" s="288" t="n">
-        <v>35000</v>
-      </c>
-      <c r="G12" s="286" t="inlineStr">
+      <c r="B12" s="312" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C12" s="313" t="inlineStr">
+        <is>
+          <t>Adore</t>
+        </is>
+      </c>
+      <c r="D12" s="313" t="inlineStr">
+        <is>
+          <t>V-HC BLACK</t>
+        </is>
+      </c>
+      <c r="E12" s="312" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F12" s="314" t="n">
+        <v>4380</v>
+      </c>
+      <c r="G12" s="312" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H12" s="289" t="inlineStr">
         <is>
-          <t>No JOF</t>
+          <t>Ready for dispatch</t>
         </is>
       </c>
       <c r="I12" s="109">
@@ -50239,38 +50429,38 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="254">
-      <c r="A13" s="290" t="n">
+      <c r="A13" s="312" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="290" t="n">
-        <v>6515</v>
-      </c>
-      <c r="C13" s="291" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D13" s="291" t="inlineStr">
-        <is>
-          <t>H.H 100GM</t>
-        </is>
-      </c>
-      <c r="E13" s="290" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F13" s="292" t="n">
-        <v>38896</v>
-      </c>
-      <c r="G13" s="290" t="inlineStr">
-        <is>
-          <t>Not Ready</t>
-        </is>
-      </c>
-      <c r="H13" s="293" t="inlineStr">
-        <is>
-          <t>To be dispatch after packing</t>
+      <c r="B13" s="312" t="n">
+        <v>6206</v>
+      </c>
+      <c r="C13" s="313" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D13" s="313" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E13" s="312" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F13" s="314" t="n">
+        <v>75000</v>
+      </c>
+      <c r="G13" s="312" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H13" s="289" t="inlineStr">
+        <is>
+          <t>No JOF</t>
         </is>
       </c>
       <c r="I13" s="109">
@@ -50279,31 +50469,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="254">
-      <c r="A14" s="290" t="n">
+      <c r="A14" s="315" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="290" t="n">
-        <v>6530</v>
-      </c>
-      <c r="C14" s="291" t="inlineStr">
-        <is>
-          <t>Adore</t>
-        </is>
-      </c>
-      <c r="D14" s="291" t="inlineStr">
-        <is>
-          <t>V- HC BROWN</t>
-        </is>
-      </c>
-      <c r="E14" s="290" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F14" s="292" t="n">
-        <v>15000</v>
-      </c>
-      <c r="G14" s="290" t="inlineStr">
+      <c r="B14" s="315" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C14" s="316" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D14" s="316" t="inlineStr">
+        <is>
+          <t>H.H 100GM</t>
+        </is>
+      </c>
+      <c r="E14" s="315" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F14" s="317" t="n">
+        <v>38896</v>
+      </c>
+      <c r="G14" s="315" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50319,31 +50509,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="254">
-      <c r="A15" s="290" t="n">
+      <c r="A15" s="315" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="290" t="n">
-        <v>6206</v>
-      </c>
-      <c r="C15" s="291" t="inlineStr">
-        <is>
-          <t>Golden Pearl Cosmetics (PVT) LTD</t>
-        </is>
-      </c>
-      <c r="D15" s="291" t="inlineStr">
-        <is>
-          <t>HELLO HAIR COLOR</t>
-        </is>
-      </c>
-      <c r="E15" s="290" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="F15" s="292" t="n">
-        <v>63674</v>
-      </c>
-      <c r="G15" s="290" t="inlineStr">
+      <c r="B15" s="315" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C15" s="316" t="inlineStr">
+        <is>
+          <t>Adore</t>
+        </is>
+      </c>
+      <c r="D15" s="316" t="inlineStr">
+        <is>
+          <t>V- HC BROWN</t>
+        </is>
+      </c>
+      <c r="E15" s="315" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F15" s="317" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G15" s="315" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50359,38 +50549,38 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="254">
-      <c r="A16" s="290" t="n">
+      <c r="A16" s="315" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="290" t="n">
-        <v>5782</v>
-      </c>
-      <c r="C16" s="291" t="inlineStr">
-        <is>
-          <t>Mega Grey</t>
-        </is>
-      </c>
-      <c r="D16" s="291" t="inlineStr">
-        <is>
-          <t>M.G</t>
-        </is>
-      </c>
-      <c r="E16" s="290" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F16" s="292" t="n">
-        <v>10500</v>
-      </c>
-      <c r="G16" s="290" t="inlineStr">
+      <c r="B16" s="315" t="n">
+        <v>6206</v>
+      </c>
+      <c r="C16" s="316" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D16" s="316" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E16" s="315" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F16" s="317" t="n">
+        <v>23674</v>
+      </c>
+      <c r="G16" s="315" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
       </c>
       <c r="H16" s="293" t="inlineStr">
         <is>
-          <t>Cap Not Available</t>
+          <t>To be dispatch after packing</t>
         </is>
       </c>
       <c r="I16" s="110">
@@ -50399,31 +50589,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="254">
-      <c r="A17" s="290" t="n">
+      <c r="A17" s="315" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="290" t="n">
-        <v>6624</v>
-      </c>
-      <c r="C17" s="291" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D17" s="291" t="inlineStr">
-        <is>
-          <t>S-45 DIA 19MM</t>
-        </is>
-      </c>
-      <c r="E17" s="290" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="F17" s="292" t="n">
-        <v>15288</v>
-      </c>
-      <c r="G17" s="290" t="inlineStr">
+      <c r="B17" s="315" t="n">
+        <v>5782</v>
+      </c>
+      <c r="C17" s="316" t="inlineStr">
+        <is>
+          <t>Mega Grey</t>
+        </is>
+      </c>
+      <c r="D17" s="316" t="inlineStr">
+        <is>
+          <t>M.G</t>
+        </is>
+      </c>
+      <c r="E17" s="315" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F17" s="317" t="n">
+        <v>10500</v>
+      </c>
+      <c r="G17" s="315" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50439,31 +50629,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="254">
-      <c r="A18" s="290" t="n">
+      <c r="A18" s="315" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="290" t="n">
-        <v>5731</v>
-      </c>
-      <c r="C18" s="291" t="inlineStr">
+      <c r="B18" s="315" t="n">
+        <v>6624</v>
+      </c>
+      <c r="C18" s="316" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="291" t="inlineStr">
-        <is>
-          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
-        </is>
-      </c>
-      <c r="E18" s="290" t="inlineStr">
-        <is>
-          <t>20.5</t>
-        </is>
-      </c>
-      <c r="F18" s="292" t="n">
-        <v>37030</v>
-      </c>
-      <c r="G18" s="290" t="inlineStr">
+      <c r="D18" s="316" t="inlineStr">
+        <is>
+          <t>S-45 DIA 19MM</t>
+        </is>
+      </c>
+      <c r="E18" s="315" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F18" s="317" t="n">
+        <v>15288</v>
+      </c>
+      <c r="G18" s="315" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50479,14 +50669,40 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="254">
-      <c r="A19" s="294" t="n"/>
-      <c r="B19" s="294" t="n"/>
-      <c r="C19" s="295" t="n"/>
-      <c r="D19" s="295" t="n"/>
-      <c r="E19" s="294" t="n"/>
-      <c r="F19" s="296" t="n"/>
-      <c r="G19" s="294" t="n"/>
-      <c r="H19" s="297" t="n"/>
+      <c r="A19" s="315" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="315" t="n">
+        <v>5731</v>
+      </c>
+      <c r="C19" s="316" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D19" s="316" t="inlineStr">
+        <is>
+          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
+        </is>
+      </c>
+      <c r="E19" s="315" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="F19" s="317" t="n">
+        <v>37030</v>
+      </c>
+      <c r="G19" s="315" t="inlineStr">
+        <is>
+          <t>Not Ready</t>
+        </is>
+      </c>
+      <c r="H19" s="293" t="inlineStr">
+        <is>
+          <t>Cap Not Available</t>
+        </is>
+      </c>
       <c r="I19" s="110">
         <f>IFERROR(SUMPRODUCT((TableBOM[Product ID]=B19)*(TableBOM[Material Category]="CAP")*TableBOM[Item ID]),0)</f>
         <v/>

</xml_diff>

<commit_message>
Full backup 12/06/2026 11:33:56
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tubex_Dashboard" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,6 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MRP'!$A$12:$J$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Product_Catalog'!$A$2:$S$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Production_Log'!$A$2:$R$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'BOM Issues'!$A$52:$J$64</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -1382,12 +1383,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="36" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="36" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1397,19 +1411,6 @@
     <xf numFmtId="0" fontId="42" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="36" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -1431,6 +1432,9 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1438,9 +1442,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2041,23 +2042,23 @@
   <dimension ref="A1:AC199"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="16.5"/>
   <cols>
-    <col width="1.5703125" customWidth="1" style="225" min="1" max="1"/>
-    <col width="7" customWidth="1" style="225" min="2" max="2"/>
-    <col width="32.7109375" customWidth="1" style="225" min="3" max="3"/>
-    <col width="38.7109375" customWidth="1" style="225" min="4" max="4"/>
-    <col width="8.85546875" customWidth="1" style="226" min="5" max="5"/>
-    <col width="9.140625" customWidth="1" style="225" min="6" max="6"/>
-    <col width="11" customWidth="1" style="227" min="7" max="7"/>
-    <col width="11.140625" customWidth="1" style="225" min="8" max="8"/>
-    <col width="10.28515625" customWidth="1" style="225" min="9" max="9"/>
-    <col width="10.5703125" customWidth="1" style="225" min="10" max="10"/>
-    <col width="9.28515625" customWidth="1" style="225" min="11" max="11"/>
-    <col width="33.85546875" customWidth="1" style="225" min="12" max="12"/>
-    <col width="14.7109375" customWidth="1" style="225" min="13" max="13"/>
-    <col width="13.28515625" customWidth="1" style="225" min="14" max="14"/>
-    <col width="9.5703125" customWidth="1" style="225" min="15" max="15"/>
-    <col width="8.7109375" customWidth="1" style="225" min="16" max="49"/>
-    <col width="8.7109375" customWidth="1" style="225" min="50" max="16384"/>
+    <col width="1.5703125" customWidth="1" style="227" min="1" max="1"/>
+    <col width="7" customWidth="1" style="227" min="2" max="2"/>
+    <col width="32.7109375" customWidth="1" style="227" min="3" max="3"/>
+    <col width="38.7109375" customWidth="1" style="227" min="4" max="4"/>
+    <col width="8.85546875" customWidth="1" style="228" min="5" max="5"/>
+    <col width="9.140625" customWidth="1" style="227" min="6" max="6"/>
+    <col width="11" customWidth="1" style="229" min="7" max="7"/>
+    <col width="11.140625" customWidth="1" style="227" min="8" max="8"/>
+    <col width="10.28515625" customWidth="1" style="227" min="9" max="9"/>
+    <col width="10.5703125" customWidth="1" style="227" min="10" max="10"/>
+    <col width="9.28515625" customWidth="1" style="227" min="11" max="11"/>
+    <col width="33.85546875" customWidth="1" style="227" min="12" max="12"/>
+    <col width="14.7109375" customWidth="1" style="227" min="13" max="13"/>
+    <col width="13.28515625" customWidth="1" style="227" min="14" max="14"/>
+    <col width="9.5703125" customWidth="1" style="227" min="15" max="15"/>
+    <col width="8.7109375" customWidth="1" style="227" min="16" max="50"/>
+    <col width="8.7109375" customWidth="1" style="227" min="51" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="6" customHeight="1" s="237">
@@ -2373,21 +2374,21 @@
     </row>
     <row r="9" ht="20.25" customHeight="1" s="237">
       <c r="A9" s="136" t="n"/>
-      <c r="B9" s="234" t="inlineStr">
+      <c r="B9" s="224" t="inlineStr">
         <is>
           <t>Summary of Production &amp; Dispatch - MTD</t>
         </is>
       </c>
-      <c r="C9" s="235" t="n"/>
-      <c r="D9" s="235" t="n"/>
-      <c r="E9" s="235" t="n"/>
-      <c r="F9" s="235" t="n"/>
-      <c r="G9" s="235" t="n"/>
-      <c r="H9" s="235" t="n"/>
-      <c r="I9" s="235" t="n"/>
-      <c r="J9" s="235" t="n"/>
-      <c r="K9" s="235" t="n"/>
-      <c r="L9" s="235" t="n"/>
+      <c r="C9" s="225" t="n"/>
+      <c r="D9" s="225" t="n"/>
+      <c r="E9" s="225" t="n"/>
+      <c r="F9" s="225" t="n"/>
+      <c r="G9" s="225" t="n"/>
+      <c r="H9" s="225" t="n"/>
+      <c r="I9" s="225" t="n"/>
+      <c r="J9" s="225" t="n"/>
+      <c r="K9" s="225" t="n"/>
+      <c r="L9" s="225" t="n"/>
       <c r="M9" s="157">
         <f>IFERROR(INDEX($S$9:$S$23,MATCH(LARGE($U$9:$U$23,3),$U$9:$U$23,0)),"")</f>
         <v/>
@@ -2710,7 +2711,9 @@
         <f>IF(G13=0,"-",H13/G13)</f>
         <v/>
       </c>
-      <c r="K13" s="287" t="n"/>
+      <c r="K13" s="287" t="n">
+        <v>62496</v>
+      </c>
       <c r="L13" s="289" t="n"/>
       <c r="M13" s="157">
         <f>IFERROR(INDEX($S$9:$S$23,MATCH(LARGE($U$9:$U$23,7),$U$9:$U$23,0)),"")</f>
@@ -2898,23 +2901,22 @@
       </c>
       <c r="C16" s="283" t="inlineStr">
         <is>
-          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D16" s="284" t="inlineStr">
         <is>
-          <t>HELLO HAIR COLOR</t>
+          <t>TUBES</t>
         </is>
       </c>
       <c r="E16" s="285" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F16" s="286" t="n">
-        <v>6206</v>
-      </c>
-      <c r="G16" s="286">
-        <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F16,MRP!$D$3:$D$9,0)),0)</f>
-        <v/>
+        <v>3726</v>
+      </c>
+      <c r="G16" s="286" t="n">
+        <v>0</v>
       </c>
       <c r="H16" s="287">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F16)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
@@ -2928,12 +2930,10 @@
         <f>IF(G16=0,"-",H16/G16)</f>
         <v/>
       </c>
-      <c r="K16" s="287" t="n"/>
-      <c r="L16" s="289" t="inlineStr">
-        <is>
-          <t>Advance Production</t>
-        </is>
-      </c>
+      <c r="K16" s="287" t="n">
+        <v>55776</v>
+      </c>
+      <c r="L16" s="289" t="n"/>
       <c r="M16" s="136" t="n"/>
       <c r="N16" s="136" t="n"/>
       <c r="O16" s="136" t="n"/>
@@ -2971,19 +2971,19 @@
       </c>
       <c r="C17" s="283" t="inlineStr">
         <is>
-          <t>Mablay Beauty PVT LTD.</t>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
       <c r="D17" s="284" t="inlineStr">
         <is>
-          <t>VINCE NURTURAL</t>
+          <t>HELLO HAIR COLOR</t>
         </is>
       </c>
       <c r="E17" s="285" t="n">
         <v>30</v>
       </c>
       <c r="F17" s="286" t="n">
-        <v>5814</v>
+        <v>6206</v>
       </c>
       <c r="G17" s="286">
         <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F17,MRP!$D$3:$D$9,0)),0)</f>
@@ -3002,7 +3002,11 @@
         <v/>
       </c>
       <c r="K17" s="287" t="n"/>
-      <c r="L17" s="289" t="n"/>
+      <c r="L17" s="289" t="inlineStr">
+        <is>
+          <t>Advance Production</t>
+        </is>
+      </c>
       <c r="P17" s="136" t="n"/>
       <c r="Q17" s="136" t="n"/>
       <c r="R17" s="136" t="n"/>
@@ -3027,19 +3031,19 @@
       </c>
       <c r="C18" s="283" t="inlineStr">
         <is>
-          <t>Adore</t>
+          <t>Mablay Beauty PVT LTD.</t>
         </is>
       </c>
       <c r="D18" s="284" t="inlineStr">
         <is>
-          <t>V- HC BROWN</t>
+          <t>VINCE NURTURAL</t>
         </is>
       </c>
       <c r="E18" s="285" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F18" s="286" t="n">
-        <v>6530</v>
+        <v>5814</v>
       </c>
       <c r="G18" s="286">
         <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F18,MRP!$D$3:$D$9,0)),0)</f>
@@ -3058,11 +3062,7 @@
         <v/>
       </c>
       <c r="K18" s="287" t="n"/>
-      <c r="L18" s="289" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hold </t>
-        </is>
-      </c>
+      <c r="L18" s="289" t="n"/>
       <c r="P18" s="136" t="n"/>
       <c r="Q18" s="136" t="n"/>
       <c r="R18" s="136" t="n"/>
@@ -3090,33 +3090,49 @@
     </row>
     <row r="19" ht="16.5" customHeight="1" s="237">
       <c r="A19" s="136" t="n"/>
-      <c r="B19" s="290" t="n"/>
-      <c r="C19" s="291" t="n"/>
-      <c r="D19" s="292" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E19" s="290" t="n"/>
-      <c r="F19" s="291" t="n"/>
-      <c r="G19" s="293">
-        <f>SUM(G11:G18)</f>
-        <v/>
-      </c>
-      <c r="H19" s="293">
-        <f>SUM(H11:H18)</f>
-        <v/>
-      </c>
-      <c r="I19" s="293">
-        <f>SUMIF(I11:I18,"&gt;"&amp;0)</f>
-        <v/>
-      </c>
-      <c r="J19" s="293" t="n"/>
-      <c r="K19" s="293">
-        <f>SUM(K11:K18)</f>
-        <v/>
-      </c>
-      <c r="L19" s="293" t="n"/>
+      <c r="B19" s="282" t="inlineStr">
+        <is>
+          <t>TUBE</t>
+        </is>
+      </c>
+      <c r="C19" s="283" t="inlineStr">
+        <is>
+          <t>Adore</t>
+        </is>
+      </c>
+      <c r="D19" s="284" t="inlineStr">
+        <is>
+          <t>V- HC BROWN</t>
+        </is>
+      </c>
+      <c r="E19" s="285" t="n">
+        <v>35</v>
+      </c>
+      <c r="F19" s="286" t="n">
+        <v>6530</v>
+      </c>
+      <c r="G19" s="286">
+        <f>IFERROR(INDEX(MRP!$F$3:$F$9,MATCH(Tubex_Dashboard!F19,MRP!$D$3:$D$9,0)),0)</f>
+        <v/>
+      </c>
+      <c r="H19" s="287">
+        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F19)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
+        <v/>
+      </c>
+      <c r="I19" s="286">
+        <f>G19-H19</f>
+        <v/>
+      </c>
+      <c r="J19" s="288">
+        <f>IF(G19=0,"-",H19/G19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="287" t="n"/>
+      <c r="L19" s="289" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hold </t>
+        </is>
+      </c>
       <c r="M19" s="136" t="n"/>
       <c r="N19" s="136" t="n"/>
       <c r="O19" s="136" t="n"/>
@@ -3147,46 +3163,33 @@
     </row>
     <row r="20" ht="16.5" customHeight="1" s="237">
       <c r="A20" s="136" t="n"/>
-      <c r="B20" s="282" t="inlineStr">
-        <is>
-          <t>PET</t>
-        </is>
-      </c>
-      <c r="C20" s="283" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D20" s="284" t="inlineStr">
-        <is>
-          <t>PET BOTTLE SMALL (120ML) YELLOW</t>
-        </is>
-      </c>
-      <c r="E20" s="285" t="inlineStr">
-        <is>
-          <t>120 ml</t>
-        </is>
-      </c>
-      <c r="F20" s="286" t="n">
-        <v>8005</v>
-      </c>
-      <c r="G20" s="286" t="n">
-        <v>19840</v>
-      </c>
-      <c r="H20" s="287">
-        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F20)*Production_Log!$H$3:$H$8963)</f>
-        <v/>
-      </c>
-      <c r="I20" s="286">
-        <f>G20-H20</f>
-        <v/>
-      </c>
-      <c r="J20" s="288">
-        <f>IF(G20=0,"-",H20/G20)</f>
-        <v/>
-      </c>
-      <c r="K20" s="287" t="n"/>
-      <c r="L20" s="289" t="n"/>
+      <c r="B20" s="290" t="n"/>
+      <c r="C20" s="291" t="n"/>
+      <c r="D20" s="292" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E20" s="290" t="n"/>
+      <c r="F20" s="291" t="n"/>
+      <c r="G20" s="293">
+        <f>SUM(G11:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="293">
+        <f>SUM(H11:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="293">
+        <f>SUMIF(I11:I19,"&gt;"&amp;0)</f>
+        <v/>
+      </c>
+      <c r="J20" s="293" t="n"/>
+      <c r="K20" s="293">
+        <f>SUM(K11:K19)</f>
+        <v/>
+      </c>
+      <c r="L20" s="293" t="n"/>
       <c r="M20" s="136" t="n"/>
       <c r="N20" s="136" t="n"/>
       <c r="O20" s="136" t="n"/>
@@ -3212,24 +3215,24 @@
       </c>
       <c r="C21" s="283" t="inlineStr">
         <is>
-          <t>Alpha Labs PVT LTD</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D21" s="284" t="inlineStr">
         <is>
-          <t>TRANSPARENT BOTTLE 150ML</t>
+          <t>PET BOTTLE SMALL (120ML) YELLOW</t>
         </is>
       </c>
       <c r="E21" s="285" t="inlineStr">
         <is>
-          <t>150 ml</t>
+          <t>120 ml</t>
         </is>
       </c>
       <c r="F21" s="286" t="n">
-        <v>8001</v>
+        <v>8005</v>
       </c>
       <c r="G21" s="286" t="n">
-        <v>249997</v>
+        <v>19840</v>
       </c>
       <c r="H21" s="287">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F21)*Production_Log!$H$3:$H$8963)</f>
@@ -3243,9 +3246,7 @@
         <f>IF(G21=0,"-",H21/G21)</f>
         <v/>
       </c>
-      <c r="K21" s="287" t="n">
-        <v>63480</v>
-      </c>
+      <c r="K21" s="287" t="n"/>
       <c r="L21" s="289" t="n"/>
       <c r="M21" s="136" t="n"/>
       <c r="N21" s="136" t="n"/>
@@ -3272,24 +3273,24 @@
       </c>
       <c r="C22" s="283" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
       <c r="D22" s="284" t="inlineStr">
         <is>
-          <t>PET BOTTLE LARGE 200ML WHITE</t>
+          <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
       <c r="E22" s="285" t="inlineStr">
         <is>
-          <t>200 ml</t>
+          <t>150 ml</t>
         </is>
       </c>
       <c r="F22" s="286" t="n">
-        <v>8007</v>
+        <v>8001</v>
       </c>
       <c r="G22" s="286" t="n">
-        <v>10000</v>
+        <v>249997</v>
       </c>
       <c r="H22" s="287">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F22)*Production_Log!$H$3:$H$8963)</f>
@@ -3303,7 +3304,9 @@
         <f>IF(G22=0,"-",H22/G22)</f>
         <v/>
       </c>
-      <c r="K22" s="287" t="n"/>
+      <c r="K22" s="287" t="n">
+        <v>63480</v>
+      </c>
       <c r="L22" s="289" t="n"/>
       <c r="M22" s="136" t="n"/>
       <c r="N22" s="136" t="n"/>
@@ -3335,7 +3338,7 @@
       </c>
       <c r="D23" s="284" t="inlineStr">
         <is>
-          <t>BT-200 ML YELLOW</t>
+          <t>PET BOTTLE LARGE 200ML WHITE</t>
         </is>
       </c>
       <c r="E23" s="285" t="inlineStr">
@@ -3344,10 +3347,10 @@
         </is>
       </c>
       <c r="F23" s="286" t="n">
-        <v>8006</v>
+        <v>8007</v>
       </c>
       <c r="G23" s="286" t="n">
-        <v>42400</v>
+        <v>10000</v>
       </c>
       <c r="H23" s="287">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F23)*Production_Log!$H$3:$H$8963)</f>
@@ -3393,7 +3396,7 @@
       </c>
       <c r="D24" s="284" t="inlineStr">
         <is>
-          <t>BT-200ML MUSTARD OIL (TRANSPARENT)</t>
+          <t>BT-200 ML YELLOW</t>
         </is>
       </c>
       <c r="E24" s="285" t="inlineStr">
@@ -3402,10 +3405,10 @@
         </is>
       </c>
       <c r="F24" s="286" t="n">
-        <v>8014</v>
+        <v>8006</v>
       </c>
       <c r="G24" s="286" t="n">
-        <v>10000</v>
+        <v>42400</v>
       </c>
       <c r="H24" s="287">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F24)*Production_Log!$H$3:$H$8963)</f>
@@ -3441,33 +3444,46 @@
     </row>
     <row r="25" ht="16.5" customHeight="1" s="237">
       <c r="A25" s="136" t="n"/>
-      <c r="B25" s="290" t="n"/>
-      <c r="C25" s="291" t="n"/>
-      <c r="D25" s="292" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="E25" s="290" t="n"/>
-      <c r="F25" s="291" t="n"/>
-      <c r="G25" s="293">
-        <f>SUM(G20:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="293">
-        <f>SUM(H20:H24)</f>
-        <v/>
-      </c>
-      <c r="I25" s="293">
-        <f>SUMIF(I20:I24,"&gt;"&amp;0)</f>
-        <v/>
-      </c>
-      <c r="J25" s="293" t="n"/>
-      <c r="K25" s="293">
-        <f>SUM(K20:K24)</f>
-        <v/>
-      </c>
-      <c r="L25" s="293" t="n"/>
+      <c r="B25" s="282" t="inlineStr">
+        <is>
+          <t>PET</t>
+        </is>
+      </c>
+      <c r="C25" s="283" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D25" s="284" t="inlineStr">
+        <is>
+          <t>BT-200ML MUSTARD OIL (TRANSPARENT)</t>
+        </is>
+      </c>
+      <c r="E25" s="285" t="inlineStr">
+        <is>
+          <t>200 ml</t>
+        </is>
+      </c>
+      <c r="F25" s="286" t="n">
+        <v>8014</v>
+      </c>
+      <c r="G25" s="286" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H25" s="287">
+        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F25)*Production_Log!$H$3:$H$8963)</f>
+        <v/>
+      </c>
+      <c r="I25" s="286">
+        <f>G25-H25</f>
+        <v/>
+      </c>
+      <c r="J25" s="288">
+        <f>IF(G25=0,"-",H25/G25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="287" t="n"/>
+      <c r="L25" s="289" t="n"/>
       <c r="M25" s="136" t="n"/>
       <c r="N25" s="136" t="n"/>
       <c r="O25" s="136" t="n"/>
@@ -3488,44 +3504,33 @@
     </row>
     <row r="26" ht="16.5" customHeight="1" s="237">
       <c r="A26" s="136" t="n"/>
-      <c r="B26" s="282" t="inlineStr">
-        <is>
-          <t>TUBE</t>
-        </is>
-      </c>
-      <c r="C26" s="283" t="inlineStr">
-        <is>
-          <t>Bahadur</t>
-        </is>
-      </c>
-      <c r="D26" s="284" t="inlineStr">
-        <is>
-          <t>BAHADUR TUBE 12.5MM</t>
-        </is>
-      </c>
-      <c r="E26" s="285" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="F26" s="286" t="n">
-        <v>9004</v>
-      </c>
-      <c r="G26" s="286" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="287">
-        <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F26)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
-        <v/>
-      </c>
-      <c r="I26" s="286">
-        <f>G26-H26</f>
-        <v/>
-      </c>
-      <c r="J26" s="288">
-        <f>IF(G26=0,"-",H26/G26)</f>
-        <v/>
-      </c>
-      <c r="K26" s="287" t="n"/>
-      <c r="L26" s="289" t="n"/>
+      <c r="B26" s="290" t="n"/>
+      <c r="C26" s="291" t="n"/>
+      <c r="D26" s="292" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E26" s="290" t="n"/>
+      <c r="F26" s="291" t="n"/>
+      <c r="G26" s="293">
+        <f>SUM(G21:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="293">
+        <f>SUM(H21:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="293">
+        <f>SUMIF(I21:I25,"&gt;"&amp;0)</f>
+        <v/>
+      </c>
+      <c r="J26" s="293" t="n"/>
+      <c r="K26" s="293">
+        <f>SUM(K21:K25)</f>
+        <v/>
+      </c>
+      <c r="L26" s="293" t="n"/>
       <c r="M26" s="136" t="n"/>
       <c r="N26" s="136" t="n"/>
       <c r="O26" s="136" t="n"/>
@@ -3553,19 +3558,19 @@
       </c>
       <c r="C27" s="283" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Bahadur</t>
         </is>
       </c>
       <c r="D27" s="284" t="inlineStr">
         <is>
-          <t>S-45 DIA 19MM</t>
+          <t>BAHADUR TUBE 12.5MM</t>
         </is>
       </c>
       <c r="E27" s="285" t="n">
-        <v>19</v>
+        <v>12.5</v>
       </c>
       <c r="F27" s="286" t="n">
-        <v>6624</v>
+        <v>9004</v>
       </c>
       <c r="G27" s="286" t="n">
         <v>0</v>
@@ -3616,14 +3621,14 @@
       </c>
       <c r="D28" s="284" t="inlineStr">
         <is>
-          <t>S-43 DIA 19MM</t>
+          <t>S-45 DIA 19MM</t>
         </is>
       </c>
       <c r="E28" s="285" t="n">
         <v>19</v>
       </c>
       <c r="F28" s="286" t="n">
-        <v>6623</v>
+        <v>6624</v>
       </c>
       <c r="G28" s="286" t="n">
         <v>0</v>
@@ -3667,19 +3672,19 @@
       </c>
       <c r="C29" s="283" t="inlineStr">
         <is>
-          <t>Brookes Pharma Private Limited</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D29" s="284" t="inlineStr">
         <is>
-          <t>PHLOGIN GEL 20G</t>
+          <t>S-43 DIA 19MM</t>
         </is>
       </c>
       <c r="E29" s="285" t="n">
         <v>19</v>
       </c>
       <c r="F29" s="286" t="n">
-        <v>6559</v>
+        <v>6623</v>
       </c>
       <c r="G29" s="286" t="n">
         <v>0</v>
@@ -3728,14 +3733,14 @@
       </c>
       <c r="D30" s="284" t="inlineStr">
         <is>
-          <t>PYODINE GEL 20GM</t>
+          <t>PHLOGIN GEL 20G</t>
         </is>
       </c>
       <c r="E30" s="285" t="n">
         <v>19</v>
       </c>
       <c r="F30" s="286" t="n">
-        <v>1085</v>
+        <v>6559</v>
       </c>
       <c r="G30" s="286" t="n">
         <v>0</v>
@@ -3786,14 +3791,14 @@
       </c>
       <c r="D31" s="284" t="inlineStr">
         <is>
-          <t>CONTRATUBEX GEL 20G</t>
+          <t>PYODINE GEL 20GM</t>
         </is>
       </c>
       <c r="E31" s="285" t="n">
         <v>19</v>
       </c>
       <c r="F31" s="286" t="n">
-        <v>6560</v>
+        <v>1085</v>
       </c>
       <c r="G31" s="286" t="n">
         <v>0</v>
@@ -3839,19 +3844,19 @@
       </c>
       <c r="C32" s="283" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Brookes Pharma Private Limited</t>
         </is>
       </c>
       <c r="D32" s="284" t="inlineStr">
         <is>
-          <t>S-43 DIA 20.5</t>
+          <t>CONTRATUBEX GEL 20G</t>
         </is>
       </c>
       <c r="E32" s="285" t="n">
-        <v>20.5</v>
+        <v>19</v>
       </c>
       <c r="F32" s="286" t="n">
-        <v>5699</v>
+        <v>6560</v>
       </c>
       <c r="G32" s="286" t="n">
         <v>0</v>
@@ -3897,19 +3902,19 @@
       </c>
       <c r="C33" s="283" t="inlineStr">
         <is>
-          <t>Mablay Beauty PVT LTD.</t>
+          <t>Samsol International Private Limited</t>
         </is>
       </c>
       <c r="D33" s="284" t="inlineStr">
         <is>
-          <t>VINCE HIS ONLY BEARD &amp; MUSTACHE COLOR CREAM</t>
+          <t>S-43 DIA 20.5</t>
         </is>
       </c>
       <c r="E33" s="285" t="n">
         <v>20.5</v>
       </c>
       <c r="F33" s="286" t="n">
-        <v>6077</v>
+        <v>5699</v>
       </c>
       <c r="G33" s="286" t="n">
         <v>0</v>
@@ -3953,19 +3958,19 @@
       </c>
       <c r="C34" s="283" t="inlineStr">
         <is>
-          <t>Samsol International Private Limited</t>
+          <t>Mablay Beauty PVT LTD.</t>
         </is>
       </c>
       <c r="D34" s="284" t="inlineStr">
         <is>
-          <t>S-45 DIA 20.5</t>
+          <t>VINCE HIS ONLY BEARD &amp; MUSTACHE COLOR CREAM</t>
         </is>
       </c>
       <c r="E34" s="285" t="n">
         <v>20.5</v>
       </c>
       <c r="F34" s="286" t="n">
-        <v>5698</v>
+        <v>6077</v>
       </c>
       <c r="G34" s="286" t="n">
         <v>0</v>
@@ -4014,14 +4019,14 @@
       </c>
       <c r="D35" s="284" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
+          <t>S-45 DIA 20.5</t>
         </is>
       </c>
       <c r="E35" s="285" t="n">
         <v>20.5</v>
       </c>
       <c r="F35" s="286" t="n">
-        <v>5731</v>
+        <v>5698</v>
       </c>
       <c r="G35" s="286" t="n">
         <v>0</v>
@@ -4070,14 +4075,14 @@
       </c>
       <c r="D36" s="284" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 43 DIA 20.5 MM</t>
+          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
       <c r="E36" s="285" t="n">
         <v>20.5</v>
       </c>
       <c r="F36" s="286" t="n">
-        <v>5732</v>
+        <v>5731</v>
       </c>
       <c r="G36" s="286" t="n">
         <v>0</v>
@@ -4099,7 +4104,7 @@
       <c r="P36" s="136" t="n"/>
       <c r="Q36" s="136" t="n"/>
       <c r="R36" s="136" t="n"/>
-      <c r="S36" s="225" t="inlineStr">
+      <c r="S36" s="227" t="inlineStr">
         <is>
           <t>Gas Shutdown</t>
         </is>
@@ -4108,7 +4113,7 @@
         <f>SUMPRODUCT((MONTH(Production_Log!$A$3:$A$8963)=MONTH(TODAY()))*(YEAR(Production_Log!$A$3:$A$8963)=YEAR(TODAY()))*Production_Log!$Q$3:$Q$8963)</f>
         <v/>
       </c>
-      <c r="U36" s="225">
+      <c r="U36" s="227">
         <f>T36+0.00006</f>
         <v/>
       </c>
@@ -4135,14 +4140,14 @@
       </c>
       <c r="D37" s="284" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 39 SMALL PURPLE</t>
+          <t>SAMSOL HAIR COLOR 43 DIA 20.5 MM</t>
         </is>
       </c>
       <c r="E37" s="285" t="n">
         <v>20.5</v>
       </c>
       <c r="F37" s="286" t="n">
-        <v>6556</v>
+        <v>5732</v>
       </c>
       <c r="G37" s="286" t="n">
         <v>0</v>
@@ -4193,14 +4198,14 @@
       </c>
       <c r="D38" s="284" t="inlineStr">
         <is>
-          <t>SAMSOL HAIR COLOR 41 SMALL PURPLE</t>
+          <t>SAMSOL HAIR COLOR 39 SMALL PURPLE</t>
         </is>
       </c>
       <c r="E38" s="285" t="n">
         <v>20.5</v>
       </c>
       <c r="F38" s="286" t="n">
-        <v>6557</v>
+        <v>6556</v>
       </c>
       <c r="G38" s="286" t="n">
         <v>0</v>
@@ -4251,14 +4256,14 @@
       </c>
       <c r="D39" s="284" t="inlineStr">
         <is>
-          <t>TUBES</t>
+          <t>SAMSOL HAIR COLOR 41 SMALL PURPLE</t>
         </is>
       </c>
       <c r="E39" s="285" t="n">
-        <v>25</v>
+        <v>20.5</v>
       </c>
       <c r="F39" s="286" t="n">
-        <v>3726</v>
+        <v>6557</v>
       </c>
       <c r="G39" s="286" t="n">
         <v>0</v>
@@ -6820,9 +6825,10 @@
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A20)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A20)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A20)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A20)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A20)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A20)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A20)&gt;0)*($H$9&gt;0),$C$9&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A20)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A20)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A20)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A20)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A20)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A20)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A20)&gt;0)*($H$9&gt;0),$C$9&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A20)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A20)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A20)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A20)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A20)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A20)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A20)&gt;0)*($H$9&gt;0),$C$9&amp;", ",""))-2),"")</f>
         <v/>
       </c>
-      <c r="I20" s="30">
-        <f>IF(E20=0,"Not needed",IF(G20&lt;0,"SHORTAGE",IF(G20&lt;F20*0.1,"LOW","OK")))</f>
-        <v/>
+      <c r="I20" s="30" t="inlineStr">
+        <is>
+          <t>100kg Shortage (13k tubes WIP)</t>
+        </is>
       </c>
       <c r="J20" s="30">
         <f>IF(B20&lt;&gt;"CAP","",SUMPRODUCT((ISNUMBER(SEARCH("Cap Not Available",'FG Stock'!$H$4:$H$100)))*('FG Stock'!$I$4:$I$100=A20)*'FG Stock'!$F$4:$F$100))</f>
@@ -13159,22 +13165,22 @@
       <filters>
         <filter val="1"/>
         <filter val="10"/>
-        <filter val="110"/>
-        <filter val="114,655"/>
         <filter val="138"/>
         <filter val="15"/>
-        <filter val="172"/>
+        <filter val="170"/>
         <filter val="188"/>
         <filter val="194"/>
         <filter val="2"/>
         <filter val="25,500"/>
+        <filter val="289"/>
         <filter val="3"/>
+        <filter val="36"/>
         <filter val="36,006"/>
-        <filter val="361"/>
-        <filter val="43"/>
+        <filter val="574"/>
         <filter val="69"/>
-        <filter val="718"/>
         <filter val="89"/>
+        <filter val="92,036"/>
+        <filter val="95"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -32247,13 +32253,13 @@
           <t>Slugs Inventory — June 2026 MONTH TO DATE</t>
         </is>
       </c>
-      <c r="B1" s="235" t="n"/>
-      <c r="C1" s="235" t="n"/>
-      <c r="D1" s="235" t="n"/>
-      <c r="E1" s="235" t="n"/>
-      <c r="F1" s="235" t="n"/>
-      <c r="G1" s="235" t="n"/>
-      <c r="H1" s="235" t="n"/>
+      <c r="B1" s="225" t="n"/>
+      <c r="C1" s="225" t="n"/>
+      <c r="D1" s="225" t="n"/>
+      <c r="E1" s="225" t="n"/>
+      <c r="F1" s="225" t="n"/>
+      <c r="G1" s="225" t="n"/>
+      <c r="H1" s="225" t="n"/>
       <c r="I1" s="69" t="inlineStr">
         <is>
           <t>Date:</t>
@@ -32501,7 +32507,7 @@
         <v/>
       </c>
       <c r="I7" s="37" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="J7" s="37">
         <f>IFERROR(IF(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])=0,"-",ROUND((H7+I7)/(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])/1000),0)),"-")</f>
@@ -40263,7 +40269,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -40402,7 +40408,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="237">
+    <row r="3" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A3" s="268" t="n">
         <v>46174</v>
       </c>
@@ -40452,7 +40458,7 @@
       <c r="R3" s="265" t="n"/>
       <c r="S3" s="265" t="n"/>
     </row>
-    <row r="4" ht="15" customHeight="1" s="237">
+    <row r="4" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A4" s="268" t="n">
         <v>46174</v>
       </c>
@@ -40500,7 +40506,7 @@
       <c r="R4" s="265" t="n"/>
       <c r="S4" s="265" t="n"/>
     </row>
-    <row r="5" ht="15" customHeight="1" s="237">
+    <row r="5" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A5" s="268" t="n">
         <v>46174</v>
       </c>
@@ -40548,7 +40554,7 @@
       <c r="R5" s="265" t="n"/>
       <c r="S5" s="265" t="n"/>
     </row>
-    <row r="6" ht="15" customHeight="1" s="237">
+    <row r="6" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A6" s="268" t="n">
         <v>46174</v>
       </c>
@@ -40600,7 +40606,7 @@
       <c r="R6" s="265" t="n"/>
       <c r="S6" s="265" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1" s="237">
+    <row r="7" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A7" s="268" t="n">
         <v>46174</v>
       </c>
@@ -40648,7 +40654,7 @@
       <c r="R7" s="265" t="n"/>
       <c r="S7" s="265" t="n"/>
     </row>
-    <row r="8" ht="15" customHeight="1" s="237">
+    <row r="8" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A8" s="268" t="n">
         <v>46174</v>
       </c>
@@ -40748,7 +40754,7 @@
       <c r="R9" s="265" t="n"/>
       <c r="S9" s="265" t="n"/>
     </row>
-    <row r="10" ht="15" customHeight="1" s="237">
+    <row r="10" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A10" s="268" t="n">
         <v>46174</v>
       </c>
@@ -40796,7 +40802,7 @@
       <c r="R10" s="265" t="n"/>
       <c r="S10" s="265" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1" s="237">
+    <row r="11" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A11" s="268" t="n">
         <v>46175</v>
       </c>
@@ -40846,7 +40852,7 @@
       <c r="R11" s="265" t="n"/>
       <c r="S11" s="265" t="n"/>
     </row>
-    <row r="12" ht="15" customHeight="1" s="237">
+    <row r="12" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A12" s="268" t="n">
         <v>46175</v>
       </c>
@@ -40894,7 +40900,7 @@
       <c r="R12" s="265" t="n"/>
       <c r="S12" s="265" t="n"/>
     </row>
-    <row r="13" ht="15" customHeight="1" s="237">
+    <row r="13" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A13" s="268" t="n">
         <v>46175</v>
       </c>
@@ -40944,7 +40950,7 @@
       <c r="R13" s="265" t="n"/>
       <c r="S13" s="265" t="n"/>
     </row>
-    <row r="14" ht="15" customHeight="1" s="237">
+    <row r="14" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A14" s="268" t="n">
         <v>46175</v>
       </c>
@@ -40996,7 +41002,7 @@
       <c r="R14" s="265" t="n"/>
       <c r="S14" s="265" t="n"/>
     </row>
-    <row r="15" ht="15" customHeight="1" s="237">
+    <row r="15" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A15" s="268" t="n">
         <v>46175</v>
       </c>
@@ -41044,7 +41050,7 @@
       <c r="R15" s="265" t="n"/>
       <c r="S15" s="265" t="n"/>
     </row>
-    <row r="16" ht="15" customHeight="1" s="237">
+    <row r="16" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A16" s="268" t="n">
         <v>46175</v>
       </c>
@@ -41142,7 +41148,7 @@
       <c r="R17" s="265" t="n"/>
       <c r="S17" s="265" t="n"/>
     </row>
-    <row r="18" ht="15" customHeight="1" s="237">
+    <row r="18" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A18" s="268" t="n">
         <v>46175</v>
       </c>
@@ -41190,7 +41196,7 @@
       <c r="R18" s="265" t="n"/>
       <c r="S18" s="265" t="n"/>
     </row>
-    <row r="19" ht="15" customHeight="1" s="237">
+    <row r="19" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A19" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41226,7 +41232,7 @@
       <c r="R19" s="265" t="n"/>
       <c r="S19" s="265" t="n"/>
     </row>
-    <row r="20" ht="15" customHeight="1" s="237">
+    <row r="20" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A20" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41262,7 +41268,7 @@
       <c r="R20" s="265" t="n"/>
       <c r="S20" s="265" t="n"/>
     </row>
-    <row r="21" ht="15" customHeight="1" s="237">
+    <row r="21" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A21" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41298,7 +41304,7 @@
       <c r="R21" s="265" t="n"/>
       <c r="S21" s="265" t="n"/>
     </row>
-    <row r="22" ht="15" customHeight="1" s="237">
+    <row r="22" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A22" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41352,7 +41358,7 @@
       <c r="R22" s="265" t="n"/>
       <c r="S22" s="265" t="n"/>
     </row>
-    <row r="23" ht="15" customHeight="1" s="237">
+    <row r="23" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A23" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41388,7 +41394,7 @@
       <c r="R23" s="265" t="n"/>
       <c r="S23" s="265" t="n"/>
     </row>
-    <row r="24" ht="15" customHeight="1" s="237">
+    <row r="24" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A24" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41424,7 +41430,7 @@
       <c r="R24" s="265" t="n"/>
       <c r="S24" s="265" t="n"/>
     </row>
-    <row r="25" ht="15" customHeight="1" s="237">
+    <row r="25" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A25" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41460,7 +41466,7 @@
       <c r="R25" s="265" t="n"/>
       <c r="S25" s="265" t="n"/>
     </row>
-    <row r="26" ht="15" customHeight="1" s="237">
+    <row r="26" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A26" s="268" t="n">
         <v>46177</v>
       </c>
@@ -41496,7 +41502,7 @@
       <c r="R26" s="265" t="n"/>
       <c r="S26" s="265" t="n"/>
     </row>
-    <row r="27" ht="15" customHeight="1" s="237">
+    <row r="27" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A27" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41532,7 +41538,7 @@
       <c r="R27" s="265" t="n"/>
       <c r="S27" s="265" t="n"/>
     </row>
-    <row r="28" ht="15" customHeight="1" s="237">
+    <row r="28" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A28" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41568,7 +41574,7 @@
       <c r="R28" s="265" t="n"/>
       <c r="S28" s="265" t="n"/>
     </row>
-    <row r="29" ht="15" customHeight="1" s="237">
+    <row r="29" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A29" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41604,7 +41610,7 @@
       <c r="R29" s="265" t="n"/>
       <c r="S29" s="265" t="n"/>
     </row>
-    <row r="30" ht="15" customHeight="1" s="237">
+    <row r="30" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A30" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41658,7 +41664,7 @@
       <c r="R30" s="265" t="n"/>
       <c r="S30" s="265" t="n"/>
     </row>
-    <row r="31" ht="15" customHeight="1" s="237">
+    <row r="31" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A31" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41694,7 +41700,7 @@
       <c r="R31" s="265" t="n"/>
       <c r="S31" s="265" t="n"/>
     </row>
-    <row r="32" ht="15" customHeight="1" s="237">
+    <row r="32" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A32" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41730,7 +41736,7 @@
       <c r="R32" s="265" t="n"/>
       <c r="S32" s="265" t="n"/>
     </row>
-    <row r="33" ht="15" customHeight="1" s="237">
+    <row r="33" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A33" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41766,7 +41772,7 @@
       <c r="R33" s="265" t="n"/>
       <c r="S33" s="265" t="n"/>
     </row>
-    <row r="34" ht="15" customHeight="1" s="237">
+    <row r="34" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A34" s="268" t="n">
         <v>46178</v>
       </c>
@@ -41802,7 +41808,7 @@
       <c r="R34" s="265" t="n"/>
       <c r="S34" s="265" t="n"/>
     </row>
-    <row r="35" ht="15" customHeight="1" s="237">
+    <row r="35" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A35" s="268" t="n">
         <v>46179</v>
       </c>
@@ -41838,7 +41844,7 @@
       <c r="R35" s="265" t="n"/>
       <c r="S35" s="265" t="n"/>
     </row>
-    <row r="36" ht="15" customHeight="1" s="237">
+    <row r="36" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A36" s="268" t="n">
         <v>46179</v>
       </c>
@@ -41874,7 +41880,7 @@
       <c r="R36" s="265" t="n"/>
       <c r="S36" s="265" t="n"/>
     </row>
-    <row r="37" ht="15" customHeight="1" s="237">
+    <row r="37" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A37" s="268" t="n">
         <v>46179</v>
       </c>
@@ -41910,7 +41916,7 @@
       <c r="R37" s="265" t="n"/>
       <c r="S37" s="265" t="n"/>
     </row>
-    <row r="38" ht="15" customHeight="1" s="237">
+    <row r="38" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A38" s="268" t="n">
         <v>46179</v>
       </c>
@@ -41966,7 +41972,7 @@
       <c r="R38" s="265" t="n"/>
       <c r="S38" s="265" t="n"/>
     </row>
-    <row r="39" ht="15" customHeight="1" s="237">
+    <row r="39" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A39" s="268" t="n">
         <v>46179</v>
       </c>
@@ -42002,7 +42008,7 @@
       <c r="R39" s="265" t="n"/>
       <c r="S39" s="265" t="n"/>
     </row>
-    <row r="40" ht="15" customHeight="1" s="237">
+    <row r="40" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A40" s="268" t="n">
         <v>46179</v>
       </c>
@@ -42038,7 +42044,7 @@
       <c r="R40" s="265" t="n"/>
       <c r="S40" s="265" t="n"/>
     </row>
-    <row r="41" ht="15" customHeight="1" s="237">
+    <row r="41" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A41" s="268" t="n">
         <v>46179</v>
       </c>
@@ -42074,7 +42080,7 @@
       <c r="R41" s="265" t="n"/>
       <c r="S41" s="265" t="n"/>
     </row>
-    <row r="42" ht="15" customHeight="1" s="237">
+    <row r="42" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A42" s="268" t="n">
         <v>46179</v>
       </c>
@@ -42110,7 +42116,7 @@
       <c r="R42" s="265" t="n"/>
       <c r="S42" s="265" t="n"/>
     </row>
-    <row r="43" ht="15" customHeight="1" s="237">
+    <row r="43" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A43" s="268" t="n">
         <v>46181</v>
       </c>
@@ -42146,7 +42152,7 @@
       <c r="R43" s="265" t="n"/>
       <c r="S43" s="265" t="n"/>
     </row>
-    <row r="44" ht="15" customHeight="1" s="237">
+    <row r="44" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A44" s="268" t="n">
         <v>46181</v>
       </c>
@@ -42194,7 +42200,7 @@
       <c r="R44" s="265" t="n"/>
       <c r="S44" s="265" t="n"/>
     </row>
-    <row r="45" ht="15" customHeight="1" s="237">
+    <row r="45" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A45" s="268" t="n">
         <v>46181</v>
       </c>
@@ -42230,7 +42236,7 @@
       <c r="R45" s="265" t="n"/>
       <c r="S45" s="265" t="n"/>
     </row>
-    <row r="46" ht="15" customHeight="1" s="237">
+    <row r="46" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A46" s="268" t="n">
         <v>46181</v>
       </c>
@@ -42284,7 +42290,7 @@
       <c r="R46" s="265" t="n"/>
       <c r="S46" s="265" t="n"/>
     </row>
-    <row r="47" ht="15" customHeight="1" s="237">
+    <row r="47" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A47" s="268" t="n">
         <v>46181</v>
       </c>
@@ -42320,7 +42326,7 @@
       <c r="R47" s="265" t="n"/>
       <c r="S47" s="265" t="n"/>
     </row>
-    <row r="48" ht="15" customHeight="1" s="237">
+    <row r="48" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A48" s="268" t="n">
         <v>46181</v>
       </c>
@@ -42418,7 +42424,7 @@
       <c r="R49" s="265" t="n"/>
       <c r="S49" s="265" t="n"/>
     </row>
-    <row r="50" ht="15" customHeight="1" s="237">
+    <row r="50" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A50" s="268" t="n">
         <v>46181</v>
       </c>
@@ -42454,7 +42460,7 @@
       <c r="R50" s="265" t="n"/>
       <c r="S50" s="265" t="n"/>
     </row>
-    <row r="51" ht="15" customHeight="1" s="237">
+    <row r="51" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A51" s="268" t="n">
         <v>46182</v>
       </c>
@@ -42490,7 +42496,7 @@
       <c r="R51" s="265" t="n"/>
       <c r="S51" s="265" t="n"/>
     </row>
-    <row r="52" ht="15" customHeight="1" s="237">
+    <row r="52" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A52" s="268" t="n">
         <v>46182</v>
       </c>
@@ -42538,7 +42544,7 @@
       <c r="R52" s="265" t="n"/>
       <c r="S52" s="265" t="n"/>
     </row>
-    <row r="53" ht="15" customHeight="1" s="237">
+    <row r="53" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A53" s="268" t="n">
         <v>46182</v>
       </c>
@@ -42574,7 +42580,7 @@
       <c r="R53" s="265" t="n"/>
       <c r="S53" s="265" t="n"/>
     </row>
-    <row r="54" ht="15" customHeight="1" s="237">
+    <row r="54" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A54" s="268" t="n">
         <v>46182</v>
       </c>
@@ -42628,7 +42634,7 @@
       <c r="R54" s="265" t="n"/>
       <c r="S54" s="265" t="n"/>
     </row>
-    <row r="55" ht="15" customHeight="1" s="237">
+    <row r="55" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A55" s="268" t="n">
         <v>46182</v>
       </c>
@@ -42664,7 +42670,7 @@
       <c r="R55" s="265" t="n"/>
       <c r="S55" s="265" t="n"/>
     </row>
-    <row r="56" ht="15" customHeight="1" s="237">
+    <row r="56" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A56" s="268" t="n">
         <v>46182</v>
       </c>
@@ -42760,7 +42766,7 @@
       <c r="R57" s="265" t="n"/>
       <c r="S57" s="265" t="n"/>
     </row>
-    <row r="58" ht="15" customHeight="1" s="237">
+    <row r="58" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A58" s="268" t="n">
         <v>46182</v>
       </c>
@@ -42796,7 +42802,7 @@
       <c r="R58" s="265" t="n"/>
       <c r="S58" s="265" t="n"/>
     </row>
-    <row r="59" ht="15" customHeight="1" s="237">
+    <row r="59" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A59" s="268" t="n">
         <v>46183</v>
       </c>
@@ -42832,7 +42838,7 @@
       <c r="R59" s="265" t="n"/>
       <c r="S59" s="265" t="n"/>
     </row>
-    <row r="60" ht="15" customHeight="1" s="237">
+    <row r="60" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A60" s="268" t="n">
         <v>46183</v>
       </c>
@@ -42880,7 +42886,7 @@
       <c r="R60" s="265" t="n"/>
       <c r="S60" s="265" t="n"/>
     </row>
-    <row r="61" ht="15" customHeight="1" s="237">
+    <row r="61" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A61" s="268" t="n">
         <v>46183</v>
       </c>
@@ -42916,7 +42922,7 @@
       <c r="R61" s="265" t="n"/>
       <c r="S61" s="265" t="n"/>
     </row>
-    <row r="62" ht="15" customHeight="1" s="237">
+    <row r="62" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A62" s="268" t="n">
         <v>46183</v>
       </c>
@@ -42968,7 +42974,7 @@
       <c r="R62" s="265" t="n"/>
       <c r="S62" s="265" t="n"/>
     </row>
-    <row r="63" ht="15" customHeight="1" s="237">
+    <row r="63" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A63" s="268" t="n">
         <v>46183</v>
       </c>
@@ -43004,7 +43010,7 @@
       <c r="R63" s="265" t="n"/>
       <c r="S63" s="265" t="n"/>
     </row>
-    <row r="64" ht="15" customHeight="1" s="237">
+    <row r="64" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A64" s="268" t="n">
         <v>46183</v>
       </c>
@@ -43100,7 +43106,7 @@
       <c r="R65" s="265" t="n"/>
       <c r="S65" s="265" t="n"/>
     </row>
-    <row r="66" ht="15" customHeight="1" s="237">
+    <row r="66" hidden="1" ht="15" customHeight="1" s="237">
       <c r="A66" s="268" t="n">
         <v>46183</v>
       </c>
@@ -45832,6 +45838,18 @@
       <c r="J247" s="91" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:R66">
+    <filterColumn colId="1" hiddenButton="0" showButton="1">
+      <filters>
+        <filter val="Printing-03"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4" hiddenButton="0" showButton="1">
+      <filters>
+        <filter val="25"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -52250,7 +52268,7 @@
         </is>
       </c>
     </row>
-    <row r="8" customFormat="1" s="246">
+    <row r="8" customFormat="1" s="247">
       <c r="A8" s="127" t="inlineStr">
         <is>
           <t>2</t>
@@ -52282,7 +52300,7 @@
         </is>
       </c>
     </row>
-    <row r="9" customFormat="1" s="246">
+    <row r="9" customFormat="1" s="247">
       <c r="A9" s="126" t="inlineStr">
         <is>
           <t>3</t>
@@ -52314,7 +52332,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customFormat="1" customHeight="1" s="246">
+    <row r="10" ht="24" customFormat="1" customHeight="1" s="247">
       <c r="A10" s="106" t="n"/>
       <c r="B10" s="107" t="inlineStr">
         <is>
@@ -52454,7 +52472,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customFormat="1" customHeight="1" s="246">
+    <row r="15" ht="24" customFormat="1" customHeight="1" s="247">
       <c r="A15" s="126" t="inlineStr">
         <is>
           <t>4</t>
@@ -52514,7 +52532,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="8.1" customFormat="1" customHeight="1" s="246">
+    <row r="17" ht="8.1" customFormat="1" customHeight="1" s="247">
       <c r="A17" s="128" t="n"/>
       <c r="B17" s="129" t="n"/>
       <c r="C17" s="129" t="n"/>
@@ -52522,21 +52540,21 @@
       <c r="E17" s="125" t="n"/>
       <c r="F17" s="125" t="n"/>
     </row>
-    <row r="18" ht="15.95" customFormat="1" customHeight="1" s="246">
+    <row r="18" ht="15.95" customFormat="1" customHeight="1" s="247">
       <c r="A18" s="263" t="inlineStr">
         <is>
           <t>Individual scripts: update_production.py also runs sort_dashboard automatically at the end.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15.95" customFormat="1" customHeight="1" s="246">
+    <row r="19" ht="15.95" customFormat="1" customHeight="1" s="247">
       <c r="A19" s="263" t="inlineStr">
         <is>
           <t>Safety: All scripts check if Excel file is open (lock guard) and warn if source files are stale (&gt;26 hours).</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15.95" customFormat="1" customHeight="1" s="246">
+    <row r="20" ht="15.95" customFormat="1" customHeight="1" s="247">
       <c r="A20" s="263" t="inlineStr">
         <is>
           <t>Logging: All output saved to Logs/ folder with timestamps. Mismatches logged to Logs/mismatches.log.</t>

</xml_diff>

<commit_message>
Full backup 12/06/2026 11:38:26
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -802,7 +802,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="20"/>
   </cellStyleXfs>
-  <cellXfs count="295">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1566,6 +1566,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32500,7 +32518,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="37" t="n">
-        <v>850</v>
+        <v>950</v>
       </c>
       <c r="H7" s="38">
         <f>E7+F7-G7</f>
@@ -33040,7 +33058,7 @@
         <v>210</v>
       </c>
       <c r="G22" s="37" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H22" s="38">
         <f>E22+F22-G22</f>
@@ -34050,7 +34068,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="37" t="n">
-        <v>50000</v>
+        <v>70000</v>
       </c>
       <c r="H46" s="38">
         <f>E46+F46-G46</f>
@@ -36082,7 +36100,7 @@
         <v>0</v>
       </c>
       <c r="G94" s="37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H94" s="38">
         <f>E94+F94-G94</f>
@@ -50357,31 +50375,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="237">
-      <c r="A4" s="269" t="n">
+      <c r="A4" s="295" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="269" t="n">
+      <c r="B4" s="295" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="270" t="inlineStr">
+      <c r="C4" s="296" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="270" t="inlineStr">
+      <c r="D4" s="296" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="269" t="inlineStr">
+      <c r="E4" s="295" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="271" t="n">
+      <c r="F4" s="297" t="n">
         <v>10580</v>
       </c>
-      <c r="G4" s="269" t="inlineStr">
+      <c r="G4" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50397,31 +50415,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="237">
-      <c r="A5" s="269" t="n">
+      <c r="A5" s="295" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="269" t="n">
+      <c r="B5" s="295" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="270" t="inlineStr">
+      <c r="C5" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="270" t="inlineStr">
+      <c r="D5" s="296" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="269" t="inlineStr">
+      <c r="E5" s="295" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="271" t="n">
+      <c r="F5" s="297" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="269" t="inlineStr">
+      <c r="G5" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50437,31 +50455,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="237">
-      <c r="A6" s="269" t="n">
+      <c r="A6" s="295" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="269" t="n">
+      <c r="B6" s="295" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="270" t="inlineStr">
+      <c r="C6" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="270" t="inlineStr">
+      <c r="D6" s="296" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="269" t="inlineStr">
+      <c r="E6" s="295" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="271" t="n">
+      <c r="F6" s="297" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="269" t="inlineStr">
+      <c r="G6" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50477,31 +50495,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="237">
-      <c r="A7" s="269" t="n">
+      <c r="A7" s="295" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="269" t="n">
+      <c r="B7" s="295" t="n">
         <v>6470</v>
       </c>
-      <c r="C7" s="270" t="inlineStr">
+      <c r="C7" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D7" s="270" t="inlineStr">
+      <c r="D7" s="296" t="inlineStr">
         <is>
           <t>TUBES COMMON RED</t>
         </is>
       </c>
-      <c r="E7" s="269" t="inlineStr">
+      <c r="E7" s="295" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F7" s="271" t="n">
+      <c r="F7" s="297" t="n">
         <v>60000</v>
       </c>
-      <c r="G7" s="269" t="inlineStr">
+      <c r="G7" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50517,31 +50535,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="237">
-      <c r="A8" s="269" t="n">
+      <c r="A8" s="295" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="269" t="n">
+      <c r="B8" s="295" t="n">
         <v>4050</v>
       </c>
-      <c r="C8" s="270" t="inlineStr">
+      <c r="C8" s="296" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D8" s="270" t="inlineStr">
+      <c r="D8" s="296" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E8" s="269" t="inlineStr">
+      <c r="E8" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="271" t="n">
+      <c r="F8" s="297" t="n">
         <v>9450</v>
       </c>
-      <c r="G8" s="269" t="inlineStr">
+      <c r="G8" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50557,31 +50575,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="237">
-      <c r="A9" s="269" t="n">
+      <c r="A9" s="295" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="269" t="n">
+      <c r="B9" s="295" t="n">
         <v>6337</v>
       </c>
-      <c r="C9" s="270" t="inlineStr">
+      <c r="C9" s="296" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="270" t="inlineStr">
+      <c r="D9" s="296" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="269" t="inlineStr">
+      <c r="E9" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="271" t="n">
+      <c r="F9" s="297" t="n">
         <v>15680</v>
       </c>
-      <c r="G9" s="269" t="inlineStr">
+      <c r="G9" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50597,31 +50615,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="237">
-      <c r="A10" s="269" t="n">
+      <c r="A10" s="295" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="269" t="n">
+      <c r="B10" s="295" t="n">
         <v>6416</v>
       </c>
-      <c r="C10" s="270" t="inlineStr">
+      <c r="C10" s="296" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D10" s="270" t="inlineStr">
+      <c r="D10" s="296" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E10" s="269" t="inlineStr">
+      <c r="E10" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F10" s="271" t="n">
+      <c r="F10" s="297" t="n">
         <v>15435</v>
       </c>
-      <c r="G10" s="269" t="inlineStr">
+      <c r="G10" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50637,31 +50655,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="237">
-      <c r="A11" s="269" t="n">
+      <c r="A11" s="295" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="269" t="n">
+      <c r="B11" s="295" t="n">
         <v>5782</v>
       </c>
-      <c r="C11" s="270" t="inlineStr">
+      <c r="C11" s="296" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D11" s="270" t="inlineStr">
+      <c r="D11" s="296" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E11" s="269" t="inlineStr">
+      <c r="E11" s="295" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F11" s="271" t="n">
+      <c r="F11" s="297" t="n">
         <v>63648</v>
       </c>
-      <c r="G11" s="269" t="inlineStr">
+      <c r="G11" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50677,31 +50695,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="237">
-      <c r="A12" s="269" t="n">
+      <c r="A12" s="295" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="269" t="n">
+      <c r="B12" s="295" t="n">
         <v>6531</v>
       </c>
-      <c r="C12" s="270" t="inlineStr">
+      <c r="C12" s="296" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D12" s="270" t="inlineStr">
+      <c r="D12" s="296" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E12" s="269" t="inlineStr">
+      <c r="E12" s="295" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F12" s="271" t="n">
+      <c r="F12" s="297" t="n">
         <v>4380</v>
       </c>
-      <c r="G12" s="269" t="inlineStr">
+      <c r="G12" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50717,31 +50735,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="237">
-      <c r="A13" s="269" t="n">
+      <c r="A13" s="295" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="269" t="n">
+      <c r="B13" s="295" t="n">
         <v>6206</v>
       </c>
-      <c r="C13" s="270" t="inlineStr">
+      <c r="C13" s="296" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D13" s="270" t="inlineStr">
+      <c r="D13" s="296" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E13" s="269" t="inlineStr">
+      <c r="E13" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F13" s="271" t="n">
+      <c r="F13" s="297" t="n">
         <v>95000</v>
       </c>
-      <c r="G13" s="269" t="inlineStr">
+      <c r="G13" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50757,31 +50775,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="237">
-      <c r="A14" s="273" t="n">
+      <c r="A14" s="298" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="273" t="n">
+      <c r="B14" s="298" t="n">
         <v>6470</v>
       </c>
-      <c r="C14" s="274" t="inlineStr">
+      <c r="C14" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D14" s="274" t="inlineStr">
+      <c r="D14" s="299" t="inlineStr">
         <is>
           <t>TUBES COMMON RED</t>
         </is>
       </c>
-      <c r="E14" s="273" t="inlineStr">
+      <c r="E14" s="298" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F14" s="275" t="n">
+      <c r="F14" s="300" t="n">
         <v>7632</v>
       </c>
-      <c r="G14" s="273" t="inlineStr">
+      <c r="G14" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50797,31 +50815,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="237">
-      <c r="A15" s="273" t="n">
+      <c r="A15" s="298" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="273" t="n">
+      <c r="B15" s="298" t="n">
         <v>6515</v>
       </c>
-      <c r="C15" s="274" t="inlineStr">
+      <c r="C15" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D15" s="274" t="inlineStr">
+      <c r="D15" s="299" t="inlineStr">
         <is>
           <t>H.H 100GM</t>
         </is>
       </c>
-      <c r="E15" s="273" t="inlineStr">
+      <c r="E15" s="298" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F15" s="275" t="n">
+      <c r="F15" s="300" t="n">
         <v>38896</v>
       </c>
-      <c r="G15" s="273" t="inlineStr">
+      <c r="G15" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50837,31 +50855,31 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="237">
-      <c r="A16" s="273" t="n">
+      <c r="A16" s="298" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="273" t="n">
+      <c r="B16" s="298" t="n">
         <v>6530</v>
       </c>
-      <c r="C16" s="274" t="inlineStr">
+      <c r="C16" s="299" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D16" s="274" t="inlineStr">
+      <c r="D16" s="299" t="inlineStr">
         <is>
           <t>V- HC BROWN</t>
         </is>
       </c>
-      <c r="E16" s="273" t="inlineStr">
+      <c r="E16" s="298" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F16" s="275" t="n">
+      <c r="F16" s="300" t="n">
         <v>15000</v>
       </c>
-      <c r="G16" s="273" t="inlineStr">
+      <c r="G16" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50877,31 +50895,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="237">
-      <c r="A17" s="273" t="n">
+      <c r="A17" s="298" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="273" t="n">
+      <c r="B17" s="298" t="n">
         <v>6206</v>
       </c>
-      <c r="C17" s="274" t="inlineStr">
+      <c r="C17" s="299" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D17" s="274" t="inlineStr">
+      <c r="D17" s="299" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E17" s="273" t="inlineStr">
+      <c r="E17" s="298" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F17" s="275" t="n">
+      <c r="F17" s="300" t="n">
         <v>3674</v>
       </c>
-      <c r="G17" s="273" t="inlineStr">
+      <c r="G17" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50917,31 +50935,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="237">
-      <c r="A18" s="273" t="n">
+      <c r="A18" s="298" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="273" t="n">
+      <c r="B18" s="298" t="n">
         <v>5782</v>
       </c>
-      <c r="C18" s="274" t="inlineStr">
+      <c r="C18" s="299" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D18" s="274" t="inlineStr">
+      <c r="D18" s="299" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E18" s="273" t="inlineStr">
+      <c r="E18" s="298" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F18" s="275" t="n">
+      <c r="F18" s="300" t="n">
         <v>10500</v>
       </c>
-      <c r="G18" s="273" t="inlineStr">
+      <c r="G18" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50957,31 +50975,31 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="237">
-      <c r="A19" s="273" t="n">
+      <c r="A19" s="298" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="273" t="n">
+      <c r="B19" s="298" t="n">
         <v>6624</v>
       </c>
-      <c r="C19" s="274" t="inlineStr">
+      <c r="C19" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D19" s="274" t="inlineStr">
+      <c r="D19" s="299" t="inlineStr">
         <is>
           <t>S-45 DIA 19MM</t>
         </is>
       </c>
-      <c r="E19" s="273" t="inlineStr">
+      <c r="E19" s="298" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F19" s="275" t="n">
+      <c r="F19" s="300" t="n">
         <v>15288</v>
       </c>
-      <c r="G19" s="273" t="inlineStr">
+      <c r="G19" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -50997,31 +51015,31 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="237">
-      <c r="A20" s="273" t="n">
+      <c r="A20" s="298" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="273" t="n">
+      <c r="B20" s="298" t="n">
         <v>5731</v>
       </c>
-      <c r="C20" s="274" t="inlineStr">
+      <c r="C20" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D20" s="274" t="inlineStr">
+      <c r="D20" s="299" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E20" s="273" t="inlineStr">
+      <c r="E20" s="298" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F20" s="275" t="n">
+      <c r="F20" s="300" t="n">
         <v>37030</v>
       </c>
-      <c r="G20" s="273" t="inlineStr">
+      <c r="G20" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>

</xml_diff>

<commit_message>
Full backup 13/06/2026 15:30:26
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tubex_Dashboard" sheetId="1" state="visible" r:id="rId1"/>
@@ -685,6 +685,13 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -697,13 +704,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -1299,10 +1299,10 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="46" fillId="10" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1364,20 +1364,20 @@
     <xf numFmtId="0" fontId="49" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="41" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1386,7 +1386,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1394,23 +1394,23 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="36" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="36" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="36" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="36" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="38" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="38" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1422,25 +1422,25 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2049,8 +2049,8 @@
     <col width="14.7109375" customWidth="1" style="227" min="13" max="13"/>
     <col width="13.28515625" customWidth="1" style="227" min="14" max="14"/>
     <col width="9.5703125" customWidth="1" style="227" min="15" max="15"/>
-    <col width="8.7109375" customWidth="1" style="227" min="16" max="53"/>
-    <col width="8.7109375" customWidth="1" style="227" min="54" max="16384"/>
+    <col width="8.7109375" customWidth="1" style="227" min="16" max="54"/>
+    <col width="8.7109375" customWidth="1" style="227" min="55" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="6" customHeight="1" s="237">
@@ -6819,10 +6819,9 @@
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A20)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A20)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A20)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A20)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A20)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A20)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A20)&gt;0)*($H$9&gt;0),$C$9&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A20)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A20)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A20)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A20)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A20)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A20)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A20)&gt;0)*($H$9&gt;0),$C$9&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A20)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A20)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A20)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A20)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A20)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A20)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A20)&gt;0)*($H$9&gt;0),$C$9&amp;", ",""))-2),"")</f>
         <v/>
       </c>
-      <c r="I20" s="30" t="inlineStr">
-        <is>
-          <t>100kg Shortage (16k tubes WIP)</t>
-        </is>
+      <c r="I20" s="30">
+        <f>IF(E20=0,"Not needed",IF(G20&lt;0,"SHORTAGE",IF(G20&lt;F20*0.1,"LOW","OK")))</f>
+        <v/>
       </c>
       <c r="J20" s="30">
         <f>IF(B20&lt;&gt;"CAP","",SUMPRODUCT((ISNUMBER(SEARCH("Cap Not Available",'FG Stock'!$H$4:$H$100)))*('FG Stock'!$I$4:$I$100=A20)*'FG Stock'!$F$4:$F$100))</f>
@@ -13161,19 +13160,19 @@
         <filter val="10"/>
         <filter val="138"/>
         <filter val="15"/>
-        <filter val="169"/>
+        <filter val="167"/>
+        <filter val="183"/>
         <filter val="188"/>
         <filter val="194"/>
         <filter val="2"/>
-        <filter val="232"/>
+        <filter val="25"/>
         <filter val="25,500"/>
         <filter val="3"/>
-        <filter val="30"/>
         <filter val="36,006"/>
-        <filter val="460"/>
+        <filter val="364"/>
+        <filter val="59,135"/>
         <filter val="69"/>
-        <filter val="74,214"/>
-        <filter val="83"/>
+        <filter val="73"/>
         <filter val="89"/>
       </filters>
     </filterColumn>
@@ -38202,7 +38201,7 @@
     <col width="8.85546875" customWidth="1" style="67" min="6" max="6"/>
     <col width="11.140625" customWidth="1" style="67" min="7" max="7"/>
     <col width="8.5703125" customWidth="1" style="68" min="8" max="8"/>
-    <col hidden="1" width="7.7109375" customWidth="1" style="67" min="9" max="9"/>
+    <col width="7.7109375" customWidth="1" style="67" min="9" max="9"/>
     <col width="16.140625" customWidth="1" style="67" min="10" max="10"/>
     <col width="18" customWidth="1" style="237" min="11" max="11"/>
   </cols>

</xml_diff>

<commit_message>
Fix inventory balance calculation and missing active orders due to openpyxl formula data_only=True limitation
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -801,7 +801,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="20"/>
   </cellStyleXfs>
-  <cellXfs count="295">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1565,6 +1565,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -50723,31 +50741,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="237">
-      <c r="A4" s="269" t="n">
+      <c r="A4" s="295" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="269" t="n">
+      <c r="B4" s="295" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="270" t="inlineStr">
+      <c r="C4" s="296" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="270" t="inlineStr">
+      <c r="D4" s="296" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="269" t="inlineStr">
+      <c r="E4" s="295" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="271" t="n">
+      <c r="F4" s="297" t="n">
         <v>10580</v>
       </c>
-      <c r="G4" s="269" t="inlineStr">
+      <c r="G4" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50763,31 +50781,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="237">
-      <c r="A5" s="269" t="n">
+      <c r="A5" s="295" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="269" t="n">
+      <c r="B5" s="295" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="270" t="inlineStr">
+      <c r="C5" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="270" t="inlineStr">
+      <c r="D5" s="296" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="269" t="inlineStr">
+      <c r="E5" s="295" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="271" t="n">
+      <c r="F5" s="297" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="269" t="inlineStr">
+      <c r="G5" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50803,31 +50821,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="237">
-      <c r="A6" s="269" t="n">
+      <c r="A6" s="295" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="269" t="n">
+      <c r="B6" s="295" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="270" t="inlineStr">
+      <c r="C6" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="270" t="inlineStr">
+      <c r="D6" s="296" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="269" t="inlineStr">
+      <c r="E6" s="295" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="271" t="n">
+      <c r="F6" s="297" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="269" t="inlineStr">
+      <c r="G6" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50843,31 +50861,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="237">
-      <c r="A7" s="269" t="n">
+      <c r="A7" s="295" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="269" t="n">
+      <c r="B7" s="295" t="n">
         <v>4050</v>
       </c>
-      <c r="C7" s="270" t="inlineStr">
+      <c r="C7" s="296" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D7" s="270" t="inlineStr">
+      <c r="D7" s="296" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E7" s="269" t="inlineStr">
+      <c r="E7" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F7" s="271" t="n">
+      <c r="F7" s="297" t="n">
         <v>9450</v>
       </c>
-      <c r="G7" s="269" t="inlineStr">
+      <c r="G7" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50883,31 +50901,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="237">
-      <c r="A8" s="269" t="n">
+      <c r="A8" s="295" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="269" t="n">
+      <c r="B8" s="295" t="n">
         <v>6337</v>
       </c>
-      <c r="C8" s="270" t="inlineStr">
+      <c r="C8" s="296" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D8" s="270" t="inlineStr">
+      <c r="D8" s="296" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E8" s="269" t="inlineStr">
+      <c r="E8" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="271" t="n">
+      <c r="F8" s="297" t="n">
         <v>15680</v>
       </c>
-      <c r="G8" s="269" t="inlineStr">
+      <c r="G8" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50923,31 +50941,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="237">
-      <c r="A9" s="269" t="n">
+      <c r="A9" s="295" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="269" t="n">
+      <c r="B9" s="295" t="n">
         <v>6416</v>
       </c>
-      <c r="C9" s="270" t="inlineStr">
+      <c r="C9" s="296" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="270" t="inlineStr">
+      <c r="D9" s="296" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="269" t="inlineStr">
+      <c r="E9" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="271" t="n">
+      <c r="F9" s="297" t="n">
         <v>15435</v>
       </c>
-      <c r="G9" s="269" t="inlineStr">
+      <c r="G9" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50963,31 +50981,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="237">
-      <c r="A10" s="269" t="n">
+      <c r="A10" s="295" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="269" t="n">
+      <c r="B10" s="295" t="n">
         <v>5782</v>
       </c>
-      <c r="C10" s="270" t="inlineStr">
+      <c r="C10" s="296" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D10" s="270" t="inlineStr">
+      <c r="D10" s="296" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E10" s="269" t="inlineStr">
+      <c r="E10" s="295" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F10" s="271" t="n">
+      <c r="F10" s="297" t="n">
         <v>63648</v>
       </c>
-      <c r="G10" s="269" t="inlineStr">
+      <c r="G10" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51003,31 +51021,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="237">
-      <c r="A11" s="269" t="n">
+      <c r="A11" s="295" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="269" t="n">
+      <c r="B11" s="295" t="n">
         <v>6531</v>
       </c>
-      <c r="C11" s="270" t="inlineStr">
+      <c r="C11" s="296" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D11" s="270" t="inlineStr">
+      <c r="D11" s="296" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E11" s="269" t="inlineStr">
+      <c r="E11" s="295" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F11" s="271" t="n">
+      <c r="F11" s="297" t="n">
         <v>4380</v>
       </c>
-      <c r="G11" s="269" t="inlineStr">
+      <c r="G11" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51043,31 +51061,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="237">
-      <c r="A12" s="269" t="n">
+      <c r="A12" s="295" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="269" t="n">
+      <c r="B12" s="295" t="n">
         <v>6532</v>
       </c>
-      <c r="C12" s="270" t="inlineStr">
+      <c r="C12" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D12" s="270" t="inlineStr">
+      <c r="D12" s="296" t="inlineStr">
         <is>
           <t>TUBE COMMON PURPLE</t>
         </is>
       </c>
-      <c r="E12" s="269" t="inlineStr">
+      <c r="E12" s="295" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F12" s="271" t="n">
+      <c r="F12" s="297" t="n">
         <v>31248</v>
       </c>
-      <c r="G12" s="269" t="inlineStr">
+      <c r="G12" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51083,31 +51101,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="237">
-      <c r="A13" s="269" t="n">
+      <c r="A13" s="295" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="269" t="n">
+      <c r="B13" s="295" t="n">
         <v>6206</v>
       </c>
-      <c r="C13" s="270" t="inlineStr">
+      <c r="C13" s="296" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D13" s="270" t="inlineStr">
+      <c r="D13" s="296" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E13" s="269" t="inlineStr">
+      <c r="E13" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F13" s="271" t="n">
+      <c r="F13" s="297" t="n">
         <v>100674</v>
       </c>
-      <c r="G13" s="269" t="inlineStr">
+      <c r="G13" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51123,31 +51141,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="237">
-      <c r="A14" s="273" t="n">
+      <c r="A14" s="298" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="273" t="n">
+      <c r="B14" s="298" t="n">
         <v>6470</v>
       </c>
-      <c r="C14" s="274" t="inlineStr">
+      <c r="C14" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D14" s="274" t="inlineStr">
+      <c r="D14" s="299" t="inlineStr">
         <is>
           <t>TUBES COMMON RED</t>
         </is>
       </c>
-      <c r="E14" s="273" t="inlineStr">
+      <c r="E14" s="298" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F14" s="275" t="n">
+      <c r="F14" s="300" t="n">
         <v>7632</v>
       </c>
-      <c r="G14" s="273" t="inlineStr">
+      <c r="G14" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51163,31 +51181,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="237">
-      <c r="A15" s="273" t="n">
+      <c r="A15" s="298" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="273" t="n">
+      <c r="B15" s="298" t="n">
         <v>6515</v>
       </c>
-      <c r="C15" s="274" t="inlineStr">
+      <c r="C15" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D15" s="274" t="inlineStr">
+      <c r="D15" s="299" t="inlineStr">
         <is>
           <t>H.H 100GM</t>
         </is>
       </c>
-      <c r="E15" s="273" t="inlineStr">
+      <c r="E15" s="298" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F15" s="275" t="n">
+      <c r="F15" s="300" t="n">
         <v>38896</v>
       </c>
-      <c r="G15" s="273" t="inlineStr">
+      <c r="G15" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51203,31 +51221,31 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="237">
-      <c r="A16" s="273" t="n">
+      <c r="A16" s="298" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="273" t="n">
+      <c r="B16" s="298" t="n">
         <v>6530</v>
       </c>
-      <c r="C16" s="274" t="inlineStr">
+      <c r="C16" s="299" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D16" s="274" t="inlineStr">
+      <c r="D16" s="299" t="inlineStr">
         <is>
           <t>V- HC BROWN</t>
         </is>
       </c>
-      <c r="E16" s="273" t="inlineStr">
+      <c r="E16" s="298" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F16" s="275" t="n">
+      <c r="F16" s="300" t="n">
         <v>15000</v>
       </c>
-      <c r="G16" s="273" t="inlineStr">
+      <c r="G16" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51243,31 +51261,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="237">
-      <c r="A17" s="273" t="n">
+      <c r="A17" s="298" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="273" t="n">
+      <c r="B17" s="298" t="n">
         <v>5782</v>
       </c>
-      <c r="C17" s="274" t="inlineStr">
+      <c r="C17" s="299" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D17" s="274" t="inlineStr">
+      <c r="D17" s="299" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E17" s="273" t="inlineStr">
+      <c r="E17" s="298" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F17" s="275" t="n">
+      <c r="F17" s="300" t="n">
         <v>10500</v>
       </c>
-      <c r="G17" s="273" t="inlineStr">
+      <c r="G17" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51283,31 +51301,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="237">
-      <c r="A18" s="273" t="n">
+      <c r="A18" s="298" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="273" t="n">
+      <c r="B18" s="298" t="n">
         <v>6624</v>
       </c>
-      <c r="C18" s="274" t="inlineStr">
+      <c r="C18" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="274" t="inlineStr">
+      <c r="D18" s="299" t="inlineStr">
         <is>
           <t>S-45 DIA 19MM</t>
         </is>
       </c>
-      <c r="E18" s="273" t="inlineStr">
+      <c r="E18" s="298" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F18" s="275" t="n">
+      <c r="F18" s="300" t="n">
         <v>15288</v>
       </c>
-      <c r="G18" s="273" t="inlineStr">
+      <c r="G18" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51323,31 +51341,31 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="237">
-      <c r="A19" s="273" t="n">
+      <c r="A19" s="298" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="273" t="n">
+      <c r="B19" s="298" t="n">
         <v>5731</v>
       </c>
-      <c r="C19" s="274" t="inlineStr">
+      <c r="C19" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D19" s="274" t="inlineStr">
+      <c r="D19" s="299" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E19" s="273" t="inlineStr">
+      <c r="E19" s="298" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F19" s="275" t="n">
+      <c r="F19" s="300" t="n">
         <v>37030</v>
       </c>
-      <c r="G19" s="273" t="inlineStr">
+      <c r="G19" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>

</xml_diff>

<commit_message>
Full backup 15/06/2026 10:20:39
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -801,7 +801,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="20"/>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="307">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1583,6 +1583,24 @@
     <xf numFmtId="3" fontId="47" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -16872,193 +16890,398 @@
       <c r="S83" s="265" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1" s="237">
-      <c r="A84" s="176" t="n"/>
-      <c r="B84" s="177" t="n"/>
-      <c r="C84" s="177" t="n"/>
-      <c r="D84" s="177" t="n"/>
-      <c r="E84" s="177" t="n"/>
-      <c r="F84" s="177" t="n"/>
-      <c r="G84" s="178" t="n"/>
-      <c r="H84" s="178" t="n"/>
-      <c r="I84" s="178" t="n"/>
-      <c r="J84" s="179" t="n"/>
-      <c r="K84" s="177" t="n"/>
-      <c r="L84" s="177" t="n"/>
-      <c r="M84" s="177" t="n"/>
-      <c r="N84" s="177" t="n"/>
-      <c r="O84" s="177" t="n"/>
-      <c r="P84" s="177" t="n"/>
-      <c r="Q84" s="177" t="n"/>
-      <c r="R84" s="177" t="n"/>
-      <c r="S84" s="177" t="n"/>
+      <c r="A84" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B84" s="265" t="inlineStr">
+        <is>
+          <t>Lacquer-02</t>
+        </is>
+      </c>
+      <c r="C84" s="265" t="inlineStr"/>
+      <c r="D84" s="265" t="inlineStr"/>
+      <c r="E84" s="265" t="inlineStr"/>
+      <c r="F84" s="265" t="n"/>
+      <c r="G84" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" s="267">
+        <f>IFERROR(I84/(H84+I84),"")</f>
+        <v/>
+      </c>
+      <c r="K84" s="265" t="n"/>
+      <c r="L84" s="265" t="n"/>
+      <c r="M84" s="265" t="n"/>
+      <c r="N84" s="265" t="n"/>
+      <c r="O84" s="265" t="n"/>
+      <c r="P84" s="265" t="n"/>
+      <c r="Q84" s="265" t="n"/>
+      <c r="R84" s="265" t="n"/>
+      <c r="S84" s="265" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="237">
-      <c r="A85" s="176" t="n"/>
-      <c r="B85" s="177" t="n"/>
-      <c r="C85" s="177" t="n"/>
-      <c r="D85" s="177" t="n"/>
-      <c r="E85" s="177" t="n"/>
-      <c r="F85" s="177" t="n"/>
-      <c r="G85" s="178" t="n"/>
-      <c r="H85" s="178" t="n"/>
-      <c r="I85" s="178" t="n"/>
-      <c r="J85" s="179" t="n"/>
-      <c r="K85" s="177" t="n"/>
-      <c r="L85" s="177" t="n"/>
-      <c r="M85" s="177" t="n"/>
-      <c r="N85" s="177" t="n"/>
-      <c r="O85" s="177" t="n"/>
-      <c r="P85" s="177" t="n"/>
-      <c r="Q85" s="177" t="n"/>
-      <c r="R85" s="177" t="n"/>
-      <c r="S85" s="177" t="n"/>
+      <c r="A85" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B85" s="265" t="inlineStr">
+        <is>
+          <t>Lacquer-04</t>
+        </is>
+      </c>
+      <c r="C85" s="265" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D85" s="265" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="E85" s="265" t="n">
+        <v>25</v>
+      </c>
+      <c r="F85" s="265" t="n">
+        <v>5389</v>
+      </c>
+      <c r="G85" s="266" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H85" s="266" t="n">
+        <v>14775</v>
+      </c>
+      <c r="I85" s="266" t="n">
+        <v>225</v>
+      </c>
+      <c r="J85" s="267">
+        <f>IFERROR(I85/(H85+I85),"")</f>
+        <v/>
+      </c>
+      <c r="K85" s="265" t="n"/>
+      <c r="L85" s="265" t="n"/>
+      <c r="M85" s="265" t="n"/>
+      <c r="N85" s="265" t="n"/>
+      <c r="O85" s="265" t="n"/>
+      <c r="P85" s="265" t="n"/>
+      <c r="Q85" s="265" t="n"/>
+      <c r="R85" s="265" t="n"/>
+      <c r="S85" s="265" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="237">
-      <c r="A86" s="176" t="n"/>
-      <c r="B86" s="177" t="n"/>
-      <c r="C86" s="177" t="n"/>
-      <c r="D86" s="177" t="n"/>
-      <c r="E86" s="177" t="n"/>
-      <c r="F86" s="177" t="n"/>
-      <c r="G86" s="178" t="n"/>
-      <c r="H86" s="178" t="n"/>
-      <c r="I86" s="178" t="n"/>
-      <c r="J86" s="179" t="n"/>
-      <c r="K86" s="177" t="n"/>
-      <c r="L86" s="177" t="n"/>
-      <c r="M86" s="177" t="n"/>
-      <c r="N86" s="177" t="n"/>
-      <c r="O86" s="177" t="n"/>
-      <c r="P86" s="177" t="n"/>
-      <c r="Q86" s="177" t="n"/>
-      <c r="R86" s="177" t="n"/>
-      <c r="S86" s="177" t="n"/>
+      <c r="A86" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B86" s="265" t="inlineStr">
+        <is>
+          <t>Latex-01</t>
+        </is>
+      </c>
+      <c r="C86" s="265" t="inlineStr"/>
+      <c r="D86" s="265" t="inlineStr"/>
+      <c r="E86" s="265" t="inlineStr"/>
+      <c r="F86" s="265" t="n"/>
+      <c r="G86" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" s="267">
+        <f>IFERROR(I86/(H86+I86),"")</f>
+        <v/>
+      </c>
+      <c r="K86" s="265" t="n"/>
+      <c r="L86" s="265" t="n"/>
+      <c r="M86" s="265" t="n"/>
+      <c r="N86" s="265" t="n"/>
+      <c r="O86" s="265" t="n"/>
+      <c r="P86" s="265" t="n"/>
+      <c r="Q86" s="265" t="n"/>
+      <c r="R86" s="265" t="n"/>
+      <c r="S86" s="265" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="237">
-      <c r="A87" s="176" t="n"/>
-      <c r="B87" s="177" t="n"/>
-      <c r="C87" s="177" t="n"/>
-      <c r="D87" s="177" t="n"/>
-      <c r="E87" s="177" t="n"/>
-      <c r="F87" s="177" t="n"/>
-      <c r="G87" s="178" t="n"/>
-      <c r="H87" s="178" t="n"/>
-      <c r="I87" s="178" t="n"/>
-      <c r="J87" s="179" t="n"/>
-      <c r="K87" s="177" t="n"/>
-      <c r="L87" s="177" t="n"/>
-      <c r="M87" s="177" t="n"/>
-      <c r="N87" s="177" t="n"/>
-      <c r="O87" s="177" t="n"/>
-      <c r="P87" s="177" t="n"/>
-      <c r="Q87" s="177" t="n"/>
-      <c r="R87" s="177" t="n"/>
-      <c r="S87" s="177" t="n"/>
+      <c r="A87" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B87" s="265" t="inlineStr">
+        <is>
+          <t>PF Machine</t>
+        </is>
+      </c>
+      <c r="C87" s="265" t="inlineStr">
+        <is>
+          <t>Alpha Labs PVT LTD</t>
+        </is>
+      </c>
+      <c r="D87" s="265" t="inlineStr">
+        <is>
+          <t>TRANSPARENT BOTTLE 150ML</t>
+        </is>
+      </c>
+      <c r="E87" s="265" t="inlineStr">
+        <is>
+          <t>150 ml</t>
+        </is>
+      </c>
+      <c r="F87" s="265" t="n">
+        <v>8001</v>
+      </c>
+      <c r="G87" s="266" t="n">
+        <v>9030</v>
+      </c>
+      <c r="H87" s="266" t="n">
+        <v>8280</v>
+      </c>
+      <c r="I87" s="266" t="n">
+        <v>750</v>
+      </c>
+      <c r="J87" s="267">
+        <f>IFERROR(I87/(H87+I87),"")</f>
+        <v/>
+      </c>
+      <c r="K87" s="265" t="n"/>
+      <c r="L87" s="265" t="n"/>
+      <c r="M87" s="265" t="n"/>
+      <c r="N87" s="265" t="n"/>
+      <c r="O87" s="265" t="n"/>
+      <c r="P87" s="265" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q87" s="265" t="n"/>
+      <c r="R87" s="265" t="n"/>
+      <c r="S87" s="265" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="237">
-      <c r="A88" s="176" t="n"/>
-      <c r="B88" s="177" t="n"/>
-      <c r="C88" s="177" t="n"/>
-      <c r="D88" s="177" t="n"/>
-      <c r="E88" s="177" t="n"/>
-      <c r="F88" s="177" t="n"/>
-      <c r="G88" s="178" t="n"/>
-      <c r="H88" s="178" t="n"/>
-      <c r="I88" s="178" t="n"/>
-      <c r="J88" s="179" t="n"/>
-      <c r="K88" s="177" t="n"/>
-      <c r="L88" s="177" t="n"/>
-      <c r="M88" s="177" t="n"/>
-      <c r="N88" s="177" t="n"/>
-      <c r="O88" s="177" t="n"/>
-      <c r="P88" s="177" t="n"/>
-      <c r="Q88" s="177" t="n"/>
-      <c r="R88" s="177" t="n"/>
-      <c r="S88" s="177" t="n"/>
+      <c r="A88" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B88" s="265" t="inlineStr">
+        <is>
+          <t>Press-04</t>
+        </is>
+      </c>
+      <c r="C88" s="265" t="inlineStr"/>
+      <c r="D88" s="265" t="inlineStr"/>
+      <c r="E88" s="265" t="inlineStr"/>
+      <c r="F88" s="265" t="n"/>
+      <c r="G88" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" s="267">
+        <f>IFERROR(I88/(H88+I88),"")</f>
+        <v/>
+      </c>
+      <c r="K88" s="265" t="n"/>
+      <c r="L88" s="265" t="n"/>
+      <c r="M88" s="265" t="n"/>
+      <c r="N88" s="265" t="n"/>
+      <c r="O88" s="265" t="n"/>
+      <c r="P88" s="265" t="n"/>
+      <c r="Q88" s="265" t="n"/>
+      <c r="R88" s="265" t="n"/>
+      <c r="S88" s="265" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1" s="237">
-      <c r="A89" s="176" t="n"/>
-      <c r="B89" s="177" t="n"/>
-      <c r="C89" s="177" t="n"/>
-      <c r="D89" s="177" t="n"/>
-      <c r="E89" s="177" t="n"/>
-      <c r="F89" s="177" t="n"/>
-      <c r="G89" s="178" t="n"/>
-      <c r="H89" s="178" t="n"/>
-      <c r="I89" s="178" t="n"/>
-      <c r="J89" s="179" t="n"/>
-      <c r="K89" s="177" t="n"/>
-      <c r="L89" s="177" t="n"/>
-      <c r="M89" s="177" t="n"/>
-      <c r="N89" s="177" t="n"/>
-      <c r="O89" s="177" t="n"/>
-      <c r="P89" s="177" t="n"/>
-      <c r="Q89" s="177" t="n"/>
-      <c r="R89" s="177" t="n"/>
-      <c r="S89" s="177" t="n"/>
+      <c r="A89" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B89" s="265" t="inlineStr">
+        <is>
+          <t>Press-06</t>
+        </is>
+      </c>
+      <c r="C89" s="265" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D89" s="265" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="E89" s="265" t="n">
+        <v>25</v>
+      </c>
+      <c r="F89" s="265" t="n">
+        <v>5389</v>
+      </c>
+      <c r="G89" s="266" t="n">
+        <v>19500</v>
+      </c>
+      <c r="H89" s="266" t="n">
+        <v>19345</v>
+      </c>
+      <c r="I89" s="266" t="n">
+        <v>155</v>
+      </c>
+      <c r="J89" s="267">
+        <f>IFERROR(I89/(H89+I89),"")</f>
+        <v/>
+      </c>
+      <c r="K89" s="265" t="n"/>
+      <c r="L89" s="265" t="n"/>
+      <c r="M89" s="265" t="n"/>
+      <c r="N89" s="265" t="n"/>
+      <c r="O89" s="265" t="n"/>
+      <c r="P89" s="265" t="n"/>
+      <c r="Q89" s="265" t="n"/>
+      <c r="R89" s="265" t="n"/>
+      <c r="S89" s="265" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1" s="237">
-      <c r="A90" s="176" t="n"/>
-      <c r="B90" s="177" t="n"/>
-      <c r="C90" s="177" t="n"/>
-      <c r="D90" s="177" t="n"/>
-      <c r="E90" s="177" t="n"/>
-      <c r="F90" s="177" t="n"/>
-      <c r="G90" s="178" t="n"/>
-      <c r="H90" s="178" t="n"/>
-      <c r="I90" s="178" t="n"/>
-      <c r="J90" s="179" t="n"/>
-      <c r="K90" s="177" t="n"/>
-      <c r="L90" s="177" t="n"/>
-      <c r="M90" s="177" t="n"/>
-      <c r="N90" s="177" t="n"/>
-      <c r="O90" s="177" t="n"/>
-      <c r="P90" s="177" t="n"/>
-      <c r="Q90" s="177" t="n"/>
-      <c r="R90" s="177" t="n"/>
-      <c r="S90" s="177" t="n"/>
+      <c r="A90" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B90" s="265" t="inlineStr">
+        <is>
+          <t>Printing-03</t>
+        </is>
+      </c>
+      <c r="C90" s="265" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D90" s="265" t="inlineStr">
+        <is>
+          <t>TUBE COMMON PURPLE</t>
+        </is>
+      </c>
+      <c r="E90" s="265" t="n">
+        <v>25</v>
+      </c>
+      <c r="F90" s="265" t="n">
+        <v>6532</v>
+      </c>
+      <c r="G90" s="266" t="n">
+        <v>3188</v>
+      </c>
+      <c r="H90" s="266" t="n">
+        <v>3024</v>
+      </c>
+      <c r="I90" s="266" t="n">
+        <v>164</v>
+      </c>
+      <c r="J90" s="267">
+        <f>IFERROR(I90/(H90+I90),"")</f>
+        <v/>
+      </c>
+      <c r="K90" s="265" t="n"/>
+      <c r="L90" s="265" t="n"/>
+      <c r="M90" s="265" t="n"/>
+      <c r="N90" s="265" t="n">
+        <v>20</v>
+      </c>
+      <c r="O90" s="265" t="n"/>
+      <c r="P90" s="265" t="n"/>
+      <c r="Q90" s="265" t="n"/>
+      <c r="R90" s="265" t="n"/>
+      <c r="S90" s="265" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1" s="237">
-      <c r="A91" s="176" t="n"/>
-      <c r="B91" s="177" t="n"/>
-      <c r="C91" s="177" t="n"/>
-      <c r="D91" s="177" t="n"/>
-      <c r="E91" s="177" t="n"/>
-      <c r="F91" s="177" t="n"/>
-      <c r="G91" s="178" t="n"/>
-      <c r="H91" s="178" t="n"/>
-      <c r="I91" s="178" t="n"/>
-      <c r="J91" s="179" t="n"/>
-      <c r="K91" s="177" t="n"/>
-      <c r="L91" s="177" t="n"/>
-      <c r="M91" s="177" t="n"/>
-      <c r="N91" s="177" t="n"/>
-      <c r="O91" s="177" t="n"/>
-      <c r="P91" s="177" t="n"/>
-      <c r="Q91" s="177" t="n"/>
-      <c r="R91" s="177" t="n"/>
-      <c r="S91" s="177" t="n"/>
+      <c r="A91" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B91" s="265" t="inlineStr">
+        <is>
+          <t>Printing-03</t>
+        </is>
+      </c>
+      <c r="C91" s="265" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D91" s="265" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="E91" s="265" t="n">
+        <v>25</v>
+      </c>
+      <c r="F91" s="265" t="n">
+        <v>5389</v>
+      </c>
+      <c r="G91" s="266" t="n">
+        <v>12762</v>
+      </c>
+      <c r="H91" s="266" t="n">
+        <v>12432</v>
+      </c>
+      <c r="I91" s="266" t="n">
+        <v>330</v>
+      </c>
+      <c r="J91" s="267">
+        <f>IFERROR(I91/(H91+I91),"")</f>
+        <v/>
+      </c>
+      <c r="K91" s="265" t="n"/>
+      <c r="L91" s="265" t="n"/>
+      <c r="M91" s="265" t="n"/>
+      <c r="N91" s="265" t="n"/>
+      <c r="O91" s="265" t="n"/>
+      <c r="P91" s="265" t="n"/>
+      <c r="Q91" s="265" t="n"/>
+      <c r="R91" s="265" t="n"/>
+      <c r="S91" s="265" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1" s="237">
-      <c r="A92" s="176" t="n"/>
-      <c r="B92" s="177" t="n"/>
-      <c r="C92" s="177" t="n"/>
-      <c r="D92" s="177" t="n"/>
-      <c r="E92" s="177" t="n"/>
-      <c r="F92" s="177" t="n"/>
-      <c r="G92" s="178" t="n"/>
-      <c r="H92" s="178" t="n"/>
-      <c r="I92" s="178" t="n"/>
-      <c r="J92" s="179" t="n"/>
-      <c r="K92" s="177" t="n"/>
-      <c r="L92" s="177" t="n"/>
-      <c r="M92" s="177" t="n"/>
-      <c r="N92" s="177" t="n"/>
-      <c r="O92" s="177" t="n"/>
-      <c r="P92" s="177" t="n"/>
-      <c r="Q92" s="177" t="n"/>
-      <c r="R92" s="177" t="n"/>
-      <c r="S92" s="177" t="n"/>
+      <c r="A92" s="268" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B92" s="265" t="inlineStr">
+        <is>
+          <t>Printing-04</t>
+        </is>
+      </c>
+      <c r="C92" s="265" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D92" s="265" t="inlineStr"/>
+      <c r="E92" s="265" t="inlineStr"/>
+      <c r="F92" s="265" t="n"/>
+      <c r="G92" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" s="266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" s="267">
+        <f>IFERROR(I92/(H92+I92),"")</f>
+        <v/>
+      </c>
+      <c r="K92" s="265" t="n"/>
+      <c r="L92" s="265" t="n"/>
+      <c r="M92" s="265" t="n"/>
+      <c r="N92" s="265" t="n"/>
+      <c r="O92" s="265" t="n"/>
+      <c r="P92" s="265" t="n"/>
+      <c r="Q92" s="265" t="n"/>
+      <c r="R92" s="265" t="n"/>
+      <c r="S92" s="265" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="237">
       <c r="A93" s="176" t="n"/>
@@ -50682,7 +50905,7 @@
     <row r="1" ht="30" customHeight="1" s="237">
       <c r="A1" s="259" t="inlineStr">
         <is>
-          <t>FG STOCK IN HAND — Last Updated: 13-Jun-2026</t>
+          <t>FG STOCK IN HAND — Last Updated: 15-Jun-2026</t>
         </is>
       </c>
     </row>
@@ -50741,31 +50964,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="237">
-      <c r="A4" s="295" t="n">
+      <c r="A4" s="301" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="295" t="n">
+      <c r="B4" s="301" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="296" t="inlineStr">
+      <c r="C4" s="302" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="296" t="inlineStr">
+      <c r="D4" s="302" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="295" t="inlineStr">
+      <c r="E4" s="301" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="297" t="n">
-        <v>10580</v>
-      </c>
-      <c r="G4" s="295" t="inlineStr">
+      <c r="F4" s="303" t="n">
+        <v>18860</v>
+      </c>
+      <c r="G4" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50781,31 +51004,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="237">
-      <c r="A5" s="295" t="n">
+      <c r="A5" s="301" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="295" t="n">
+      <c r="B5" s="301" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="296" t="inlineStr">
+      <c r="C5" s="302" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="296" t="inlineStr">
+      <c r="D5" s="302" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="295" t="inlineStr">
+      <c r="E5" s="301" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="297" t="n">
+      <c r="F5" s="303" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="295" t="inlineStr">
+      <c r="G5" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50821,31 +51044,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="237">
-      <c r="A6" s="295" t="n">
+      <c r="A6" s="301" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="295" t="n">
+      <c r="B6" s="301" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="296" t="inlineStr">
+      <c r="C6" s="302" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="296" t="inlineStr">
+      <c r="D6" s="302" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="295" t="inlineStr">
+      <c r="E6" s="301" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="297" t="n">
+      <c r="F6" s="303" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="295" t="inlineStr">
+      <c r="G6" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50861,31 +51084,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="237">
-      <c r="A7" s="295" t="n">
+      <c r="A7" s="301" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="295" t="n">
-        <v>4050</v>
-      </c>
-      <c r="C7" s="296" t="inlineStr">
-        <is>
-          <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
-        </is>
-      </c>
-      <c r="D7" s="296" t="inlineStr">
-        <is>
-          <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
-        </is>
-      </c>
-      <c r="E7" s="295" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="F7" s="297" t="n">
-        <v>9450</v>
-      </c>
-      <c r="G7" s="295" t="inlineStr">
+      <c r="B7" s="301" t="n">
+        <v>5389</v>
+      </c>
+      <c r="C7" s="302" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D7" s="302" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="E7" s="301" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F7" s="303" t="n">
+        <v>11088</v>
+      </c>
+      <c r="G7" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50901,31 +51124,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="237">
-      <c r="A8" s="295" t="n">
+      <c r="A8" s="301" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="295" t="n">
-        <v>6337</v>
-      </c>
-      <c r="C8" s="296" t="inlineStr">
-        <is>
-          <t>Al-Rehman Group</t>
-        </is>
-      </c>
-      <c r="D8" s="296" t="inlineStr">
-        <is>
-          <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
-        </is>
-      </c>
-      <c r="E8" s="295" t="inlineStr">
+      <c r="B8" s="301" t="n">
+        <v>4050</v>
+      </c>
+      <c r="C8" s="302" t="inlineStr">
+        <is>
+          <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
+        </is>
+      </c>
+      <c r="D8" s="302" t="inlineStr">
+        <is>
+          <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
+        </is>
+      </c>
+      <c r="E8" s="301" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="297" t="n">
-        <v>15680</v>
-      </c>
-      <c r="G8" s="295" t="inlineStr">
+      <c r="F8" s="303" t="n">
+        <v>9450</v>
+      </c>
+      <c r="G8" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50941,31 +51164,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="237">
-      <c r="A9" s="295" t="n">
+      <c r="A9" s="301" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="295" t="n">
-        <v>6416</v>
-      </c>
-      <c r="C9" s="296" t="inlineStr">
+      <c r="B9" s="301" t="n">
+        <v>6337</v>
+      </c>
+      <c r="C9" s="302" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="296" t="inlineStr">
-        <is>
-          <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
-        </is>
-      </c>
-      <c r="E9" s="295" t="inlineStr">
+      <c r="D9" s="302" t="inlineStr">
+        <is>
+          <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
+        </is>
+      </c>
+      <c r="E9" s="301" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="297" t="n">
-        <v>15435</v>
-      </c>
-      <c r="G9" s="295" t="inlineStr">
+      <c r="F9" s="303" t="n">
+        <v>15680</v>
+      </c>
+      <c r="G9" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -50981,31 +51204,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="237">
-      <c r="A10" s="295" t="n">
+      <c r="A10" s="301" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="295" t="n">
-        <v>5782</v>
-      </c>
-      <c r="C10" s="296" t="inlineStr">
-        <is>
-          <t>Mega Grey</t>
-        </is>
-      </c>
-      <c r="D10" s="296" t="inlineStr">
-        <is>
-          <t>M.G</t>
-        </is>
-      </c>
-      <c r="E10" s="295" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F10" s="297" t="n">
-        <v>63648</v>
-      </c>
-      <c r="G10" s="295" t="inlineStr">
+      <c r="B10" s="301" t="n">
+        <v>6416</v>
+      </c>
+      <c r="C10" s="302" t="inlineStr">
+        <is>
+          <t>Al-Rehman Group</t>
+        </is>
+      </c>
+      <c r="D10" s="302" t="inlineStr">
+        <is>
+          <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
+        </is>
+      </c>
+      <c r="E10" s="301" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F10" s="303" t="n">
+        <v>15435</v>
+      </c>
+      <c r="G10" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51021,31 +51244,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="237">
-      <c r="A11" s="295" t="n">
+      <c r="A11" s="301" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="295" t="n">
-        <v>6531</v>
-      </c>
-      <c r="C11" s="296" t="inlineStr">
-        <is>
-          <t>Adore</t>
-        </is>
-      </c>
-      <c r="D11" s="296" t="inlineStr">
-        <is>
-          <t>V-HC BLACK</t>
-        </is>
-      </c>
-      <c r="E11" s="295" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F11" s="297" t="n">
-        <v>4380</v>
-      </c>
-      <c r="G11" s="295" t="inlineStr">
+      <c r="B11" s="301" t="n">
+        <v>5782</v>
+      </c>
+      <c r="C11" s="302" t="inlineStr">
+        <is>
+          <t>Mega Grey</t>
+        </is>
+      </c>
+      <c r="D11" s="302" t="inlineStr">
+        <is>
+          <t>M.G</t>
+        </is>
+      </c>
+      <c r="E11" s="301" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F11" s="303" t="n">
+        <v>63648</v>
+      </c>
+      <c r="G11" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51061,31 +51284,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="237">
-      <c r="A12" s="295" t="n">
+      <c r="A12" s="301" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="295" t="n">
-        <v>6532</v>
-      </c>
-      <c r="C12" s="296" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D12" s="296" t="inlineStr">
-        <is>
-          <t>TUBE COMMON PURPLE</t>
-        </is>
-      </c>
-      <c r="E12" s="295" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F12" s="297" t="n">
-        <v>31248</v>
-      </c>
-      <c r="G12" s="295" t="inlineStr">
+      <c r="B12" s="301" t="n">
+        <v>6531</v>
+      </c>
+      <c r="C12" s="302" t="inlineStr">
+        <is>
+          <t>Adore</t>
+        </is>
+      </c>
+      <c r="D12" s="302" t="inlineStr">
+        <is>
+          <t>V-HC BLACK</t>
+        </is>
+      </c>
+      <c r="E12" s="301" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F12" s="303" t="n">
+        <v>4380</v>
+      </c>
+      <c r="G12" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51101,31 +51324,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="237">
-      <c r="A13" s="295" t="n">
+      <c r="A13" s="301" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="295" t="n">
+      <c r="B13" s="301" t="n">
         <v>6206</v>
       </c>
-      <c r="C13" s="296" t="inlineStr">
+      <c r="C13" s="302" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D13" s="296" t="inlineStr">
+      <c r="D13" s="302" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E13" s="295" t="inlineStr">
+      <c r="E13" s="301" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F13" s="297" t="n">
+      <c r="F13" s="303" t="n">
         <v>100674</v>
       </c>
-      <c r="G13" s="295" t="inlineStr">
+      <c r="G13" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51141,31 +51364,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="237">
-      <c r="A14" s="298" t="n">
+      <c r="A14" s="304" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="298" t="n">
-        <v>6470</v>
-      </c>
-      <c r="C14" s="299" t="inlineStr">
+      <c r="B14" s="304" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C14" s="305" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D14" s="299" t="inlineStr">
-        <is>
-          <t>TUBES COMMON RED</t>
-        </is>
-      </c>
-      <c r="E14" s="298" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F14" s="300" t="n">
-        <v>7632</v>
-      </c>
-      <c r="G14" s="298" t="inlineStr">
+      <c r="D14" s="305" t="inlineStr">
+        <is>
+          <t>H.H 100GM</t>
+        </is>
+      </c>
+      <c r="E14" s="304" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F14" s="306" t="n">
+        <v>38896</v>
+      </c>
+      <c r="G14" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51181,38 +51404,38 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="237">
-      <c r="A15" s="298" t="n">
+      <c r="A15" s="304" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="298" t="n">
-        <v>6515</v>
-      </c>
-      <c r="C15" s="299" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D15" s="299" t="inlineStr">
-        <is>
-          <t>H.H 100GM</t>
-        </is>
-      </c>
-      <c r="E15" s="298" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F15" s="300" t="n">
-        <v>38896</v>
-      </c>
-      <c r="G15" s="298" t="inlineStr">
+      <c r="B15" s="304" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C15" s="305" t="inlineStr">
+        <is>
+          <t>Adore</t>
+        </is>
+      </c>
+      <c r="D15" s="305" t="inlineStr">
+        <is>
+          <t>V- HC BROWN</t>
+        </is>
+      </c>
+      <c r="E15" s="304" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F15" s="306" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G15" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
       </c>
       <c r="H15" s="276" t="inlineStr">
         <is>
-          <t>To be dispatch after packing</t>
+          <t>Cap Not Available</t>
         </is>
       </c>
       <c r="I15" s="95">
@@ -51221,38 +51444,38 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="237">
-      <c r="A16" s="298" t="n">
+      <c r="A16" s="304" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="298" t="n">
-        <v>6530</v>
-      </c>
-      <c r="C16" s="299" t="inlineStr">
-        <is>
-          <t>Adore</t>
-        </is>
-      </c>
-      <c r="D16" s="299" t="inlineStr">
-        <is>
-          <t>V- HC BROWN</t>
-        </is>
-      </c>
-      <c r="E16" s="298" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F16" s="300" t="n">
-        <v>15000</v>
-      </c>
-      <c r="G16" s="298" t="inlineStr">
+      <c r="B16" s="304" t="n">
+        <v>5782</v>
+      </c>
+      <c r="C16" s="305" t="inlineStr">
+        <is>
+          <t>Mega Grey</t>
+        </is>
+      </c>
+      <c r="D16" s="305" t="inlineStr">
+        <is>
+          <t>M.G</t>
+        </is>
+      </c>
+      <c r="E16" s="304" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F16" s="306" t="n">
+        <v>10500</v>
+      </c>
+      <c r="G16" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
       </c>
       <c r="H16" s="276" t="inlineStr">
         <is>
-          <t>To be dispatch after packing</t>
+          <t>Cap Not Available</t>
         </is>
       </c>
       <c r="I16" s="95">
@@ -51261,31 +51484,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="237">
-      <c r="A17" s="298" t="n">
+      <c r="A17" s="304" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="298" t="n">
-        <v>5782</v>
-      </c>
-      <c r="C17" s="299" t="inlineStr">
-        <is>
-          <t>Mega Grey</t>
-        </is>
-      </c>
-      <c r="D17" s="299" t="inlineStr">
-        <is>
-          <t>M.G</t>
-        </is>
-      </c>
-      <c r="E17" s="298" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F17" s="300" t="n">
-        <v>10500</v>
-      </c>
-      <c r="G17" s="298" t="inlineStr">
+      <c r="B17" s="304" t="n">
+        <v>6624</v>
+      </c>
+      <c r="C17" s="305" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D17" s="305" t="inlineStr">
+        <is>
+          <t>S-45 DIA 19MM</t>
+        </is>
+      </c>
+      <c r="E17" s="304" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F17" s="306" t="n">
+        <v>15288</v>
+      </c>
+      <c r="G17" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51301,31 +51524,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="237">
-      <c r="A18" s="298" t="n">
+      <c r="A18" s="304" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="298" t="n">
-        <v>6624</v>
-      </c>
-      <c r="C18" s="299" t="inlineStr">
+      <c r="B18" s="304" t="n">
+        <v>5731</v>
+      </c>
+      <c r="C18" s="305" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="299" t="inlineStr">
-        <is>
-          <t>S-45 DIA 19MM</t>
-        </is>
-      </c>
-      <c r="E18" s="298" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="F18" s="300" t="n">
-        <v>15288</v>
-      </c>
-      <c r="G18" s="298" t="inlineStr">
+      <c r="D18" s="305" t="inlineStr">
+        <is>
+          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
+        </is>
+      </c>
+      <c r="E18" s="304" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="F18" s="306" t="n">
+        <v>37030</v>
+      </c>
+      <c r="G18" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51341,40 +51564,14 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="237">
-      <c r="A19" s="298" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="298" t="n">
-        <v>5731</v>
-      </c>
-      <c r="C19" s="299" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D19" s="299" t="inlineStr">
-        <is>
-          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
-        </is>
-      </c>
-      <c r="E19" s="298" t="inlineStr">
-        <is>
-          <t>20.5</t>
-        </is>
-      </c>
-      <c r="F19" s="300" t="n">
-        <v>37030</v>
-      </c>
-      <c r="G19" s="298" t="inlineStr">
-        <is>
-          <t>Not Ready</t>
-        </is>
-      </c>
-      <c r="H19" s="276" t="inlineStr">
-        <is>
-          <t>Cap Not Available</t>
-        </is>
-      </c>
+      <c r="A19" s="277" t="n"/>
+      <c r="B19" s="277" t="n"/>
+      <c r="C19" s="278" t="n"/>
+      <c r="D19" s="278" t="n"/>
+      <c r="E19" s="277" t="n"/>
+      <c r="F19" s="279" t="n"/>
+      <c r="G19" s="277" t="n"/>
+      <c r="H19" s="280" t="n"/>
       <c r="I19" s="95">
         <f>IFERROR(SUMPRODUCT((TableBOM[Product ID]=B19)*(TableBOM[Material Category]="CAP")*TableBOM[Item ID]),0)</f>
         <v/>

</xml_diff>

<commit_message>
Full backup 15/06/2026 10:23:51
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -801,7 +801,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="20"/>
   </cellStyleXfs>
-  <cellXfs count="307">
+  <cellXfs count="313">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1601,6 +1601,24 @@
     <xf numFmtId="3" fontId="47" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2818,7 +2836,9 @@
         <f>IF(G14=0,"-",H14/G14)</f>
         <v/>
       </c>
-      <c r="K14" s="287" t="n"/>
+      <c r="K14" s="287" t="n">
+        <v>31248</v>
+      </c>
       <c r="L14" s="289" t="n"/>
       <c r="M14" s="155" t="inlineStr">
         <is>
@@ -38700,7 +38720,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="37" t="n">
-        <v>1050</v>
+        <v>1150</v>
       </c>
       <c r="H7" s="38">
         <f>E7+F7-G7</f>
@@ -38968,7 +38988,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="37" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H15" s="38">
         <f>E15+F15-G15</f>
@@ -39240,7 +39260,7 @@
         <v>210</v>
       </c>
       <c r="G22" s="37" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="H22" s="38">
         <f>E22+F22-G22</f>
@@ -41082,7 +41102,7 @@
         <v>0</v>
       </c>
       <c r="G65" s="37" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="H65" s="38">
         <f>E65+F65-G65</f>
@@ -50964,31 +50984,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="237">
-      <c r="A4" s="301" t="n">
+      <c r="A4" s="307" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="301" t="n">
+      <c r="B4" s="307" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="302" t="inlineStr">
+      <c r="C4" s="308" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="302" t="inlineStr">
+      <c r="D4" s="308" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="301" t="inlineStr">
+      <c r="E4" s="307" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="303" t="n">
+      <c r="F4" s="309" t="n">
         <v>18860</v>
       </c>
-      <c r="G4" s="301" t="inlineStr">
+      <c r="G4" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51004,31 +51024,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="237">
-      <c r="A5" s="301" t="n">
+      <c r="A5" s="307" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="301" t="n">
+      <c r="B5" s="307" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="302" t="inlineStr">
+      <c r="C5" s="308" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="302" t="inlineStr">
+      <c r="D5" s="308" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="301" t="inlineStr">
+      <c r="E5" s="307" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="303" t="n">
+      <c r="F5" s="309" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="301" t="inlineStr">
+      <c r="G5" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51044,31 +51064,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="237">
-      <c r="A6" s="301" t="n">
+      <c r="A6" s="307" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="301" t="n">
+      <c r="B6" s="307" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="302" t="inlineStr">
+      <c r="C6" s="308" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="302" t="inlineStr">
+      <c r="D6" s="308" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="301" t="inlineStr">
+      <c r="E6" s="307" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="303" t="n">
+      <c r="F6" s="309" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="301" t="inlineStr">
+      <c r="G6" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51084,31 +51104,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="237">
-      <c r="A7" s="301" t="n">
+      <c r="A7" s="307" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="301" t="n">
+      <c r="B7" s="307" t="n">
         <v>5389</v>
       </c>
-      <c r="C7" s="302" t="inlineStr">
+      <c r="C7" s="308" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D7" s="302" t="inlineStr">
+      <c r="D7" s="308" t="inlineStr">
         <is>
           <t>S-45</t>
         </is>
       </c>
-      <c r="E7" s="301" t="inlineStr">
+      <c r="E7" s="307" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F7" s="303" t="n">
+      <c r="F7" s="309" t="n">
         <v>11088</v>
       </c>
-      <c r="G7" s="301" t="inlineStr">
+      <c r="G7" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51124,31 +51144,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="237">
-      <c r="A8" s="301" t="n">
+      <c r="A8" s="307" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="301" t="n">
+      <c r="B8" s="307" t="n">
         <v>4050</v>
       </c>
-      <c r="C8" s="302" t="inlineStr">
+      <c r="C8" s="308" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D8" s="302" t="inlineStr">
+      <c r="D8" s="308" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E8" s="301" t="inlineStr">
+      <c r="E8" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="303" t="n">
+      <c r="F8" s="309" t="n">
         <v>9450</v>
       </c>
-      <c r="G8" s="301" t="inlineStr">
+      <c r="G8" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51164,31 +51184,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="237">
-      <c r="A9" s="301" t="n">
+      <c r="A9" s="307" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="301" t="n">
+      <c r="B9" s="307" t="n">
         <v>6337</v>
       </c>
-      <c r="C9" s="302" t="inlineStr">
+      <c r="C9" s="308" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="302" t="inlineStr">
+      <c r="D9" s="308" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="301" t="inlineStr">
+      <c r="E9" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="303" t="n">
+      <c r="F9" s="309" t="n">
         <v>15680</v>
       </c>
-      <c r="G9" s="301" t="inlineStr">
+      <c r="G9" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51204,31 +51224,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="237">
-      <c r="A10" s="301" t="n">
+      <c r="A10" s="307" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="301" t="n">
+      <c r="B10" s="307" t="n">
         <v>6416</v>
       </c>
-      <c r="C10" s="302" t="inlineStr">
+      <c r="C10" s="308" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D10" s="302" t="inlineStr">
+      <c r="D10" s="308" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E10" s="301" t="inlineStr">
+      <c r="E10" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F10" s="303" t="n">
+      <c r="F10" s="309" t="n">
         <v>15435</v>
       </c>
-      <c r="G10" s="301" t="inlineStr">
+      <c r="G10" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51244,31 +51264,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="237">
-      <c r="A11" s="301" t="n">
+      <c r="A11" s="307" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="301" t="n">
+      <c r="B11" s="307" t="n">
         <v>5782</v>
       </c>
-      <c r="C11" s="302" t="inlineStr">
+      <c r="C11" s="308" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D11" s="302" t="inlineStr">
+      <c r="D11" s="308" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E11" s="301" t="inlineStr">
+      <c r="E11" s="307" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F11" s="303" t="n">
+      <c r="F11" s="309" t="n">
         <v>63648</v>
       </c>
-      <c r="G11" s="301" t="inlineStr">
+      <c r="G11" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51284,31 +51304,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="237">
-      <c r="A12" s="301" t="n">
+      <c r="A12" s="307" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="301" t="n">
+      <c r="B12" s="307" t="n">
         <v>6531</v>
       </c>
-      <c r="C12" s="302" t="inlineStr">
+      <c r="C12" s="308" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D12" s="302" t="inlineStr">
+      <c r="D12" s="308" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E12" s="301" t="inlineStr">
+      <c r="E12" s="307" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F12" s="303" t="n">
+      <c r="F12" s="309" t="n">
         <v>4380</v>
       </c>
-      <c r="G12" s="301" t="inlineStr">
+      <c r="G12" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51324,31 +51344,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="237">
-      <c r="A13" s="301" t="n">
+      <c r="A13" s="307" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="301" t="n">
+      <c r="B13" s="307" t="n">
         <v>6206</v>
       </c>
-      <c r="C13" s="302" t="inlineStr">
+      <c r="C13" s="308" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D13" s="302" t="inlineStr">
+      <c r="D13" s="308" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E13" s="301" t="inlineStr">
+      <c r="E13" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F13" s="303" t="n">
+      <c r="F13" s="309" t="n">
         <v>100674</v>
       </c>
-      <c r="G13" s="301" t="inlineStr">
+      <c r="G13" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51364,31 +51384,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="237">
-      <c r="A14" s="304" t="n">
+      <c r="A14" s="310" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="304" t="n">
+      <c r="B14" s="310" t="n">
         <v>6515</v>
       </c>
-      <c r="C14" s="305" t="inlineStr">
+      <c r="C14" s="311" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D14" s="305" t="inlineStr">
+      <c r="D14" s="311" t="inlineStr">
         <is>
           <t>H.H 100GM</t>
         </is>
       </c>
-      <c r="E14" s="304" t="inlineStr">
+      <c r="E14" s="310" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F14" s="306" t="n">
+      <c r="F14" s="312" t="n">
         <v>38896</v>
       </c>
-      <c r="G14" s="304" t="inlineStr">
+      <c r="G14" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51404,31 +51424,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="237">
-      <c r="A15" s="304" t="n">
+      <c r="A15" s="310" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="304" t="n">
+      <c r="B15" s="310" t="n">
         <v>6530</v>
       </c>
-      <c r="C15" s="305" t="inlineStr">
+      <c r="C15" s="311" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D15" s="305" t="inlineStr">
+      <c r="D15" s="311" t="inlineStr">
         <is>
           <t>V- HC BROWN</t>
         </is>
       </c>
-      <c r="E15" s="304" t="inlineStr">
+      <c r="E15" s="310" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F15" s="306" t="n">
+      <c r="F15" s="312" t="n">
         <v>15000</v>
       </c>
-      <c r="G15" s="304" t="inlineStr">
+      <c r="G15" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51444,31 +51464,31 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="237">
-      <c r="A16" s="304" t="n">
+      <c r="A16" s="310" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="304" t="n">
+      <c r="B16" s="310" t="n">
         <v>5782</v>
       </c>
-      <c r="C16" s="305" t="inlineStr">
+      <c r="C16" s="311" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D16" s="305" t="inlineStr">
+      <c r="D16" s="311" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E16" s="304" t="inlineStr">
+      <c r="E16" s="310" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F16" s="306" t="n">
+      <c r="F16" s="312" t="n">
         <v>10500</v>
       </c>
-      <c r="G16" s="304" t="inlineStr">
+      <c r="G16" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51484,31 +51504,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="237">
-      <c r="A17" s="304" t="n">
+      <c r="A17" s="310" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="304" t="n">
+      <c r="B17" s="310" t="n">
         <v>6624</v>
       </c>
-      <c r="C17" s="305" t="inlineStr">
+      <c r="C17" s="311" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D17" s="305" t="inlineStr">
+      <c r="D17" s="311" t="inlineStr">
         <is>
           <t>S-45 DIA 19MM</t>
         </is>
       </c>
-      <c r="E17" s="304" t="inlineStr">
+      <c r="E17" s="310" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F17" s="306" t="n">
+      <c r="F17" s="312" t="n">
         <v>15288</v>
       </c>
-      <c r="G17" s="304" t="inlineStr">
+      <c r="G17" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51524,31 +51544,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="237">
-      <c r="A18" s="304" t="n">
+      <c r="A18" s="310" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="304" t="n">
+      <c r="B18" s="310" t="n">
         <v>5731</v>
       </c>
-      <c r="C18" s="305" t="inlineStr">
+      <c r="C18" s="311" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="305" t="inlineStr">
+      <c r="D18" s="311" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E18" s="304" t="inlineStr">
+      <c r="E18" s="310" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F18" s="306" t="n">
+      <c r="F18" s="312" t="n">
         <v>37030</v>
       </c>
-      <c r="G18" s="304" t="inlineStr">
+      <c r="G18" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>

</xml_diff>

<commit_message>
Full backup 16/06/2026 11:36:52
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Guide" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MRP'!$A$13:$K$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Production_Log'!$A$2:$R$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'BOM Issues'!$A$52:$J$64</definedName>
   </definedNames>
@@ -482,7 +483,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -684,6 +685,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
@@ -785,20 +801,20 @@
     </border>
   </borders>
   <cellStyleXfs count="10">
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
-    <xf numFmtId="173" fontId="24" fillId="0" borderId="20"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
+    <xf numFmtId="173" fontId="24" fillId="0" borderId="21"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="20"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
+    <xf numFmtId="43" fontId="24" fillId="0" borderId="21"/>
   </cellStyleXfs>
   <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1298,136 +1314,136 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="10" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="24" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="24" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="47" fillId="10" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="47" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="46" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="48" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="48" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="48" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="48" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="48" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="48" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="49" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="49" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="48" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="48" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="41" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="41" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="36" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="36" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="38" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="38" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="36" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="36" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1439,149 +1455,149 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="38" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="38" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="36" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="36" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="36" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="36" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="172" fontId="24" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="24" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="24" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="172" fontId="24" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="24" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="24" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="24" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="47" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="10" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="47" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="11" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="46" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="48" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="48" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="48" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="48" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="48" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="48" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="49" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="49" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="48" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="48" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="41" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="41" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="41" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="41" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2051,23 +2067,23 @@
   <dimension ref="A1:AC199"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="16.5"/>
   <cols>
-    <col width="1.5703125" customWidth="1" style="231" min="1" max="1"/>
-    <col width="7" customWidth="1" style="231" min="2" max="2"/>
-    <col width="32.7109375" customWidth="1" style="231" min="3" max="3"/>
-    <col width="38.7109375" customWidth="1" style="231" min="4" max="4"/>
-    <col width="8.85546875" customWidth="1" style="232" min="5" max="5"/>
-    <col width="9.140625" customWidth="1" style="231" min="6" max="6"/>
-    <col width="11" customWidth="1" style="233" min="7" max="7"/>
-    <col width="11.140625" customWidth="1" style="231" min="8" max="8"/>
-    <col width="10.28515625" customWidth="1" style="231" min="9" max="9"/>
-    <col width="10.5703125" customWidth="1" style="231" min="10" max="10"/>
-    <col width="9.28515625" customWidth="1" style="231" min="11" max="11"/>
-    <col width="33.85546875" customWidth="1" style="231" min="12" max="12"/>
-    <col width="14.7109375" customWidth="1" style="231" min="13" max="13"/>
-    <col width="13.28515625" customWidth="1" style="231" min="14" max="14"/>
-    <col width="9.5703125" customWidth="1" style="231" min="15" max="15"/>
-    <col width="8.7109375" customWidth="1" style="231" min="16" max="56"/>
-    <col width="8.7109375" customWidth="1" style="231" min="57" max="16384"/>
+    <col width="1.5703125" customWidth="1" style="228" min="1" max="1"/>
+    <col width="7" customWidth="1" style="228" min="2" max="2"/>
+    <col width="32.7109375" customWidth="1" style="228" min="3" max="3"/>
+    <col width="38.7109375" customWidth="1" style="228" min="4" max="4"/>
+    <col width="8.85546875" customWidth="1" style="229" min="5" max="5"/>
+    <col width="9.140625" customWidth="1" style="228" min="6" max="6"/>
+    <col width="11" customWidth="1" style="230" min="7" max="7"/>
+    <col width="11.140625" customWidth="1" style="228" min="8" max="8"/>
+    <col width="10.28515625" customWidth="1" style="228" min="9" max="9"/>
+    <col width="10.5703125" customWidth="1" style="228" min="10" max="10"/>
+    <col width="9.28515625" customWidth="1" style="228" min="11" max="11"/>
+    <col width="35.140625" customWidth="1" style="228" min="12" max="12"/>
+    <col width="14.7109375" customWidth="1" style="228" min="13" max="13"/>
+    <col width="13.28515625" customWidth="1" style="228" min="14" max="14"/>
+    <col width="9.5703125" customWidth="1" style="228" min="15" max="15"/>
+    <col width="8.7109375" customWidth="1" style="228" min="16" max="57"/>
+    <col width="8.7109375" customWidth="1" style="228" min="58" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="6" customHeight="1" s="243">
@@ -2383,21 +2399,21 @@
     </row>
     <row r="9" ht="20.25" customHeight="1" s="243">
       <c r="A9" s="136" t="n"/>
-      <c r="B9" s="240" t="inlineStr">
+      <c r="B9" s="237" t="inlineStr">
         <is>
           <t>Summary of Production &amp; Dispatch - MTD</t>
         </is>
       </c>
-      <c r="C9" s="241" t="n"/>
-      <c r="D9" s="241" t="n"/>
-      <c r="E9" s="241" t="n"/>
-      <c r="F9" s="241" t="n"/>
-      <c r="G9" s="241" t="n"/>
-      <c r="H9" s="241" t="n"/>
-      <c r="I9" s="241" t="n"/>
-      <c r="J9" s="241" t="n"/>
-      <c r="K9" s="241" t="n"/>
-      <c r="L9" s="241" t="n"/>
+      <c r="C9" s="238" t="n"/>
+      <c r="D9" s="238" t="n"/>
+      <c r="E9" s="238" t="n"/>
+      <c r="F9" s="238" t="n"/>
+      <c r="G9" s="238" t="n"/>
+      <c r="H9" s="238" t="n"/>
+      <c r="I9" s="238" t="n"/>
+      <c r="J9" s="238" t="n"/>
+      <c r="K9" s="238" t="n"/>
+      <c r="L9" s="238" t="n"/>
       <c r="M9" s="157">
         <f>IFERROR(INDEX($S$9:$S$23,MATCH(LARGE($U$9:$U$23,3),$U$9:$U$23,0)),"")</f>
         <v/>
@@ -3020,7 +3036,7 @@
       <c r="K17" s="293" t="n"/>
       <c r="L17" s="295" t="inlineStr">
         <is>
-          <t>2.6k Advance Production</t>
+          <t>400k Order, 100k Advance Production</t>
         </is>
       </c>
       <c r="P17" s="136" t="n"/>
@@ -4132,7 +4148,7 @@
       <c r="P36" s="136" t="n"/>
       <c r="Q36" s="136" t="n"/>
       <c r="R36" s="136" t="n"/>
-      <c r="S36" s="231" t="inlineStr">
+      <c r="S36" s="228" t="inlineStr">
         <is>
           <t>Gas Shutdown</t>
         </is>
@@ -4141,7 +4157,7 @@
         <f>SUMPRODUCT((MONTH(Production_Log!$A$3:$A$8963)=MONTH(TODAY()))*(YEAR(Production_Log!$A$3:$A$8963)=YEAR(TODAY()))*Production_Log!$Q$3:$Q$8963)</f>
         <v/>
       </c>
-      <c r="U36" s="231">
+      <c r="U36" s="228">
         <f>T36+0.00006</f>
         <v/>
       </c>
@@ -5939,7 +5955,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -5978,8 +5994,9 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="H1" s="163" t="n">
-        <v>46171</v>
+      <c r="H1" s="163">
+        <f>TODAY()</f>
+        <v/>
       </c>
       <c r="I1" s="10" t="n"/>
       <c r="J1" s="11" t="n"/>
@@ -6198,7 +6215,7 @@
         <v>6894</v>
       </c>
       <c r="F6" s="185" t="n">
-        <v>30000</v>
+        <v>32592</v>
       </c>
       <c r="G6" s="19">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$58,MATCH(MRP!D6,Tubex_Dashboard!$F$11:$F$58,0))</f>
@@ -6231,7 +6248,7 @@
         <v>6893</v>
       </c>
       <c r="F7" s="185" t="n">
-        <v>62000</v>
+        <v>62496</v>
       </c>
       <c r="G7" s="19">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$58,MATCH(MRP!D7,Tubex_Dashboard!$F$11:$F$58,0))</f>
@@ -6264,7 +6281,7 @@
         <v>6887</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>22000</v>
+        <v>52000</v>
       </c>
       <c r="G8" s="19">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$58,MATCH(MRP!D8,Tubex_Dashboard!$F$11:$F$58,0))</f>
@@ -6309,8 +6326,9 @@
           <t>Awaited</t>
         </is>
       </c>
-      <c r="F9" s="193" t="n">
-        <v>300000</v>
+      <c r="F9" s="193">
+        <f>400000-98056</f>
+        <v/>
       </c>
       <c r="G9" s="194">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$100,MATCH(MRP!D9,Tubex_Dashboard!$F$11:$F$100,0))</f>
@@ -6322,7 +6340,7 @@
       </c>
       <c r="I9" s="195" t="inlineStr">
         <is>
-          <t>2.6k Already in FG Stock</t>
+          <t>400k Order, 100k already in FG Stock</t>
         </is>
       </c>
     </row>
@@ -6503,7 +6521,7 @@
       <c r="T13" s="11" t="n"/>
       <c r="U13" s="2" t="n"/>
     </row>
-    <row r="14" ht="24" customHeight="1" s="243">
+    <row r="14" hidden="1" ht="24" customHeight="1" s="243">
       <c r="A14" s="21" t="n">
         <v>33</v>
       </c>
@@ -6561,7 +6579,7 @@
       <c r="T14" s="11" t="n"/>
       <c r="U14" s="2" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" hidden="1" s="243">
       <c r="A15" s="21" t="n">
         <v>31</v>
       </c>
@@ -6677,7 +6695,7 @@
       <c r="T16" s="11" t="n"/>
       <c r="U16" s="2" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" hidden="1" s="243">
       <c r="A17" s="21" t="n">
         <v>25</v>
       </c>
@@ -6735,7 +6753,7 @@
       <c r="T17" s="11" t="n"/>
       <c r="U17" s="2" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" hidden="1" s="243">
       <c r="A18" s="21" t="n">
         <v>22</v>
       </c>
@@ -6783,7 +6801,7 @@
         <v/>
       </c>
     </row>
-    <row r="19">
+    <row r="19" hidden="1" s="243">
       <c r="A19" s="21" t="n">
         <v>19</v>
       </c>
@@ -6831,7 +6849,7 @@
         <v/>
       </c>
     </row>
-    <row r="20">
+    <row r="20" hidden="1" s="243">
       <c r="A20" s="21" t="n">
         <v>4179</v>
       </c>
@@ -6927,7 +6945,7 @@
         <v/>
       </c>
     </row>
-    <row r="22">
+    <row r="22" hidden="1" s="243">
       <c r="A22" s="21" t="n">
         <v>10</v>
       </c>
@@ -6975,7 +6993,7 @@
         <v/>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="1" s="243">
       <c r="A23" s="21" t="n">
         <v>2</v>
       </c>
@@ -7081,7 +7099,7 @@
       <c r="T24" s="11" t="n"/>
       <c r="U24" s="2" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" hidden="1" s="243">
       <c r="A25" s="21" t="n">
         <v>6961</v>
       </c>
@@ -7139,7 +7157,7 @@
       <c r="T25" s="11" t="n"/>
       <c r="U25" s="2" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" hidden="1" s="243">
       <c r="A26" s="21" t="n">
         <v>3935</v>
       </c>
@@ -7232,9 +7250,10 @@
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A27)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A27)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A27)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A27)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A27)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A27)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A27)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A27)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A27)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A27)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A27)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A27)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A27)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A27)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A27)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A27)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A27)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A27)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A27)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A27)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A27)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A27)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A27)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A27)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))-2),"")</f>
         <v/>
       </c>
-      <c r="I27" s="30">
-        <f>IF(E27=0,"Not needed",IF(G27&lt;0,"SHORTAGE",IF(G27&lt;F27*0.1,"LOW","OK")))</f>
-        <v/>
+      <c r="I27" s="30" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
       </c>
       <c r="J27" s="30">
         <f>IF(B27&lt;&gt;"CAP","",SUMPRODUCT((ISNUMBER(SEARCH("Cap Not Available",'FG Stock'!$H$4:$H$100)))*('FG Stock'!$I$4:$I$100=A27)*'FG Stock'!$F$4:$F$100))</f>
@@ -7245,7 +7264,7 @@
         <v/>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="1" s="243">
       <c r="A28" s="21" t="n">
         <v>184</v>
       </c>
@@ -7361,7 +7380,7 @@
       <c r="T29" s="11" t="n"/>
       <c r="U29" s="2" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" hidden="1" s="243">
       <c r="A30" s="21" t="n">
         <v>188</v>
       </c>
@@ -7419,7 +7438,7 @@
       <c r="T30" s="11" t="n"/>
       <c r="U30" s="2" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" hidden="1" s="243">
       <c r="A31" s="21" t="n">
         <v>1065</v>
       </c>
@@ -7535,7 +7554,7 @@
       <c r="T32" s="11" t="n"/>
       <c r="U32" s="2" t="n"/>
     </row>
-    <row r="33">
+    <row r="33" hidden="1" s="243">
       <c r="A33" s="21" t="n">
         <v>170</v>
       </c>
@@ -7593,7 +7612,7 @@
       <c r="T33" s="11" t="n"/>
       <c r="U33" s="2" t="n"/>
     </row>
-    <row r="34">
+    <row r="34" hidden="1" s="243">
       <c r="A34" s="21" t="n">
         <v>175</v>
       </c>
@@ -7651,7 +7670,7 @@
       <c r="T34" s="11" t="n"/>
       <c r="U34" s="2" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" hidden="1" s="243">
       <c r="A35" s="21" t="n">
         <v>192</v>
       </c>
@@ -7767,7 +7786,7 @@
       <c r="T36" s="11" t="n"/>
       <c r="U36" s="2" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" hidden="1" s="243">
       <c r="A37" s="21" t="n">
         <v>3869</v>
       </c>
@@ -7825,7 +7844,7 @@
       <c r="T37" s="11" t="n"/>
       <c r="U37" s="2" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" hidden="1" s="243">
       <c r="A38" s="21" t="n">
         <v>4156</v>
       </c>
@@ -7873,7 +7892,7 @@
         <v/>
       </c>
     </row>
-    <row r="39">
+    <row r="39" hidden="1" s="243">
       <c r="A39" s="21" t="n">
         <v>4157</v>
       </c>
@@ -7921,7 +7940,7 @@
         <v/>
       </c>
     </row>
-    <row r="40">
+    <row r="40" hidden="1" s="243">
       <c r="A40" s="21" t="n">
         <v>5895</v>
       </c>
@@ -7979,7 +7998,7 @@
       <c r="T40" s="11" t="n"/>
       <c r="U40" s="2" t="n"/>
     </row>
-    <row r="41">
+    <row r="41" hidden="1" s="243">
       <c r="A41" s="21" t="n">
         <v>5974</v>
       </c>
@@ -8027,7 +8046,7 @@
         <v/>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="1" s="243">
       <c r="A42" s="21" t="n">
         <v>177</v>
       </c>
@@ -8075,7 +8094,7 @@
         <v/>
       </c>
     </row>
-    <row r="43">
+    <row r="43" hidden="1" s="243">
       <c r="A43" s="21" t="n">
         <v>6132</v>
       </c>
@@ -8219,7 +8238,7 @@
         <v/>
       </c>
     </row>
-    <row r="46">
+    <row r="46" hidden="1" s="243">
       <c r="A46" s="21" t="n">
         <v>4165</v>
       </c>
@@ -8312,9 +8331,10 @@
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A47)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A47)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A47)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A47)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A47)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A47)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A47)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A47)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A47)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A47)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A47)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A47)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A47)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A47)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A47)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A47)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A47)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A47)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A47)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A47)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A47)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A47)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A47)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A47)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))-2),"")</f>
         <v/>
       </c>
-      <c r="I47" s="30">
-        <f>IF(E47=0,"Not needed",IF(G47&lt;0,"SHORTAGE",IF(G47&lt;F47*0.1,"LOW","OK")))</f>
-        <v/>
+      <c r="I47" s="30" t="inlineStr">
+        <is>
+          <t>Hold. Caps not approved</t>
+        </is>
       </c>
       <c r="J47" s="30">
         <f>IF(B47&lt;&gt;"CAP","",SUMPRODUCT((ISNUMBER(SEARCH("Cap Not Available",'FG Stock'!$H$4:$H$100)))*('FG Stock'!$I$4:$I$100=A47)*'FG Stock'!$F$4:$F$100))</f>
@@ -8325,7 +8345,7 @@
         <v/>
       </c>
     </row>
-    <row r="48">
+    <row r="48" hidden="1" s="243">
       <c r="A48" s="21" t="n">
         <v>99</v>
       </c>
@@ -8383,7 +8403,7 @@
       <c r="T48" s="11" t="n"/>
       <c r="U48" s="2" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" hidden="1" s="243">
       <c r="A49" s="21" t="n">
         <v>72</v>
       </c>
@@ -8441,7 +8461,7 @@
       <c r="T49" s="11" t="n"/>
       <c r="U49" s="2" t="n"/>
     </row>
-    <row r="50">
+    <row r="50" hidden="1" s="243">
       <c r="A50" s="21" t="n">
         <v>79</v>
       </c>
@@ -8499,7 +8519,7 @@
       <c r="T50" s="11" t="n"/>
       <c r="U50" s="2" t="n"/>
     </row>
-    <row r="51">
+    <row r="51" hidden="1" s="243">
       <c r="A51" s="21" t="n">
         <v>80</v>
       </c>
@@ -8547,7 +8567,7 @@
         <v/>
       </c>
     </row>
-    <row r="52">
+    <row r="52" hidden="1" s="243">
       <c r="A52" s="21" t="n">
         <v>81</v>
       </c>
@@ -8595,7 +8615,7 @@
         <v/>
       </c>
     </row>
-    <row r="53">
+    <row r="53" hidden="1" s="243">
       <c r="A53" s="21" t="n">
         <v>1800</v>
       </c>
@@ -8643,7 +8663,7 @@
         <v/>
       </c>
     </row>
-    <row r="54">
+    <row r="54" hidden="1" s="243">
       <c r="A54" s="21" t="n">
         <v>3211</v>
       </c>
@@ -8691,7 +8711,7 @@
         <v/>
       </c>
     </row>
-    <row r="55">
+    <row r="55" hidden="1" s="243">
       <c r="A55" s="21" t="n">
         <v>4015</v>
       </c>
@@ -8739,7 +8759,7 @@
         <v/>
       </c>
     </row>
-    <row r="56">
+    <row r="56" hidden="1" s="243">
       <c r="A56" s="21" t="n">
         <v>4044</v>
       </c>
@@ -8787,7 +8807,7 @@
         <v/>
       </c>
     </row>
-    <row r="57">
+    <row r="57" hidden="1" s="243">
       <c r="A57" s="21" t="n">
         <v>4088</v>
       </c>
@@ -8835,7 +8855,7 @@
         <v/>
       </c>
     </row>
-    <row r="58">
+    <row r="58" hidden="1" s="243">
       <c r="A58" s="21" t="n">
         <v>4143</v>
       </c>
@@ -8883,7 +8903,7 @@
         <v/>
       </c>
     </row>
-    <row r="59">
+    <row r="59" hidden="1" s="243">
       <c r="A59" s="21" t="n">
         <v>6971</v>
       </c>
@@ -8931,7 +8951,7 @@
         <v/>
       </c>
     </row>
-    <row r="60">
+    <row r="60" hidden="1" s="243">
       <c r="A60" s="21" t="n">
         <v>7370</v>
       </c>
@@ -9027,7 +9047,7 @@
         <v/>
       </c>
     </row>
-    <row r="62">
+    <row r="62" hidden="1" s="243">
       <c r="A62" s="21" t="n">
         <v>102</v>
       </c>
@@ -9075,7 +9095,7 @@
         <v/>
       </c>
     </row>
-    <row r="63">
+    <row r="63" hidden="1" s="243">
       <c r="A63" s="21" t="n">
         <v>1073</v>
       </c>
@@ -9123,7 +9143,7 @@
         <v/>
       </c>
     </row>
-    <row r="64">
+    <row r="64" hidden="1" s="243">
       <c r="A64" s="21" t="n">
         <v>1285</v>
       </c>
@@ -9171,7 +9191,7 @@
         <v/>
       </c>
     </row>
-    <row r="65">
+    <row r="65" hidden="1" s="243">
       <c r="A65" s="21" t="n">
         <v>3522</v>
       </c>
@@ -9219,7 +9239,7 @@
         <v/>
       </c>
     </row>
-    <row r="66">
+    <row r="66" hidden="1" s="243">
       <c r="A66" s="21" t="n">
         <v>3866</v>
       </c>
@@ -9315,7 +9335,7 @@
         <v/>
       </c>
     </row>
-    <row r="68">
+    <row r="68" hidden="1" s="243">
       <c r="A68" s="21" t="n">
         <v>9902</v>
       </c>
@@ -9363,7 +9383,7 @@
         <v/>
       </c>
     </row>
-    <row r="69">
+    <row r="69" hidden="1" s="243">
       <c r="A69" s="21" t="n">
         <v>9903</v>
       </c>
@@ -9446,9 +9466,10 @@
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A70)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A70)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A70)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A70)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A70)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A70)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A70)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A70)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A70)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A70)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A70)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A70)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A70)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A70)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A70)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A70)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A70)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A70)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A70)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A70)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A70)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A70)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A70)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A70)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))-2),"")</f>
         <v/>
       </c>
-      <c r="I70" s="30">
-        <f>IF(E70=0,"Not needed",IF(G70&lt;0,"SHORTAGE",IF(G70&lt;F70*0.1,"LOW","OK")))</f>
-        <v/>
+      <c r="I70" s="30" t="inlineStr">
+        <is>
+          <t>Hold. Caps not approved</t>
+        </is>
       </c>
       <c r="J70">
         <f>IF(B70&lt;&gt;"CAP","",SUMPRODUCT((ISNUMBER(SEARCH("Cap Not Available",'FG Stock'!$H$4:$H$100)))*('FG Stock'!$I$4:$I$100=A70)*'FG Stock'!$F$4:$F$100))</f>
@@ -9494,9 +9515,10 @@
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A71)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A71)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A71)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A71)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A71)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A71)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A71)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A71)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A71)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A71)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A71)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A71)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A71)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A71)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A71)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A71)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A71)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A71)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A71)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A71)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A71)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A71)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A71)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A71)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))-2),"")</f>
         <v/>
       </c>
-      <c r="I71" s="30">
-        <f>IF(E71=0,"Not needed",IF(G71&lt;0,"SHORTAGE",IF(G71&lt;F71*0.1,"LOW","OK")))</f>
-        <v/>
+      <c r="I71" s="30" t="inlineStr">
+        <is>
+          <t>Hold. Caps not approved</t>
+        </is>
       </c>
       <c r="J71" s="30">
         <f>IF(B71&lt;&gt;"CAP","",SUMPRODUCT((ISNUMBER(SEARCH("Cap Not Available",'FG Stock'!$H$4:$H$100)))*('FG Stock'!$I$4:$I$100=A71)*'FG Stock'!$F$4:$F$100))</f>
@@ -9507,7 +9529,7 @@
         <v/>
       </c>
     </row>
-    <row r="72">
+    <row r="72" hidden="1" s="243">
       <c r="A72" s="21" t="n">
         <v>39</v>
       </c>
@@ -9555,7 +9577,7 @@
         <v/>
       </c>
     </row>
-    <row r="73">
+    <row r="73" hidden="1" s="243">
       <c r="A73" s="21" t="n">
         <v>3619</v>
       </c>
@@ -9651,7 +9673,7 @@
         <v/>
       </c>
     </row>
-    <row r="75">
+    <row r="75" hidden="1" s="243">
       <c r="A75" s="21" t="n">
         <v>45</v>
       </c>
@@ -9747,7 +9769,7 @@
         <v/>
       </c>
     </row>
-    <row r="77">
+    <row r="77" hidden="1" s="243">
       <c r="A77" s="21" t="n">
         <v>5977</v>
       </c>
@@ -9891,7 +9913,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" s="243">
+    <row r="80" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A80" s="21" t="n">
         <v>191</v>
       </c>
@@ -9939,7 +9961,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" ht="15" customHeight="1" s="243">
+    <row r="81" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A81" s="21" t="n">
         <v>2680</v>
       </c>
@@ -9987,7 +10009,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" ht="15" customHeight="1" s="243">
+    <row r="82" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A82" s="21" t="n">
         <v>3492</v>
       </c>
@@ -10035,7 +10057,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" ht="15" customHeight="1" s="243">
+    <row r="83" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A83" s="21" t="n">
         <v>4002</v>
       </c>
@@ -10083,7 +10105,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" ht="15" customHeight="1" s="243">
+    <row r="84" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A84" s="21" t="n">
         <v>4070</v>
       </c>
@@ -10131,7 +10153,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" ht="15" customHeight="1" s="243">
+    <row r="85" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A85" s="21" t="n">
         <v>4310</v>
       </c>
@@ -10179,7 +10201,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" ht="15" customHeight="1" s="243">
+    <row r="86" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A86" s="21" t="n">
         <v>5625</v>
       </c>
@@ -10227,7 +10249,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" ht="15" customHeight="1" s="243">
+    <row r="87" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A87" s="21" t="n">
         <v>5816</v>
       </c>
@@ -10275,7 +10297,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" ht="15" customHeight="1" s="243">
+    <row r="88" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A88" s="21" t="n">
         <v>6135</v>
       </c>
@@ -10323,7 +10345,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" ht="15" customHeight="1" s="243">
+    <row r="89" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A89" s="21" t="n">
         <v>7133</v>
       </c>
@@ -10371,7 +10393,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" ht="15" customHeight="1" s="243">
+    <row r="90" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A90" s="21" t="n">
         <v>7412</v>
       </c>
@@ -10419,7 +10441,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" ht="15" customHeight="1" s="243">
+    <row r="91" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A91" s="21" t="n">
         <v>3752</v>
       </c>
@@ -10467,7 +10489,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" ht="15" customHeight="1" s="243">
+    <row r="92" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A92" s="21" t="n">
         <v>4248</v>
       </c>
@@ -10515,7 +10537,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" ht="16.5" customHeight="1" s="243">
+    <row r="93" hidden="1" ht="16.5" customHeight="1" s="243">
       <c r="A93" s="21" t="n">
         <v>6042</v>
       </c>
@@ -10563,7 +10585,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" ht="15" customHeight="1" s="243">
+    <row r="94" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A94" s="21" t="n">
         <v>2267</v>
       </c>
@@ -10611,7 +10633,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" ht="15" customHeight="1" s="243">
+    <row r="95" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A95" s="21" t="n">
         <v>3043</v>
       </c>
@@ -10687,14 +10709,14 @@
           <t>June 2026 PET Required Pet Orders</t>
         </is>
       </c>
-      <c r="B98" s="228" t="n"/>
-      <c r="C98" s="228" t="n"/>
-      <c r="D98" s="228" t="n"/>
-      <c r="E98" s="228" t="n"/>
-      <c r="F98" s="228" t="n"/>
+      <c r="B98" s="240" t="n"/>
+      <c r="C98" s="240" t="n"/>
+      <c r="D98" s="240" t="n"/>
+      <c r="E98" s="240" t="n"/>
+      <c r="F98" s="240" t="n"/>
       <c r="G98" s="188" t="n"/>
-      <c r="H98" s="228" t="n"/>
-      <c r="I98" s="229" t="n"/>
+      <c r="H98" s="240" t="n"/>
+      <c r="I98" s="241" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="243">
       <c r="A99" s="12" t="inlineStr">
@@ -10949,14 +10971,14 @@
           <t>JUNE PET MATERIAL REQUIREMENT PLAN</t>
         </is>
       </c>
-      <c r="B106" s="228" t="n"/>
-      <c r="C106" s="228" t="n"/>
-      <c r="D106" s="228" t="n"/>
-      <c r="E106" s="228" t="n"/>
-      <c r="F106" s="228" t="n"/>
+      <c r="B106" s="240" t="n"/>
+      <c r="C106" s="240" t="n"/>
+      <c r="D106" s="240" t="n"/>
+      <c r="E106" s="240" t="n"/>
+      <c r="F106" s="240" t="n"/>
       <c r="G106" s="188" t="n"/>
-      <c r="H106" s="228" t="n"/>
-      <c r="I106" s="228" t="n"/>
+      <c r="H106" s="240" t="n"/>
+      <c r="I106" s="240" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="243">
       <c r="A107" s="41" t="inlineStr">
@@ -11146,31 +11168,31 @@
       <c r="A111" s="262" t="n">
         <v>5977</v>
       </c>
-      <c r="B111" s="228" t="n"/>
-      <c r="C111" s="228" t="n"/>
-      <c r="D111" s="228" t="n"/>
-      <c r="E111" s="228" t="n"/>
-      <c r="F111" s="228" t="n"/>
-      <c r="G111" s="228" t="n"/>
-      <c r="H111" s="228" t="n"/>
-      <c r="I111" s="229" t="n"/>
+      <c r="B111" s="240" t="n"/>
+      <c r="C111" s="240" t="n"/>
+      <c r="D111" s="240" t="n"/>
+      <c r="E111" s="240" t="n"/>
+      <c r="F111" s="240" t="n"/>
+      <c r="G111" s="240" t="n"/>
+      <c r="H111" s="240" t="n"/>
+      <c r="I111" s="241" t="n"/>
       <c r="K111" s="47">
         <f>IF(E106=0,"",MAX(0,E106-F106))</f>
         <v/>
       </c>
     </row>
     <row r="112" ht="30" customHeight="1" s="243">
-      <c r="A112" s="227" t="n">
+      <c r="A112" s="196" t="n">
         <v>2267</v>
       </c>
-      <c r="B112" s="228" t="n"/>
-      <c r="C112" s="228" t="n"/>
-      <c r="D112" s="228" t="n"/>
-      <c r="E112" s="228" t="n"/>
-      <c r="F112" s="228" t="n"/>
-      <c r="G112" s="228" t="n"/>
-      <c r="H112" s="228" t="n"/>
-      <c r="I112" s="229" t="n"/>
+      <c r="B112" s="240" t="n"/>
+      <c r="C112" s="240" t="n"/>
+      <c r="D112" s="240" t="n"/>
+      <c r="E112" s="240" t="n"/>
+      <c r="F112" s="240" t="n"/>
+      <c r="G112" s="240" t="n"/>
+      <c r="H112" s="240" t="n"/>
+      <c r="I112" s="241" t="n"/>
       <c r="K112" s="48">
         <f>IF(E107=0,"",MAX(0,E107-F107))</f>
         <v/>
@@ -11310,14 +11332,14 @@
     </row>
     <row r="116" ht="15" customHeight="1" s="243">
       <c r="A116" s="187" t="n"/>
-      <c r="B116" s="228" t="n"/>
-      <c r="C116" s="228" t="n"/>
-      <c r="D116" s="228" t="n"/>
-      <c r="E116" s="228" t="n"/>
-      <c r="F116" s="228" t="n"/>
+      <c r="B116" s="240" t="n"/>
+      <c r="C116" s="240" t="n"/>
+      <c r="D116" s="240" t="n"/>
+      <c r="E116" s="240" t="n"/>
+      <c r="F116" s="240" t="n"/>
       <c r="G116" s="188" t="n"/>
-      <c r="H116" s="228" t="n"/>
-      <c r="I116" s="229" t="n"/>
+      <c r="H116" s="240" t="n"/>
+      <c r="I116" s="241" t="n"/>
     </row>
     <row r="117" ht="15" customHeight="1" s="243">
       <c r="A117" s="6" t="inlineStr">
@@ -13217,6 +13239,30 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A13:K95">
+    <filterColumn colId="4" hiddenButton="0" showButton="1">
+      <filters>
+        <filter val="1,516"/>
+        <filter val="111"/>
+        <filter val="138"/>
+        <filter val="15"/>
+        <filter val="188"/>
+        <filter val="2"/>
+        <filter val="20"/>
+        <filter val="222"/>
+        <filter val="25,500"/>
+        <filter val="263"/>
+        <filter val="3"/>
+        <filter val="3,092"/>
+        <filter val="305"/>
+        <filter val="347,688"/>
+        <filter val="66,606"/>
+        <filter val="69"/>
+        <filter val="89"/>
+        <filter val="99"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A111:I111"/>
   </mergeCells>
@@ -13253,15 +13299,15 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F125:G125 H2:I3 H8:I10 H123:H130 I6:I10 I11:I12 I14 I16:I19 I22 I24:I25 I27:I29 I31:I37 I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F125:G125 H2:I3 H8:I10 H123:H130 I6:I12 I14 I16:I19 I22 I24:I25 I27:I29 I31:I37 I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Confirmed,1st Week,2nd Week,Tentative,In Process,Initial Stage,Completed,Cancelled"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B6:B10 B11:B19 B127 B131:B132 B137:B138 C3 C8:C9 C124:C126 C128:C130 C133:C135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B6:B19 B127 B131:B132 B137:B138 C3 C8:C9 C124:C126 C128:C130 C133:C135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alpha Lab,Brookes Pharma,DTM,Golden Pearl,Mabley Beauty,Mega Grey,PBS,Samsol"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C6:C10 C11:C19 C127 C131:C132 C137:C138 D3 D8:D10 D124:D136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C6:C19 C127 C131:C132 C137:C138 D3 D8:D10 D124:D136" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CONTRATUBEX GEL 20G,DTM DIA 25MM,EAZICOLOR PREMIUM 60ML,H.H 100GM,HELLO HAIR COLOR,M.G (Mega Grey),PHLOGIN GEL 20G,PYODINE GEL 20GM,S 43 25MM,S-43 DIA 20.5,S-45 DIA 20.5,TRANSPARENT BOTTLE 150ML,TUBES (Samsol 25),V-HC BLACK (Vince),VINCE NURTURAL (VARNISH"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -17288,193 +17334,420 @@
       <c r="S92" s="271" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="243">
-      <c r="A93" s="176" t="n"/>
-      <c r="B93" s="177" t="n"/>
-      <c r="C93" s="177" t="n"/>
-      <c r="D93" s="177" t="n"/>
-      <c r="E93" s="177" t="n"/>
-      <c r="F93" s="177" t="n"/>
-      <c r="G93" s="178" t="n"/>
-      <c r="H93" s="178" t="n"/>
-      <c r="I93" s="178" t="n"/>
-      <c r="J93" s="179" t="n"/>
-      <c r="K93" s="177" t="n"/>
-      <c r="L93" s="177" t="n"/>
-      <c r="M93" s="177" t="n"/>
-      <c r="N93" s="177" t="n"/>
-      <c r="O93" s="177" t="n"/>
-      <c r="P93" s="177" t="n"/>
-      <c r="Q93" s="177" t="n"/>
-      <c r="R93" s="177" t="n"/>
-      <c r="S93" s="177" t="n"/>
+      <c r="A93" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B93" s="271" t="inlineStr">
+        <is>
+          <t>Lacquer-02</t>
+        </is>
+      </c>
+      <c r="C93" s="271" t="inlineStr"/>
+      <c r="D93" s="271" t="inlineStr"/>
+      <c r="E93" s="271" t="inlineStr"/>
+      <c r="F93" s="271" t="n"/>
+      <c r="G93" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" s="273">
+        <f>IFERROR(I93/(H93+I93),"")</f>
+        <v/>
+      </c>
+      <c r="K93" s="271" t="n"/>
+      <c r="L93" s="271" t="n"/>
+      <c r="M93" s="271" t="n"/>
+      <c r="N93" s="271" t="n"/>
+      <c r="O93" s="271" t="n"/>
+      <c r="P93" s="271" t="n"/>
+      <c r="Q93" s="271" t="n"/>
+      <c r="R93" s="271" t="n"/>
+      <c r="S93" s="271" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="243">
-      <c r="A94" s="176" t="n"/>
-      <c r="B94" s="177" t="n"/>
-      <c r="C94" s="177" t="n"/>
-      <c r="D94" s="177" t="n"/>
-      <c r="E94" s="177" t="n"/>
-      <c r="F94" s="177" t="n"/>
-      <c r="G94" s="178" t="n"/>
-      <c r="H94" s="178" t="n"/>
-      <c r="I94" s="178" t="n"/>
-      <c r="J94" s="179" t="n"/>
-      <c r="K94" s="177" t="n"/>
-      <c r="L94" s="177" t="n"/>
-      <c r="M94" s="177" t="n"/>
-      <c r="N94" s="177" t="n"/>
-      <c r="O94" s="177" t="n"/>
-      <c r="P94" s="177" t="n"/>
-      <c r="Q94" s="177" t="n"/>
-      <c r="R94" s="177" t="n"/>
-      <c r="S94" s="177" t="n"/>
+      <c r="A94" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B94" s="271" t="inlineStr">
+        <is>
+          <t>Lacquer-04</t>
+        </is>
+      </c>
+      <c r="C94" s="271" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D94" s="271" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="E94" s="271" t="n">
+        <v>25</v>
+      </c>
+      <c r="F94" s="271" t="n">
+        <v>5389</v>
+      </c>
+      <c r="G94" s="272" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H94" s="272" t="n">
+        <v>15715</v>
+      </c>
+      <c r="I94" s="272" t="n">
+        <v>285</v>
+      </c>
+      <c r="J94" s="273">
+        <f>IFERROR(I94/(H94+I94),"")</f>
+        <v/>
+      </c>
+      <c r="K94" s="271" t="n"/>
+      <c r="L94" s="271" t="n"/>
+      <c r="M94" s="271" t="n">
+        <v>90</v>
+      </c>
+      <c r="N94" s="271" t="n"/>
+      <c r="O94" s="271" t="n"/>
+      <c r="P94" s="271" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q94" s="271" t="n"/>
+      <c r="R94" s="271" t="n"/>
+      <c r="S94" s="271" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="243">
-      <c r="A95" s="176" t="n"/>
-      <c r="B95" s="177" t="n"/>
-      <c r="C95" s="177" t="n"/>
-      <c r="D95" s="177" t="n"/>
-      <c r="E95" s="177" t="n"/>
-      <c r="F95" s="177" t="n"/>
-      <c r="G95" s="178" t="n"/>
-      <c r="H95" s="178" t="n"/>
-      <c r="I95" s="178" t="n"/>
-      <c r="J95" s="179" t="n"/>
-      <c r="K95" s="177" t="n"/>
-      <c r="L95" s="177" t="n"/>
-      <c r="M95" s="177" t="n"/>
-      <c r="N95" s="177" t="n"/>
-      <c r="O95" s="177" t="n"/>
-      <c r="P95" s="177" t="n"/>
-      <c r="Q95" s="177" t="n"/>
-      <c r="R95" s="177" t="n"/>
-      <c r="S95" s="177" t="n"/>
+      <c r="A95" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B95" s="271" t="inlineStr">
+        <is>
+          <t>Latex-01</t>
+        </is>
+      </c>
+      <c r="C95" s="271" t="inlineStr"/>
+      <c r="D95" s="271" t="inlineStr"/>
+      <c r="E95" s="271" t="inlineStr"/>
+      <c r="F95" s="271" t="n"/>
+      <c r="G95" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" s="273">
+        <f>IFERROR(I95/(H95+I95),"")</f>
+        <v/>
+      </c>
+      <c r="K95" s="271" t="n"/>
+      <c r="L95" s="271" t="n"/>
+      <c r="M95" s="271" t="n"/>
+      <c r="N95" s="271" t="n"/>
+      <c r="O95" s="271" t="n"/>
+      <c r="P95" s="271" t="n"/>
+      <c r="Q95" s="271" t="n"/>
+      <c r="R95" s="271" t="n"/>
+      <c r="S95" s="271" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1" s="243">
-      <c r="A96" s="176" t="n"/>
-      <c r="B96" s="177" t="n"/>
-      <c r="C96" s="177" t="n"/>
-      <c r="D96" s="177" t="n"/>
-      <c r="E96" s="177" t="n"/>
-      <c r="F96" s="177" t="n"/>
-      <c r="G96" s="178" t="n"/>
-      <c r="H96" s="178" t="n"/>
-      <c r="I96" s="178" t="n"/>
-      <c r="J96" s="179" t="n"/>
-      <c r="K96" s="177" t="n"/>
-      <c r="L96" s="177" t="n"/>
-      <c r="M96" s="177" t="n"/>
-      <c r="N96" s="177" t="n"/>
-      <c r="O96" s="177" t="n"/>
-      <c r="P96" s="177" t="n"/>
-      <c r="Q96" s="177" t="n"/>
-      <c r="R96" s="177" t="n"/>
-      <c r="S96" s="177" t="n"/>
+      <c r="A96" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B96" s="271" t="inlineStr">
+        <is>
+          <t>PF Machine</t>
+        </is>
+      </c>
+      <c r="C96" s="271" t="inlineStr">
+        <is>
+          <t>Alpha Labs PVT LTD</t>
+        </is>
+      </c>
+      <c r="D96" s="271" t="inlineStr">
+        <is>
+          <t>TRANSPARENT BOTTLE 150ML</t>
+        </is>
+      </c>
+      <c r="E96" s="271" t="inlineStr">
+        <is>
+          <t>150 ml</t>
+        </is>
+      </c>
+      <c r="F96" s="271" t="n">
+        <v>8001</v>
+      </c>
+      <c r="G96" s="272" t="n">
+        <v>6020</v>
+      </c>
+      <c r="H96" s="272" t="n">
+        <v>5520</v>
+      </c>
+      <c r="I96" s="272" t="n">
+        <v>500</v>
+      </c>
+      <c r="J96" s="273">
+        <f>IFERROR(I96/(H96+I96),"")</f>
+        <v/>
+      </c>
+      <c r="K96" s="271" t="n"/>
+      <c r="L96" s="271" t="n"/>
+      <c r="M96" s="271" t="n"/>
+      <c r="N96" s="271" t="n"/>
+      <c r="O96" s="271" t="n"/>
+      <c r="P96" s="271" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q96" s="271" t="n"/>
+      <c r="R96" s="271" t="n"/>
+      <c r="S96" s="271" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1" s="243">
-      <c r="A97" s="176" t="n"/>
-      <c r="B97" s="177" t="n"/>
-      <c r="C97" s="177" t="n"/>
-      <c r="D97" s="177" t="n"/>
-      <c r="E97" s="177" t="n"/>
-      <c r="F97" s="177" t="n"/>
-      <c r="G97" s="178" t="n"/>
-      <c r="H97" s="178" t="n"/>
-      <c r="I97" s="178" t="n"/>
-      <c r="J97" s="179" t="n"/>
-      <c r="K97" s="177" t="n"/>
-      <c r="L97" s="177" t="n"/>
-      <c r="M97" s="177" t="n"/>
-      <c r="N97" s="177" t="n"/>
-      <c r="O97" s="177" t="n"/>
-      <c r="P97" s="177" t="n"/>
-      <c r="Q97" s="177" t="n"/>
-      <c r="R97" s="177" t="n"/>
-      <c r="S97" s="177" t="n"/>
+      <c r="A97" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B97" s="271" t="inlineStr">
+        <is>
+          <t>Press-04</t>
+        </is>
+      </c>
+      <c r="C97" s="271" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D97" s="271" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E97" s="271" t="n">
+        <v>30</v>
+      </c>
+      <c r="F97" s="271" t="n">
+        <v>6206</v>
+      </c>
+      <c r="G97" s="272" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H97" s="272" t="n">
+        <v>9890</v>
+      </c>
+      <c r="I97" s="272" t="n">
+        <v>110</v>
+      </c>
+      <c r="J97" s="273">
+        <f>IFERROR(I97/(H97+I97),"")</f>
+        <v/>
+      </c>
+      <c r="K97" s="271" t="n"/>
+      <c r="L97" s="271" t="n"/>
+      <c r="M97" s="271" t="n"/>
+      <c r="N97" s="271" t="n">
+        <v>210</v>
+      </c>
+      <c r="O97" s="271" t="n"/>
+      <c r="P97" s="271" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q97" s="271" t="n"/>
+      <c r="R97" s="271" t="n"/>
+      <c r="S97" s="271" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1" s="243">
-      <c r="A98" s="176" t="n"/>
-      <c r="B98" s="177" t="n"/>
-      <c r="C98" s="177" t="n"/>
-      <c r="D98" s="177" t="n"/>
-      <c r="E98" s="177" t="n"/>
-      <c r="F98" s="177" t="n"/>
-      <c r="G98" s="178" t="n"/>
-      <c r="H98" s="178" t="n"/>
-      <c r="I98" s="178" t="n"/>
-      <c r="J98" s="179" t="n"/>
-      <c r="K98" s="177" t="n"/>
-      <c r="L98" s="177" t="n"/>
-      <c r="M98" s="177" t="n"/>
-      <c r="N98" s="177" t="n"/>
-      <c r="O98" s="177" t="n"/>
-      <c r="P98" s="177" t="n"/>
-      <c r="Q98" s="177" t="n"/>
-      <c r="R98" s="177" t="n"/>
-      <c r="S98" s="177" t="n"/>
+      <c r="A98" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B98" s="271" t="inlineStr">
+        <is>
+          <t>Press-06</t>
+        </is>
+      </c>
+      <c r="C98" s="271" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D98" s="271" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="E98" s="271" t="n">
+        <v>25</v>
+      </c>
+      <c r="F98" s="271" t="n">
+        <v>5389</v>
+      </c>
+      <c r="G98" s="272" t="n">
+        <v>18500</v>
+      </c>
+      <c r="H98" s="272" t="n">
+        <v>18375</v>
+      </c>
+      <c r="I98" s="272" t="n">
+        <v>125</v>
+      </c>
+      <c r="J98" s="273">
+        <f>IFERROR(I98/(H98+I98),"")</f>
+        <v/>
+      </c>
+      <c r="K98" s="271" t="n">
+        <v>60</v>
+      </c>
+      <c r="L98" s="271" t="n"/>
+      <c r="M98" s="271" t="n"/>
+      <c r="N98" s="271" t="n"/>
+      <c r="O98" s="271" t="n"/>
+      <c r="P98" s="271" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q98" s="271" t="n"/>
+      <c r="R98" s="271" t="n"/>
+      <c r="S98" s="271" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="243">
-      <c r="A99" s="176" t="n"/>
-      <c r="B99" s="177" t="n"/>
-      <c r="C99" s="177" t="n"/>
-      <c r="D99" s="177" t="n"/>
-      <c r="E99" s="177" t="n"/>
-      <c r="F99" s="177" t="n"/>
-      <c r="G99" s="178" t="n"/>
-      <c r="H99" s="178" t="n"/>
-      <c r="I99" s="178" t="n"/>
-      <c r="J99" s="179" t="n"/>
-      <c r="K99" s="177" t="n"/>
-      <c r="L99" s="177" t="n"/>
-      <c r="M99" s="177" t="n"/>
-      <c r="N99" s="177" t="n"/>
-      <c r="O99" s="177" t="n"/>
-      <c r="P99" s="177" t="n"/>
-      <c r="Q99" s="177" t="n"/>
-      <c r="R99" s="177" t="n"/>
-      <c r="S99" s="177" t="n"/>
+      <c r="A99" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B99" s="271" t="inlineStr">
+        <is>
+          <t>Printing-03</t>
+        </is>
+      </c>
+      <c r="C99" s="271" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D99" s="271" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="E99" s="271" t="n">
+        <v>25</v>
+      </c>
+      <c r="F99" s="271" t="n">
+        <v>5389</v>
+      </c>
+      <c r="G99" s="272" t="n">
+        <v>14898</v>
+      </c>
+      <c r="H99" s="272" t="n">
+        <v>14448</v>
+      </c>
+      <c r="I99" s="272" t="n">
+        <v>450</v>
+      </c>
+      <c r="J99" s="273">
+        <f>IFERROR(I99/(H99+I99),"")</f>
+        <v/>
+      </c>
+      <c r="K99" s="271" t="n"/>
+      <c r="L99" s="271" t="n"/>
+      <c r="M99" s="271" t="n"/>
+      <c r="N99" s="271" t="n"/>
+      <c r="O99" s="271" t="n"/>
+      <c r="P99" s="271" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q99" s="271" t="n"/>
+      <c r="R99" s="271" t="n"/>
+      <c r="S99" s="271" t="n"/>
     </row>
     <row r="100" ht="15" customHeight="1" s="243">
-      <c r="A100" s="176" t="n"/>
-      <c r="B100" s="177" t="n"/>
-      <c r="C100" s="177" t="n"/>
-      <c r="D100" s="177" t="n"/>
-      <c r="E100" s="177" t="n"/>
-      <c r="F100" s="177" t="n"/>
-      <c r="G100" s="178" t="n"/>
-      <c r="H100" s="178" t="n"/>
-      <c r="I100" s="178" t="n"/>
-      <c r="J100" s="179" t="n"/>
-      <c r="K100" s="177" t="n"/>
-      <c r="L100" s="177" t="n"/>
-      <c r="M100" s="177" t="n"/>
-      <c r="N100" s="177" t="n"/>
-      <c r="O100" s="177" t="n"/>
-      <c r="P100" s="177" t="n"/>
-      <c r="Q100" s="177" t="n"/>
-      <c r="R100" s="177" t="n"/>
-      <c r="S100" s="177" t="n"/>
+      <c r="A100" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B100" s="271" t="inlineStr">
+        <is>
+          <t>Printing-03</t>
+        </is>
+      </c>
+      <c r="C100" s="271" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D100" s="271" t="inlineStr">
+        <is>
+          <t>S 43 25MM</t>
+        </is>
+      </c>
+      <c r="E100" s="271" t="n">
+        <v>25</v>
+      </c>
+      <c r="F100" s="271" t="n">
+        <v>3447</v>
+      </c>
+      <c r="G100" s="272" t="n">
+        <v>4864</v>
+      </c>
+      <c r="H100" s="272" t="n">
+        <v>4704</v>
+      </c>
+      <c r="I100" s="272" t="n">
+        <v>160</v>
+      </c>
+      <c r="J100" s="273">
+        <f>IFERROR(I100/(H100+I100),"")</f>
+        <v/>
+      </c>
+      <c r="K100" s="271" t="n"/>
+      <c r="L100" s="271" t="n"/>
+      <c r="M100" s="271" t="n"/>
+      <c r="N100" s="271" t="n">
+        <v>30</v>
+      </c>
+      <c r="O100" s="271" t="n"/>
+      <c r="P100" s="271" t="n"/>
+      <c r="Q100" s="271" t="n"/>
+      <c r="R100" s="271" t="n"/>
+      <c r="S100" s="271" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1" s="243">
-      <c r="A101" s="176" t="n"/>
-      <c r="B101" s="177" t="n"/>
-      <c r="C101" s="177" t="n"/>
-      <c r="D101" s="177" t="n"/>
-      <c r="E101" s="177" t="n"/>
-      <c r="F101" s="177" t="n"/>
-      <c r="G101" s="178" t="n"/>
-      <c r="H101" s="178" t="n"/>
-      <c r="I101" s="178" t="n"/>
-      <c r="J101" s="179" t="n"/>
-      <c r="K101" s="177" t="n"/>
-      <c r="L101" s="177" t="n"/>
-      <c r="M101" s="177" t="n"/>
-      <c r="N101" s="177" t="n"/>
-      <c r="O101" s="177" t="n"/>
-      <c r="P101" s="177" t="n"/>
-      <c r="Q101" s="177" t="n"/>
-      <c r="R101" s="177" t="n"/>
-      <c r="S101" s="177" t="n"/>
+      <c r="A101" s="274" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B101" s="271" t="inlineStr">
+        <is>
+          <t>Printing-04</t>
+        </is>
+      </c>
+      <c r="C101" s="271" t="inlineStr"/>
+      <c r="D101" s="271" t="inlineStr"/>
+      <c r="E101" s="271" t="inlineStr"/>
+      <c r="F101" s="271" t="n"/>
+      <c r="G101" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" s="272" t="n">
+        <v>0</v>
+      </c>
+      <c r="J101" s="273">
+        <f>IFERROR(I101/(H101+I101),"")</f>
+        <v/>
+      </c>
+      <c r="K101" s="271" t="n"/>
+      <c r="L101" s="271" t="n"/>
+      <c r="M101" s="271" t="n"/>
+      <c r="N101" s="271" t="n"/>
+      <c r="O101" s="271" t="n"/>
+      <c r="P101" s="271" t="n"/>
+      <c r="Q101" s="271" t="n"/>
+      <c r="R101" s="271" t="n"/>
+      <c r="S101" s="271" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1" s="243">
       <c r="A102" s="176" t="n"/>
@@ -38440,13 +38713,13 @@
   <cols>
     <col width="10" customWidth="1" style="243" min="1" max="1"/>
     <col width="15.28515625" customWidth="1" style="243" min="2" max="2"/>
-    <col width="16.85546875" customWidth="1" style="243" min="3" max="3"/>
+    <col width="33.140625" customWidth="1" style="243" min="3" max="3"/>
     <col width="6" customWidth="1" style="243" min="4" max="4"/>
     <col width="8.5703125" customWidth="1" style="67" min="5" max="5"/>
     <col width="8.85546875" customWidth="1" style="67" min="6" max="6"/>
     <col width="11.140625" customWidth="1" style="67" min="7" max="7"/>
     <col width="8.5703125" customWidth="1" style="68" min="8" max="8"/>
-    <col width="7.7109375" customWidth="1" style="67" min="9" max="9"/>
+    <col hidden="1" width="7.7109375" customWidth="1" style="67" min="9" max="9"/>
     <col width="16.140625" customWidth="1" style="67" min="10" max="10"/>
     <col width="18" customWidth="1" style="243" min="11" max="11"/>
   </cols>
@@ -38457,13 +38730,13 @@
           <t>Slugs Inventory — June 2026 MONTH TO DATE</t>
         </is>
       </c>
-      <c r="B1" s="241" t="n"/>
-      <c r="C1" s="241" t="n"/>
-      <c r="D1" s="241" t="n"/>
-      <c r="E1" s="241" t="n"/>
-      <c r="F1" s="241" t="n"/>
-      <c r="G1" s="241" t="n"/>
-      <c r="H1" s="241" t="n"/>
+      <c r="B1" s="238" t="n"/>
+      <c r="C1" s="238" t="n"/>
+      <c r="D1" s="238" t="n"/>
+      <c r="E1" s="238" t="n"/>
+      <c r="F1" s="238" t="n"/>
+      <c r="G1" s="238" t="n"/>
+      <c r="H1" s="238" t="n"/>
       <c r="I1" s="69" t="inlineStr">
         <is>
           <t>Date:</t>
@@ -38704,14 +38977,14 @@
         <v>0</v>
       </c>
       <c r="G7" s="37" t="n">
-        <v>1150</v>
+        <v>1215</v>
       </c>
       <c r="H7" s="38">
         <f>E7+F7-G7</f>
         <v/>
       </c>
       <c r="I7" s="37" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="J7" s="37">
         <f>IFERROR(IF(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])=0,"-",ROUND((H7+I7)/(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])/1000),0)),"-")</f>
@@ -38750,7 +39023,9 @@
         <f>E8+F8-G8</f>
         <v/>
       </c>
-      <c r="I8" s="37" t="n"/>
+      <c r="I8" s="37" t="n">
+        <v>10</v>
+      </c>
       <c r="J8" s="37">
         <f>IFERROR(IF(AVERAGEIF(TableBOM[Item ID],A8,TableBOM[Per 1000 Units])=0,"-",ROUND((H8+I8)/(AVERAGEIF(TableBOM[Item ID],A8,TableBOM[Per 1000 Units])/1000),0)),"-")</f>
         <v/>
@@ -39088,7 +39363,7 @@
         <v>100</v>
       </c>
       <c r="G18" s="37" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="H18" s="38">
         <f>E18+F18-G18</f>
@@ -39244,7 +39519,7 @@
         <v>210</v>
       </c>
       <c r="G22" s="37" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="H22" s="38">
         <f>E22+F22-G22</f>
@@ -40251,10 +40526,10 @@
         <v>70000</v>
       </c>
       <c r="F46" s="37" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="G46" s="37" t="n">
-        <v>70000</v>
+        <v>100000</v>
       </c>
       <c r="H46" s="38">
         <f>E46+F46-G46</f>
@@ -40514,13 +40789,13 @@
         </is>
       </c>
       <c r="E52" s="37" t="n">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="F52" s="37" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="37" t="n">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="H52" s="38">
         <f>E52+F52-G52</f>
@@ -40954,7 +41229,7 @@
         <v>0</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="H62" s="38">
         <f>E62+F62-G62</f>
@@ -41481,7 +41756,7 @@
         <v>0</v>
       </c>
       <c r="F74" s="37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G74" s="37" t="n">
         <v>0</v>
@@ -41792,7 +42067,7 @@
         <v>1</v>
       </c>
       <c r="G81" s="37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H81" s="38">
         <f>E81+F81-G81</f>
@@ -42245,7 +42520,7 @@
         <v>1</v>
       </c>
       <c r="F93" s="37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G93" s="37" t="n">
         <v>0</v>
@@ -50876,11 +51151,11 @@
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A92:K92"/>
-    <mergeCell ref="A23:K23"/>
     <mergeCell ref="A65:K65"/>
     <mergeCell ref="A81:K81"/>
+    <mergeCell ref="A75:K75"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A75:K75"/>
+    <mergeCell ref="A23:K23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
@@ -55597,8 +55872,8 @@
     <mergeCell ref="A68:F68"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A94:F94"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A94:F94"/>
     <mergeCell ref="A110:F110"/>
     <mergeCell ref="A119:F119"/>
   </mergeCells>

</xml_diff>

<commit_message>
Full backup 16/06/2026 12:34:05
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tubex_Dashboard" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'MRP'!$A$13:$K$95</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Production_Log'!$A$2:$R$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Production_Log'!$A$2:$R$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'BOM Issues'!$A$52:$J$64</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -1410,12 +1410,30 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="36" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="36" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1425,24 +1443,6 @@
     <xf numFmtId="0" fontId="42" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="36" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -1464,6 +1464,9 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1471,9 +1474,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2067,23 +2067,23 @@
   <dimension ref="A1:AC199"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="16.5"/>
   <cols>
-    <col width="1.5703125" customWidth="1" style="228" min="1" max="1"/>
-    <col width="7" customWidth="1" style="228" min="2" max="2"/>
-    <col width="32.7109375" customWidth="1" style="228" min="3" max="3"/>
-    <col width="38.7109375" customWidth="1" style="228" min="4" max="4"/>
-    <col width="8.85546875" customWidth="1" style="229" min="5" max="5"/>
-    <col width="9.140625" customWidth="1" style="228" min="6" max="6"/>
-    <col width="11" customWidth="1" style="230" min="7" max="7"/>
-    <col width="11.140625" customWidth="1" style="228" min="8" max="8"/>
-    <col width="10.28515625" customWidth="1" style="228" min="9" max="9"/>
-    <col width="10.5703125" customWidth="1" style="228" min="10" max="10"/>
-    <col width="9.28515625" customWidth="1" style="228" min="11" max="11"/>
-    <col width="35.140625" customWidth="1" style="228" min="12" max="12"/>
-    <col width="14.7109375" customWidth="1" style="228" min="13" max="13"/>
-    <col width="13.28515625" customWidth="1" style="228" min="14" max="14"/>
-    <col width="9.5703125" customWidth="1" style="228" min="15" max="15"/>
-    <col width="8.7109375" customWidth="1" style="228" min="16" max="57"/>
-    <col width="8.7109375" customWidth="1" style="228" min="58" max="16384"/>
+    <col width="1.5703125" customWidth="1" style="233" min="1" max="1"/>
+    <col width="7" customWidth="1" style="233" min="2" max="2"/>
+    <col width="32.7109375" customWidth="1" style="233" min="3" max="3"/>
+    <col width="38.7109375" customWidth="1" style="233" min="4" max="4"/>
+    <col width="8.85546875" customWidth="1" style="234" min="5" max="5"/>
+    <col width="9.140625" customWidth="1" style="233" min="6" max="6"/>
+    <col width="11" customWidth="1" style="235" min="7" max="7"/>
+    <col width="11.140625" customWidth="1" style="233" min="8" max="8"/>
+    <col width="10.28515625" customWidth="1" style="233" min="9" max="9"/>
+    <col width="10.5703125" customWidth="1" style="233" min="10" max="10"/>
+    <col width="9.28515625" customWidth="1" style="233" min="11" max="11"/>
+    <col width="35.140625" customWidth="1" style="233" min="12" max="12"/>
+    <col width="14.7109375" customWidth="1" style="233" min="13" max="13"/>
+    <col width="13.28515625" customWidth="1" style="233" min="14" max="14"/>
+    <col width="9.5703125" customWidth="1" style="233" min="15" max="15"/>
+    <col width="8.7109375" customWidth="1" style="233" min="16" max="58"/>
+    <col width="8.7109375" customWidth="1" style="233" min="59" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="6" customHeight="1" s="243">
@@ -2399,21 +2399,21 @@
     </row>
     <row r="9" ht="20.25" customHeight="1" s="243">
       <c r="A9" s="136" t="n"/>
-      <c r="B9" s="237" t="inlineStr">
+      <c r="B9" s="230" t="inlineStr">
         <is>
           <t>Summary of Production &amp; Dispatch - MTD</t>
         </is>
       </c>
-      <c r="C9" s="238" t="n"/>
-      <c r="D9" s="238" t="n"/>
-      <c r="E9" s="238" t="n"/>
-      <c r="F9" s="238" t="n"/>
-      <c r="G9" s="238" t="n"/>
-      <c r="H9" s="238" t="n"/>
-      <c r="I9" s="238" t="n"/>
-      <c r="J9" s="238" t="n"/>
-      <c r="K9" s="238" t="n"/>
-      <c r="L9" s="238" t="n"/>
+      <c r="C9" s="231" t="n"/>
+      <c r="D9" s="231" t="n"/>
+      <c r="E9" s="231" t="n"/>
+      <c r="F9" s="231" t="n"/>
+      <c r="G9" s="231" t="n"/>
+      <c r="H9" s="231" t="n"/>
+      <c r="I9" s="231" t="n"/>
+      <c r="J9" s="231" t="n"/>
+      <c r="K9" s="231" t="n"/>
+      <c r="L9" s="231" t="n"/>
       <c r="M9" s="157">
         <f>IFERROR(INDEX($S$9:$S$23,MATCH(LARGE($U$9:$U$23,3),$U$9:$U$23,0)),"")</f>
         <v/>
@@ -2884,9 +2884,8 @@
       <c r="F15" s="292" t="n">
         <v>5389</v>
       </c>
-      <c r="G15" s="292">
-        <f>IFERROR(INDEX(MRP!$F$3:$F$10,MATCH(Tubex_Dashboard!F15,MRP!$D$3:$D$10,0)),0)</f>
-        <v/>
+      <c r="G15" s="292" t="n">
+        <v>49056</v>
       </c>
       <c r="H15" s="293">
         <f>SUMPRODUCT((Production_Log!$F$3:$F$8963=F15)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
@@ -4148,7 +4147,7 @@
       <c r="P36" s="136" t="n"/>
       <c r="Q36" s="136" t="n"/>
       <c r="R36" s="136" t="n"/>
-      <c r="S36" s="228" t="inlineStr">
+      <c r="S36" s="233" t="inlineStr">
         <is>
           <t>Gas Shutdown</t>
         </is>
@@ -4157,7 +4156,7 @@
         <f>SUMPRODUCT((MONTH(Production_Log!$A$3:$A$8963)=MONTH(TODAY()))*(YEAR(Production_Log!$A$3:$A$8963)=YEAR(TODAY()))*Production_Log!$Q$3:$Q$8963)</f>
         <v/>
       </c>
-      <c r="U36" s="228">
+      <c r="U36" s="233">
         <f>T36+0.00006</f>
         <v/>
       </c>
@@ -6140,7 +6139,7 @@
         <v>6892</v>
       </c>
       <c r="F4" s="185" t="n">
-        <v>48176</v>
+        <v>49056</v>
       </c>
       <c r="G4" s="19">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$58,MATCH(MRP!D4,Tubex_Dashboard!$F$11:$F$58,0))</f>
@@ -6281,7 +6280,7 @@
         <v>6887</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>52000</v>
+        <v>30000</v>
       </c>
       <c r="G8" s="19">
         <f>INDEX(Tubex_Dashboard!$H$11:$H$58,MATCH(MRP!D8,Tubex_Dashboard!$F$11:$F$58,0))</f>
@@ -6932,9 +6931,10 @@
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A21)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A21)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A21)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A21)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A21)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A21)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A21)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A21)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A21)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A21)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A21)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A21)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A21)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A21)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A21)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A21)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A21)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A21)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A21)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A21)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A21)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A21)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A21)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A21)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))-2),"")</f>
         <v/>
       </c>
-      <c r="I21" s="30">
-        <f>IF(E21=0,"Not needed",IF(G21&lt;0,"SHORTAGE",IF(G21&lt;F21*0.1,"LOW","OK")))</f>
-        <v/>
+      <c r="I21" s="30" t="inlineStr">
+        <is>
+          <t>100kg Shortage. 15k Tubes WIP</t>
+        </is>
       </c>
       <c r="J21" s="30">
         <f>IF(B21&lt;&gt;"CAP","",SUMPRODUCT((ISNUMBER(SEARCH("Cap Not Available",'FG Stock'!$H$4:$H$100)))*('FG Stock'!$I$4:$I$100=A21)*'FG Stock'!$F$4:$F$100))</f>
@@ -10709,14 +10709,14 @@
           <t>June 2026 PET Required Pet Orders</t>
         </is>
       </c>
-      <c r="B98" s="240" t="n"/>
-      <c r="C98" s="240" t="n"/>
-      <c r="D98" s="240" t="n"/>
-      <c r="E98" s="240" t="n"/>
-      <c r="F98" s="240" t="n"/>
+      <c r="B98" s="228" t="n"/>
+      <c r="C98" s="228" t="n"/>
+      <c r="D98" s="228" t="n"/>
+      <c r="E98" s="228" t="n"/>
+      <c r="F98" s="228" t="n"/>
       <c r="G98" s="188" t="n"/>
-      <c r="H98" s="240" t="n"/>
-      <c r="I98" s="241" t="n"/>
+      <c r="H98" s="228" t="n"/>
+      <c r="I98" s="229" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="243">
       <c r="A99" s="12" t="inlineStr">
@@ -10971,14 +10971,14 @@
           <t>JUNE PET MATERIAL REQUIREMENT PLAN</t>
         </is>
       </c>
-      <c r="B106" s="240" t="n"/>
-      <c r="C106" s="240" t="n"/>
-      <c r="D106" s="240" t="n"/>
-      <c r="E106" s="240" t="n"/>
-      <c r="F106" s="240" t="n"/>
+      <c r="B106" s="228" t="n"/>
+      <c r="C106" s="228" t="n"/>
+      <c r="D106" s="228" t="n"/>
+      <c r="E106" s="228" t="n"/>
+      <c r="F106" s="228" t="n"/>
       <c r="G106" s="188" t="n"/>
-      <c r="H106" s="240" t="n"/>
-      <c r="I106" s="240" t="n"/>
+      <c r="H106" s="228" t="n"/>
+      <c r="I106" s="228" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="243">
       <c r="A107" s="41" t="inlineStr">
@@ -11168,14 +11168,14 @@
       <c r="A111" s="262" t="n">
         <v>5977</v>
       </c>
-      <c r="B111" s="240" t="n"/>
-      <c r="C111" s="240" t="n"/>
-      <c r="D111" s="240" t="n"/>
-      <c r="E111" s="240" t="n"/>
-      <c r="F111" s="240" t="n"/>
-      <c r="G111" s="240" t="n"/>
-      <c r="H111" s="240" t="n"/>
-      <c r="I111" s="241" t="n"/>
+      <c r="B111" s="228" t="n"/>
+      <c r="C111" s="228" t="n"/>
+      <c r="D111" s="228" t="n"/>
+      <c r="E111" s="228" t="n"/>
+      <c r="F111" s="228" t="n"/>
+      <c r="G111" s="228" t="n"/>
+      <c r="H111" s="228" t="n"/>
+      <c r="I111" s="229" t="n"/>
       <c r="K111" s="47">
         <f>IF(E106=0,"",MAX(0,E106-F106))</f>
         <v/>
@@ -11185,14 +11185,14 @@
       <c r="A112" s="196" t="n">
         <v>2267</v>
       </c>
-      <c r="B112" s="240" t="n"/>
-      <c r="C112" s="240" t="n"/>
-      <c r="D112" s="240" t="n"/>
-      <c r="E112" s="240" t="n"/>
-      <c r="F112" s="240" t="n"/>
-      <c r="G112" s="240" t="n"/>
-      <c r="H112" s="240" t="n"/>
-      <c r="I112" s="241" t="n"/>
+      <c r="B112" s="228" t="n"/>
+      <c r="C112" s="228" t="n"/>
+      <c r="D112" s="228" t="n"/>
+      <c r="E112" s="228" t="n"/>
+      <c r="F112" s="228" t="n"/>
+      <c r="G112" s="228" t="n"/>
+      <c r="H112" s="228" t="n"/>
+      <c r="I112" s="229" t="n"/>
       <c r="K112" s="48">
         <f>IF(E107=0,"",MAX(0,E107-F107))</f>
         <v/>
@@ -11332,14 +11332,14 @@
     </row>
     <row r="116" ht="15" customHeight="1" s="243">
       <c r="A116" s="187" t="n"/>
-      <c r="B116" s="240" t="n"/>
-      <c r="C116" s="240" t="n"/>
-      <c r="D116" s="240" t="n"/>
-      <c r="E116" s="240" t="n"/>
-      <c r="F116" s="240" t="n"/>
+      <c r="B116" s="228" t="n"/>
+      <c r="C116" s="228" t="n"/>
+      <c r="D116" s="228" t="n"/>
+      <c r="E116" s="228" t="n"/>
+      <c r="F116" s="228" t="n"/>
       <c r="G116" s="188" t="n"/>
-      <c r="H116" s="240" t="n"/>
-      <c r="I116" s="241" t="n"/>
+      <c r="H116" s="228" t="n"/>
+      <c r="I116" s="229" t="n"/>
     </row>
     <row r="117" ht="15" customHeight="1" s="243">
       <c r="A117" s="6" t="inlineStr">
@@ -13242,24 +13242,23 @@
   <autoFilter ref="A13:K95">
     <filterColumn colId="4" hiddenButton="0" showButton="1">
       <filters>
-        <filter val="1,516"/>
-        <filter val="111"/>
+        <filter val="1,466"/>
+        <filter val="104"/>
         <filter val="138"/>
         <filter val="15"/>
+        <filter val="165"/>
         <filter val="188"/>
+        <filter val="193"/>
         <filter val="2"/>
-        <filter val="20"/>
-        <filter val="222"/>
+        <filter val="2,898"/>
         <filter val="25,500"/>
-        <filter val="263"/>
+        <filter val="279"/>
         <filter val="3"/>
-        <filter val="3,092"/>
-        <filter val="305"/>
-        <filter val="347,688"/>
-        <filter val="66,606"/>
+        <filter val="331,114"/>
+        <filter val="44,166"/>
         <filter val="69"/>
         <filter val="89"/>
-        <filter val="99"/>
+        <filter val="96"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -13320,7 +13319,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -13459,7 +13458,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="243">
+    <row r="3" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A3" s="274" t="n">
         <v>46174</v>
       </c>
@@ -13509,7 +13508,7 @@
       <c r="R3" s="271" t="n"/>
       <c r="S3" s="271" t="n"/>
     </row>
-    <row r="4" ht="15" customHeight="1" s="243">
+    <row r="4" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A4" s="274" t="n">
         <v>46174</v>
       </c>
@@ -13557,7 +13556,7 @@
       <c r="R4" s="271" t="n"/>
       <c r="S4" s="271" t="n"/>
     </row>
-    <row r="5" ht="15" customHeight="1" s="243">
+    <row r="5" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A5" s="274" t="n">
         <v>46174</v>
       </c>
@@ -13605,7 +13604,7 @@
       <c r="R5" s="271" t="n"/>
       <c r="S5" s="271" t="n"/>
     </row>
-    <row r="6" ht="15" customHeight="1" s="243">
+    <row r="6" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A6" s="274" t="n">
         <v>46174</v>
       </c>
@@ -13657,7 +13656,7 @@
       <c r="R6" s="271" t="n"/>
       <c r="S6" s="271" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1" s="243">
+    <row r="7" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A7" s="274" t="n">
         <v>46174</v>
       </c>
@@ -13753,7 +13752,7 @@
       <c r="R8" s="271" t="n"/>
       <c r="S8" s="271" t="n"/>
     </row>
-    <row r="9" ht="15" customHeight="1" s="243">
+    <row r="9" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A9" s="274" t="n">
         <v>46174</v>
       </c>
@@ -13805,7 +13804,7 @@
       <c r="R9" s="271" t="n"/>
       <c r="S9" s="271" t="n"/>
     </row>
-    <row r="10" ht="15" customHeight="1" s="243">
+    <row r="10" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A10" s="274" t="n">
         <v>46174</v>
       </c>
@@ -13853,7 +13852,7 @@
       <c r="R10" s="271" t="n"/>
       <c r="S10" s="271" t="n"/>
     </row>
-    <row r="11" ht="15" customHeight="1" s="243">
+    <row r="11" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A11" s="274" t="n">
         <v>46175</v>
       </c>
@@ -13903,7 +13902,7 @@
       <c r="R11" s="271" t="n"/>
       <c r="S11" s="271" t="n"/>
     </row>
-    <row r="12" ht="15" customHeight="1" s="243">
+    <row r="12" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A12" s="274" t="n">
         <v>46175</v>
       </c>
@@ -13951,7 +13950,7 @@
       <c r="R12" s="271" t="n"/>
       <c r="S12" s="271" t="n"/>
     </row>
-    <row r="13" ht="15" customHeight="1" s="243">
+    <row r="13" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A13" s="274" t="n">
         <v>46175</v>
       </c>
@@ -14001,7 +14000,7 @@
       <c r="R13" s="271" t="n"/>
       <c r="S13" s="271" t="n"/>
     </row>
-    <row r="14" ht="15" customHeight="1" s="243">
+    <row r="14" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A14" s="274" t="n">
         <v>46175</v>
       </c>
@@ -14053,7 +14052,7 @@
       <c r="R14" s="271" t="n"/>
       <c r="S14" s="271" t="n"/>
     </row>
-    <row r="15" ht="15" customHeight="1" s="243">
+    <row r="15" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A15" s="274" t="n">
         <v>46175</v>
       </c>
@@ -14149,7 +14148,7 @@
       <c r="R16" s="271" t="n"/>
       <c r="S16" s="271" t="n"/>
     </row>
-    <row r="17" ht="15" customHeight="1" s="243">
+    <row r="17" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A17" s="274" t="n">
         <v>46175</v>
       </c>
@@ -14199,7 +14198,7 @@
       <c r="R17" s="271" t="n"/>
       <c r="S17" s="271" t="n"/>
     </row>
-    <row r="18" ht="15" customHeight="1" s="243">
+    <row r="18" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A18" s="274" t="n">
         <v>46175</v>
       </c>
@@ -14247,7 +14246,7 @@
       <c r="R18" s="271" t="n"/>
       <c r="S18" s="271" t="n"/>
     </row>
-    <row r="19" ht="15" customHeight="1" s="243">
+    <row r="19" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A19" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14283,7 +14282,7 @@
       <c r="R19" s="271" t="n"/>
       <c r="S19" s="271" t="n"/>
     </row>
-    <row r="20" ht="15" customHeight="1" s="243">
+    <row r="20" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A20" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14319,7 +14318,7 @@
       <c r="R20" s="271" t="n"/>
       <c r="S20" s="271" t="n"/>
     </row>
-    <row r="21" ht="15" customHeight="1" s="243">
+    <row r="21" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A21" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14355,7 +14354,7 @@
       <c r="R21" s="271" t="n"/>
       <c r="S21" s="271" t="n"/>
     </row>
-    <row r="22" ht="15" customHeight="1" s="243">
+    <row r="22" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A22" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14409,7 +14408,7 @@
       <c r="R22" s="271" t="n"/>
       <c r="S22" s="271" t="n"/>
     </row>
-    <row r="23" ht="15" customHeight="1" s="243">
+    <row r="23" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A23" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14445,7 +14444,7 @@
       <c r="R23" s="271" t="n"/>
       <c r="S23" s="271" t="n"/>
     </row>
-    <row r="24" ht="15" customHeight="1" s="243">
+    <row r="24" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A24" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14481,7 +14480,7 @@
       <c r="R24" s="271" t="n"/>
       <c r="S24" s="271" t="n"/>
     </row>
-    <row r="25" ht="15" customHeight="1" s="243">
+    <row r="25" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A25" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14517,7 +14516,7 @@
       <c r="R25" s="271" t="n"/>
       <c r="S25" s="271" t="n"/>
     </row>
-    <row r="26" ht="15" customHeight="1" s="243">
+    <row r="26" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A26" s="274" t="n">
         <v>46177</v>
       </c>
@@ -14553,7 +14552,7 @@
       <c r="R26" s="271" t="n"/>
       <c r="S26" s="271" t="n"/>
     </row>
-    <row r="27" ht="15" customHeight="1" s="243">
+    <row r="27" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A27" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14589,7 +14588,7 @@
       <c r="R27" s="271" t="n"/>
       <c r="S27" s="271" t="n"/>
     </row>
-    <row r="28" ht="15" customHeight="1" s="243">
+    <row r="28" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A28" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14625,7 +14624,7 @@
       <c r="R28" s="271" t="n"/>
       <c r="S28" s="271" t="n"/>
     </row>
-    <row r="29" ht="15" customHeight="1" s="243">
+    <row r="29" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A29" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14661,7 +14660,7 @@
       <c r="R29" s="271" t="n"/>
       <c r="S29" s="271" t="n"/>
     </row>
-    <row r="30" ht="15" customHeight="1" s="243">
+    <row r="30" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A30" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14715,7 +14714,7 @@
       <c r="R30" s="271" t="n"/>
       <c r="S30" s="271" t="n"/>
     </row>
-    <row r="31" ht="15" customHeight="1" s="243">
+    <row r="31" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A31" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14751,7 +14750,7 @@
       <c r="R31" s="271" t="n"/>
       <c r="S31" s="271" t="n"/>
     </row>
-    <row r="32" ht="15" customHeight="1" s="243">
+    <row r="32" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A32" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14787,7 +14786,7 @@
       <c r="R32" s="271" t="n"/>
       <c r="S32" s="271" t="n"/>
     </row>
-    <row r="33" ht="15" customHeight="1" s="243">
+    <row r="33" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A33" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14823,7 +14822,7 @@
       <c r="R33" s="271" t="n"/>
       <c r="S33" s="271" t="n"/>
     </row>
-    <row r="34" ht="15" customHeight="1" s="243">
+    <row r="34" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A34" s="274" t="n">
         <v>46178</v>
       </c>
@@ -14859,7 +14858,7 @@
       <c r="R34" s="271" t="n"/>
       <c r="S34" s="271" t="n"/>
     </row>
-    <row r="35" ht="15" customHeight="1" s="243">
+    <row r="35" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A35" s="274" t="n">
         <v>46179</v>
       </c>
@@ -14895,7 +14894,7 @@
       <c r="R35" s="271" t="n"/>
       <c r="S35" s="271" t="n"/>
     </row>
-    <row r="36" ht="15" customHeight="1" s="243">
+    <row r="36" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A36" s="274" t="n">
         <v>46179</v>
       </c>
@@ -14931,7 +14930,7 @@
       <c r="R36" s="271" t="n"/>
       <c r="S36" s="271" t="n"/>
     </row>
-    <row r="37" ht="15" customHeight="1" s="243">
+    <row r="37" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A37" s="274" t="n">
         <v>46179</v>
       </c>
@@ -14967,7 +14966,7 @@
       <c r="R37" s="271" t="n"/>
       <c r="S37" s="271" t="n"/>
     </row>
-    <row r="38" ht="15" customHeight="1" s="243">
+    <row r="38" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A38" s="274" t="n">
         <v>46179</v>
       </c>
@@ -15023,7 +15022,7 @@
       <c r="R38" s="271" t="n"/>
       <c r="S38" s="271" t="n"/>
     </row>
-    <row r="39" ht="15" customHeight="1" s="243">
+    <row r="39" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A39" s="274" t="n">
         <v>46179</v>
       </c>
@@ -15059,7 +15058,7 @@
       <c r="R39" s="271" t="n"/>
       <c r="S39" s="271" t="n"/>
     </row>
-    <row r="40" ht="15" customHeight="1" s="243">
+    <row r="40" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A40" s="274" t="n">
         <v>46179</v>
       </c>
@@ -15095,7 +15094,7 @@
       <c r="R40" s="271" t="n"/>
       <c r="S40" s="271" t="n"/>
     </row>
-    <row r="41" ht="15" customHeight="1" s="243">
+    <row r="41" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A41" s="274" t="n">
         <v>46179</v>
       </c>
@@ -15131,7 +15130,7 @@
       <c r="R41" s="271" t="n"/>
       <c r="S41" s="271" t="n"/>
     </row>
-    <row r="42" ht="15" customHeight="1" s="243">
+    <row r="42" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A42" s="274" t="n">
         <v>46179</v>
       </c>
@@ -15167,7 +15166,7 @@
       <c r="R42" s="271" t="n"/>
       <c r="S42" s="271" t="n"/>
     </row>
-    <row r="43" ht="15" customHeight="1" s="243">
+    <row r="43" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A43" s="274" t="n">
         <v>46181</v>
       </c>
@@ -15203,7 +15202,7 @@
       <c r="R43" s="271" t="n"/>
       <c r="S43" s="271" t="n"/>
     </row>
-    <row r="44" ht="15" customHeight="1" s="243">
+    <row r="44" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A44" s="274" t="n">
         <v>46181</v>
       </c>
@@ -15251,7 +15250,7 @@
       <c r="R44" s="271" t="n"/>
       <c r="S44" s="271" t="n"/>
     </row>
-    <row r="45" ht="15" customHeight="1" s="243">
+    <row r="45" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A45" s="274" t="n">
         <v>46181</v>
       </c>
@@ -15287,7 +15286,7 @@
       <c r="R45" s="271" t="n"/>
       <c r="S45" s="271" t="n"/>
     </row>
-    <row r="46" ht="15" customHeight="1" s="243">
+    <row r="46" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A46" s="274" t="n">
         <v>46181</v>
       </c>
@@ -15341,7 +15340,7 @@
       <c r="R46" s="271" t="n"/>
       <c r="S46" s="271" t="n"/>
     </row>
-    <row r="47" ht="15" customHeight="1" s="243">
+    <row r="47" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A47" s="274" t="n">
         <v>46181</v>
       </c>
@@ -15425,7 +15424,7 @@
       <c r="R48" s="271" t="n"/>
       <c r="S48" s="271" t="n"/>
     </row>
-    <row r="49" ht="15" customHeight="1" s="243">
+    <row r="49" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A49" s="274" t="n">
         <v>46181</v>
       </c>
@@ -15475,7 +15474,7 @@
       <c r="R49" s="271" t="n"/>
       <c r="S49" s="271" t="n"/>
     </row>
-    <row r="50" ht="15" customHeight="1" s="243">
+    <row r="50" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A50" s="274" t="n">
         <v>46181</v>
       </c>
@@ -15511,7 +15510,7 @@
       <c r="R50" s="271" t="n"/>
       <c r="S50" s="271" t="n"/>
     </row>
-    <row r="51" ht="15" customHeight="1" s="243">
+    <row r="51" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A51" s="274" t="n">
         <v>46182</v>
       </c>
@@ -15547,7 +15546,7 @@
       <c r="R51" s="271" t="n"/>
       <c r="S51" s="271" t="n"/>
     </row>
-    <row r="52" ht="15" customHeight="1" s="243">
+    <row r="52" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A52" s="274" t="n">
         <v>46182</v>
       </c>
@@ -15595,7 +15594,7 @@
       <c r="R52" s="271" t="n"/>
       <c r="S52" s="271" t="n"/>
     </row>
-    <row r="53" ht="15" customHeight="1" s="243">
+    <row r="53" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A53" s="274" t="n">
         <v>46182</v>
       </c>
@@ -15631,7 +15630,7 @@
       <c r="R53" s="271" t="n"/>
       <c r="S53" s="271" t="n"/>
     </row>
-    <row r="54" ht="15" customHeight="1" s="243">
+    <row r="54" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A54" s="274" t="n">
         <v>46182</v>
       </c>
@@ -15685,7 +15684,7 @@
       <c r="R54" s="271" t="n"/>
       <c r="S54" s="271" t="n"/>
     </row>
-    <row r="55" ht="15" customHeight="1" s="243">
+    <row r="55" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A55" s="274" t="n">
         <v>46182</v>
       </c>
@@ -15769,7 +15768,7 @@
       <c r="R56" s="271" t="n"/>
       <c r="S56" s="271" t="n"/>
     </row>
-    <row r="57" ht="15" customHeight="1" s="243">
+    <row r="57" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A57" s="274" t="n">
         <v>46182</v>
       </c>
@@ -15817,7 +15816,7 @@
       <c r="R57" s="271" t="n"/>
       <c r="S57" s="271" t="n"/>
     </row>
-    <row r="58" ht="15" customHeight="1" s="243">
+    <row r="58" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A58" s="274" t="n">
         <v>46182</v>
       </c>
@@ -15853,7 +15852,7 @@
       <c r="R58" s="271" t="n"/>
       <c r="S58" s="271" t="n"/>
     </row>
-    <row r="59" ht="15" customHeight="1" s="243">
+    <row r="59" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A59" s="274" t="n">
         <v>46183</v>
       </c>
@@ -15889,7 +15888,7 @@
       <c r="R59" s="271" t="n"/>
       <c r="S59" s="271" t="n"/>
     </row>
-    <row r="60" ht="15" customHeight="1" s="243">
+    <row r="60" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A60" s="274" t="n">
         <v>46183</v>
       </c>
@@ -15937,7 +15936,7 @@
       <c r="R60" s="271" t="n"/>
       <c r="S60" s="271" t="n"/>
     </row>
-    <row r="61" ht="15" customHeight="1" s="243">
+    <row r="61" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A61" s="274" t="n">
         <v>46183</v>
       </c>
@@ -15973,7 +15972,7 @@
       <c r="R61" s="271" t="n"/>
       <c r="S61" s="271" t="n"/>
     </row>
-    <row r="62" ht="15" customHeight="1" s="243">
+    <row r="62" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A62" s="274" t="n">
         <v>46183</v>
       </c>
@@ -16025,7 +16024,7 @@
       <c r="R62" s="271" t="n"/>
       <c r="S62" s="271" t="n"/>
     </row>
-    <row r="63" ht="15" customHeight="1" s="243">
+    <row r="63" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A63" s="274" t="n">
         <v>46183</v>
       </c>
@@ -16109,7 +16108,7 @@
       <c r="R64" s="271" t="n"/>
       <c r="S64" s="271" t="n"/>
     </row>
-    <row r="65" ht="15" customHeight="1" s="243">
+    <row r="65" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A65" s="274" t="n">
         <v>46183</v>
       </c>
@@ -16157,7 +16156,7 @@
       <c r="R65" s="271" t="n"/>
       <c r="S65" s="271" t="n"/>
     </row>
-    <row r="66" ht="15" customHeight="1" s="243">
+    <row r="66" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A66" s="274" t="n">
         <v>46183</v>
       </c>
@@ -16193,7 +16192,7 @@
       <c r="R66" s="271" t="n"/>
       <c r="S66" s="271" t="n"/>
     </row>
-    <row r="67" ht="15" customHeight="1" s="243">
+    <row r="67" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A67" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16229,7 +16228,7 @@
       <c r="R67" s="271" t="n"/>
       <c r="S67" s="271" t="n"/>
     </row>
-    <row r="68" ht="15" customHeight="1" s="243">
+    <row r="68" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A68" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16279,7 +16278,7 @@
       <c r="R68" s="271" t="n"/>
       <c r="S68" s="271" t="n"/>
     </row>
-    <row r="69" ht="15" customHeight="1" s="243">
+    <row r="69" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A69" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16315,7 +16314,7 @@
       <c r="R69" s="271" t="n"/>
       <c r="S69" s="271" t="n"/>
     </row>
-    <row r="70" ht="15" customHeight="1" s="243">
+    <row r="70" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A70" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16367,7 +16366,7 @@
       <c r="R70" s="271" t="n"/>
       <c r="S70" s="271" t="n"/>
     </row>
-    <row r="71" ht="15" customHeight="1" s="243">
+    <row r="71" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A71" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16453,7 +16452,7 @@
       <c r="R72" s="271" t="n"/>
       <c r="S72" s="271" t="n"/>
     </row>
-    <row r="73" ht="15" customHeight="1" s="243">
+    <row r="73" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A73" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16503,7 +16502,7 @@
       <c r="R73" s="271" t="n"/>
       <c r="S73" s="271" t="n"/>
     </row>
-    <row r="74" ht="15" customHeight="1" s="243">
+    <row r="74" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A74" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16553,7 +16552,7 @@
       <c r="R74" s="271" t="n"/>
       <c r="S74" s="271" t="n"/>
     </row>
-    <row r="75" ht="15" customHeight="1" s="243">
+    <row r="75" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A75" s="274" t="n">
         <v>46184</v>
       </c>
@@ -16589,7 +16588,7 @@
       <c r="R75" s="271" t="n"/>
       <c r="S75" s="271" t="n"/>
     </row>
-    <row r="76" ht="15" customHeight="1" s="243">
+    <row r="76" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A76" s="274" t="n">
         <v>46185</v>
       </c>
@@ -16625,7 +16624,7 @@
       <c r="R76" s="271" t="n"/>
       <c r="S76" s="271" t="n"/>
     </row>
-    <row r="77" ht="15" customHeight="1" s="243">
+    <row r="77" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A77" s="274" t="n">
         <v>46185</v>
       </c>
@@ -16675,7 +16674,7 @@
       <c r="R77" s="271" t="n"/>
       <c r="S77" s="271" t="n"/>
     </row>
-    <row r="78" ht="15" customHeight="1" s="243">
+    <row r="78" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A78" s="274" t="n">
         <v>46185</v>
       </c>
@@ -16711,7 +16710,7 @@
       <c r="R78" s="271" t="n"/>
       <c r="S78" s="271" t="n"/>
     </row>
-    <row r="79" ht="15" customHeight="1" s="243">
+    <row r="79" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A79" s="274" t="n">
         <v>46185</v>
       </c>
@@ -16763,7 +16762,7 @@
       <c r="R79" s="271" t="n"/>
       <c r="S79" s="271" t="n"/>
     </row>
-    <row r="80" ht="15" customHeight="1" s="243">
+    <row r="80" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A80" s="274" t="n">
         <v>46185</v>
       </c>
@@ -16849,7 +16848,7 @@
       <c r="R81" s="271" t="n"/>
       <c r="S81" s="271" t="n"/>
     </row>
-    <row r="82" ht="15" customHeight="1" s="243">
+    <row r="82" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A82" s="274" t="n">
         <v>46185</v>
       </c>
@@ -16899,7 +16898,7 @@
       <c r="R82" s="271" t="n"/>
       <c r="S82" s="271" t="n"/>
     </row>
-    <row r="83" ht="15" customHeight="1" s="243">
+    <row r="83" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A83" s="274" t="n">
         <v>46185</v>
       </c>
@@ -16939,7 +16938,7 @@
       <c r="R83" s="271" t="n"/>
       <c r="S83" s="271" t="n"/>
     </row>
-    <row r="84" ht="15" customHeight="1" s="243">
+    <row r="84" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A84" s="274" t="n">
         <v>46186</v>
       </c>
@@ -16975,7 +16974,7 @@
       <c r="R84" s="271" t="n"/>
       <c r="S84" s="271" t="n"/>
     </row>
-    <row r="85" ht="15" customHeight="1" s="243">
+    <row r="85" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A85" s="274" t="n">
         <v>46186</v>
       </c>
@@ -17023,7 +17022,7 @@
       <c r="R85" s="271" t="n"/>
       <c r="S85" s="271" t="n"/>
     </row>
-    <row r="86" ht="15" customHeight="1" s="243">
+    <row r="86" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A86" s="274" t="n">
         <v>46186</v>
       </c>
@@ -17059,7 +17058,7 @@
       <c r="R86" s="271" t="n"/>
       <c r="S86" s="271" t="n"/>
     </row>
-    <row r="87" ht="15" customHeight="1" s="243">
+    <row r="87" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A87" s="274" t="n">
         <v>46186</v>
       </c>
@@ -17111,7 +17110,7 @@
       <c r="R87" s="271" t="n"/>
       <c r="S87" s="271" t="n"/>
     </row>
-    <row r="88" ht="15" customHeight="1" s="243">
+    <row r="88" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A88" s="274" t="n">
         <v>46186</v>
       </c>
@@ -17195,7 +17194,7 @@
       <c r="R89" s="271" t="n"/>
       <c r="S89" s="271" t="n"/>
     </row>
-    <row r="90" ht="15" customHeight="1" s="243">
+    <row r="90" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A90" s="274" t="n">
         <v>46186</v>
       </c>
@@ -17245,7 +17244,7 @@
       <c r="R90" s="271" t="n"/>
       <c r="S90" s="271" t="n"/>
     </row>
-    <row r="91" ht="15" customHeight="1" s="243">
+    <row r="91" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A91" s="274" t="n">
         <v>46186</v>
       </c>
@@ -17293,7 +17292,7 @@
       <c r="R91" s="271" t="n"/>
       <c r="S91" s="271" t="n"/>
     </row>
-    <row r="92" ht="15" customHeight="1" s="243">
+    <row r="92" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A92" s="274" t="n">
         <v>46186</v>
       </c>
@@ -17333,7 +17332,7 @@
       <c r="R92" s="271" t="n"/>
       <c r="S92" s="271" t="n"/>
     </row>
-    <row r="93" ht="15" customHeight="1" s="243">
+    <row r="93" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A93" s="274" t="n">
         <v>46188</v>
       </c>
@@ -17369,7 +17368,7 @@
       <c r="R93" s="271" t="n"/>
       <c r="S93" s="271" t="n"/>
     </row>
-    <row r="94" ht="15" customHeight="1" s="243">
+    <row r="94" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A94" s="274" t="n">
         <v>46188</v>
       </c>
@@ -17421,7 +17420,7 @@
       <c r="R94" s="271" t="n"/>
       <c r="S94" s="271" t="n"/>
     </row>
-    <row r="95" ht="15" customHeight="1" s="243">
+    <row r="95" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A95" s="274" t="n">
         <v>46188</v>
       </c>
@@ -17457,7 +17456,7 @@
       <c r="R95" s="271" t="n"/>
       <c r="S95" s="271" t="n"/>
     </row>
-    <row r="96" ht="15" customHeight="1" s="243">
+    <row r="96" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A96" s="274" t="n">
         <v>46188</v>
       </c>
@@ -17509,7 +17508,7 @@
       <c r="R96" s="271" t="n"/>
       <c r="S96" s="271" t="n"/>
     </row>
-    <row r="97" ht="15" customHeight="1" s="243">
+    <row r="97" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A97" s="274" t="n">
         <v>46188</v>
       </c>
@@ -17613,7 +17612,7 @@
       <c r="R98" s="271" t="n"/>
       <c r="S98" s="271" t="n"/>
     </row>
-    <row r="99" ht="15" customHeight="1" s="243">
+    <row r="99" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A99" s="274" t="n">
         <v>46188</v>
       </c>
@@ -17663,7 +17662,7 @@
       <c r="R99" s="271" t="n"/>
       <c r="S99" s="271" t="n"/>
     </row>
-    <row r="100" ht="15" customHeight="1" s="243">
+    <row r="100" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A100" s="274" t="n">
         <v>46188</v>
       </c>
@@ -17713,7 +17712,7 @@
       <c r="R100" s="271" t="n"/>
       <c r="S100" s="271" t="n"/>
     </row>
-    <row r="101" ht="15" customHeight="1" s="243">
+    <row r="101" hidden="1" ht="15" customHeight="1" s="243">
       <c r="A101" s="274" t="n">
         <v>46188</v>
       </c>
@@ -19710,7 +19709,18 @@
       <c r="J247" s="91" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:R83"/>
+  <autoFilter ref="A2:R101">
+    <filterColumn colId="1" hiddenButton="0" showButton="1">
+      <filters>
+        <filter val="Press-06"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4" hiddenButton="0" showButton="1">
+      <filters>
+        <filter val="25"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -38713,7 +38723,7 @@
   <cols>
     <col width="10" customWidth="1" style="243" min="1" max="1"/>
     <col width="15.28515625" customWidth="1" style="243" min="2" max="2"/>
-    <col width="33.140625" customWidth="1" style="243" min="3" max="3"/>
+    <col width="33.42578125" customWidth="1" style="243" min="3" max="3"/>
     <col width="6" customWidth="1" style="243" min="4" max="4"/>
     <col width="8.5703125" customWidth="1" style="67" min="5" max="5"/>
     <col width="8.85546875" customWidth="1" style="67" min="6" max="6"/>
@@ -38730,13 +38740,13 @@
           <t>Slugs Inventory — June 2026 MONTH TO DATE</t>
         </is>
       </c>
-      <c r="B1" s="238" t="n"/>
-      <c r="C1" s="238" t="n"/>
-      <c r="D1" s="238" t="n"/>
-      <c r="E1" s="238" t="n"/>
-      <c r="F1" s="238" t="n"/>
-      <c r="G1" s="238" t="n"/>
-      <c r="H1" s="238" t="n"/>
+      <c r="B1" s="231" t="n"/>
+      <c r="C1" s="231" t="n"/>
+      <c r="D1" s="231" t="n"/>
+      <c r="E1" s="231" t="n"/>
+      <c r="F1" s="231" t="n"/>
+      <c r="G1" s="231" t="n"/>
+      <c r="H1" s="231" t="n"/>
       <c r="I1" s="69" t="inlineStr">
         <is>
           <t>Date:</t>
@@ -53102,7 +53112,7 @@
         </is>
       </c>
     </row>
-    <row r="8" customFormat="1" s="252">
+    <row r="8" customFormat="1" s="253">
       <c r="A8" s="127" t="inlineStr">
         <is>
           <t>2</t>
@@ -53134,7 +53144,7 @@
         </is>
       </c>
     </row>
-    <row r="9" customFormat="1" s="252">
+    <row r="9" customFormat="1" s="253">
       <c r="A9" s="126" t="inlineStr">
         <is>
           <t>3</t>
@@ -53166,7 +53176,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customFormat="1" customHeight="1" s="252">
+    <row r="10" ht="24" customFormat="1" customHeight="1" s="253">
       <c r="A10" s="106" t="n"/>
       <c r="B10" s="107" t="inlineStr">
         <is>
@@ -53306,7 +53316,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customFormat="1" customHeight="1" s="252">
+    <row r="15" ht="24" customFormat="1" customHeight="1" s="253">
       <c r="A15" s="126" t="inlineStr">
         <is>
           <t>4</t>
@@ -53366,7 +53376,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="8.1" customFormat="1" customHeight="1" s="252">
+    <row r="17" ht="8.1" customFormat="1" customHeight="1" s="253">
       <c r="A17" s="128" t="n"/>
       <c r="B17" s="129" t="n"/>
       <c r="C17" s="129" t="n"/>
@@ -53374,21 +53384,21 @@
       <c r="E17" s="125" t="n"/>
       <c r="F17" s="125" t="n"/>
     </row>
-    <row r="18" ht="15.95" customFormat="1" customHeight="1" s="252">
+    <row r="18" ht="15.95" customFormat="1" customHeight="1" s="253">
       <c r="A18" s="269" t="inlineStr">
         <is>
           <t>Individual scripts: update_production.py also runs sort_dashboard automatically at the end.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15.95" customFormat="1" customHeight="1" s="252">
+    <row r="19" ht="15.95" customFormat="1" customHeight="1" s="253">
       <c r="A19" s="269" t="inlineStr">
         <is>
           <t>Safety: All scripts check if Excel file is open (lock guard) and warn if source files are stale (&gt;26 hours).</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15.95" customFormat="1" customHeight="1" s="252">
+    <row r="20" ht="15.95" customFormat="1" customHeight="1" s="253">
       <c r="A20" s="269" t="inlineStr">
         <is>
           <t>Logging: All output saved to Logs/ folder with timestamps. Mismatches logged to Logs/mismatches.log.</t>
@@ -55872,8 +55882,8 @@
     <mergeCell ref="A68:F68"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A94:F94"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A110:F110"/>
     <mergeCell ref="A119:F119"/>
   </mergeCells>

</xml_diff>

<commit_message>
Full backup 16/06/2026 12:53:22
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -816,7 +816,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="21"/>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="307">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1598,6 +1598,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -51253,31 +51271,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="243">
-      <c r="A4" s="275" t="n">
+      <c r="A4" s="301" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="275" t="n">
+      <c r="B4" s="301" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="276" t="inlineStr">
+      <c r="C4" s="302" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="276" t="inlineStr">
+      <c r="D4" s="302" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="275" t="inlineStr">
+      <c r="E4" s="301" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="277" t="n">
+      <c r="F4" s="303" t="n">
         <v>18860</v>
       </c>
-      <c r="G4" s="275" t="inlineStr">
+      <c r="G4" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51293,31 +51311,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="243">
-      <c r="A5" s="275" t="n">
+      <c r="A5" s="301" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="275" t="n">
+      <c r="B5" s="301" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="276" t="inlineStr">
+      <c r="C5" s="302" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="276" t="inlineStr">
+      <c r="D5" s="302" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="275" t="inlineStr">
+      <c r="E5" s="301" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="277" t="n">
+      <c r="F5" s="303" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="275" t="inlineStr">
+      <c r="G5" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51333,31 +51351,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="243">
-      <c r="A6" s="275" t="n">
+      <c r="A6" s="301" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="275" t="n">
+      <c r="B6" s="301" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="276" t="inlineStr">
+      <c r="C6" s="302" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="276" t="inlineStr">
+      <c r="D6" s="302" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="275" t="inlineStr">
+      <c r="E6" s="301" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="277" t="n">
+      <c r="F6" s="303" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="275" t="inlineStr">
+      <c r="G6" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51373,31 +51391,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="243">
-      <c r="A7" s="275" t="n">
+      <c r="A7" s="301" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="275" t="n">
+      <c r="B7" s="301" t="n">
         <v>5389</v>
       </c>
-      <c r="C7" s="276" t="inlineStr">
+      <c r="C7" s="302" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D7" s="276" t="inlineStr">
+      <c r="D7" s="302" t="inlineStr">
         <is>
           <t>S-45</t>
         </is>
       </c>
-      <c r="E7" s="275" t="inlineStr">
+      <c r="E7" s="301" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F7" s="277" t="n">
+      <c r="F7" s="303" t="n">
         <v>11088</v>
       </c>
-      <c r="G7" s="275" t="inlineStr">
+      <c r="G7" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51413,31 +51431,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="243">
-      <c r="A8" s="275" t="n">
+      <c r="A8" s="301" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="275" t="n">
+      <c r="B8" s="301" t="n">
         <v>4050</v>
       </c>
-      <c r="C8" s="276" t="inlineStr">
+      <c r="C8" s="302" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D8" s="276" t="inlineStr">
+      <c r="D8" s="302" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E8" s="275" t="inlineStr">
+      <c r="E8" s="301" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="277" t="n">
+      <c r="F8" s="303" t="n">
         <v>9450</v>
       </c>
-      <c r="G8" s="275" t="inlineStr">
+      <c r="G8" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51453,31 +51471,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="243">
-      <c r="A9" s="275" t="n">
+      <c r="A9" s="301" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="275" t="n">
+      <c r="B9" s="301" t="n">
         <v>6337</v>
       </c>
-      <c r="C9" s="276" t="inlineStr">
+      <c r="C9" s="302" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="276" t="inlineStr">
+      <c r="D9" s="302" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="275" t="inlineStr">
+      <c r="E9" s="301" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="277" t="n">
+      <c r="F9" s="303" t="n">
         <v>15680</v>
       </c>
-      <c r="G9" s="275" t="inlineStr">
+      <c r="G9" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51493,31 +51511,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="243">
-      <c r="A10" s="275" t="n">
+      <c r="A10" s="301" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="275" t="n">
+      <c r="B10" s="301" t="n">
         <v>6416</v>
       </c>
-      <c r="C10" s="276" t="inlineStr">
+      <c r="C10" s="302" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D10" s="276" t="inlineStr">
+      <c r="D10" s="302" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E10" s="275" t="inlineStr">
+      <c r="E10" s="301" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F10" s="277" t="n">
+      <c r="F10" s="303" t="n">
         <v>15435</v>
       </c>
-      <c r="G10" s="275" t="inlineStr">
+      <c r="G10" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51533,31 +51551,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="243">
-      <c r="A11" s="275" t="n">
+      <c r="A11" s="301" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="275" t="n">
+      <c r="B11" s="301" t="n">
         <v>5782</v>
       </c>
-      <c r="C11" s="276" t="inlineStr">
+      <c r="C11" s="302" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D11" s="276" t="inlineStr">
+      <c r="D11" s="302" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E11" s="275" t="inlineStr">
+      <c r="E11" s="301" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F11" s="277" t="n">
+      <c r="F11" s="303" t="n">
         <v>63648</v>
       </c>
-      <c r="G11" s="275" t="inlineStr">
+      <c r="G11" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51573,31 +51591,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="243">
-      <c r="A12" s="275" t="n">
+      <c r="A12" s="301" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="275" t="n">
+      <c r="B12" s="301" t="n">
         <v>6531</v>
       </c>
-      <c r="C12" s="276" t="inlineStr">
+      <c r="C12" s="302" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D12" s="276" t="inlineStr">
+      <c r="D12" s="302" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E12" s="275" t="inlineStr">
+      <c r="E12" s="301" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F12" s="277" t="n">
+      <c r="F12" s="303" t="n">
         <v>4380</v>
       </c>
-      <c r="G12" s="275" t="inlineStr">
+      <c r="G12" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51613,31 +51631,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="243">
-      <c r="A13" s="275" t="n">
+      <c r="A13" s="301" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="275" t="n">
+      <c r="B13" s="301" t="n">
         <v>6206</v>
       </c>
-      <c r="C13" s="276" t="inlineStr">
+      <c r="C13" s="302" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D13" s="276" t="inlineStr">
+      <c r="D13" s="302" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E13" s="275" t="inlineStr">
+      <c r="E13" s="301" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F13" s="277" t="n">
+      <c r="F13" s="303" t="n">
         <v>100674</v>
       </c>
-      <c r="G13" s="275" t="inlineStr">
+      <c r="G13" s="301" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51653,31 +51671,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="243">
-      <c r="A14" s="279" t="n">
+      <c r="A14" s="304" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="279" t="n">
+      <c r="B14" s="304" t="n">
         <v>6515</v>
       </c>
-      <c r="C14" s="280" t="inlineStr">
+      <c r="C14" s="305" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D14" s="280" t="inlineStr">
+      <c r="D14" s="305" t="inlineStr">
         <is>
           <t>H.H 100GM</t>
         </is>
       </c>
-      <c r="E14" s="279" t="inlineStr">
+      <c r="E14" s="304" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F14" s="281" t="n">
+      <c r="F14" s="306" t="n">
         <v>38896</v>
       </c>
-      <c r="G14" s="279" t="inlineStr">
+      <c r="G14" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51693,31 +51711,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="243">
-      <c r="A15" s="279" t="n">
+      <c r="A15" s="304" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="279" t="n">
+      <c r="B15" s="304" t="n">
         <v>6530</v>
       </c>
-      <c r="C15" s="280" t="inlineStr">
+      <c r="C15" s="305" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D15" s="280" t="inlineStr">
+      <c r="D15" s="305" t="inlineStr">
         <is>
           <t>V- HC BROWN</t>
         </is>
       </c>
-      <c r="E15" s="279" t="inlineStr">
+      <c r="E15" s="304" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F15" s="281" t="n">
+      <c r="F15" s="306" t="n">
         <v>15000</v>
       </c>
-      <c r="G15" s="279" t="inlineStr">
+      <c r="G15" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51733,31 +51751,31 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="243">
-      <c r="A16" s="279" t="n">
+      <c r="A16" s="304" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="279" t="n">
+      <c r="B16" s="304" t="n">
         <v>5782</v>
       </c>
-      <c r="C16" s="280" t="inlineStr">
+      <c r="C16" s="305" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D16" s="280" t="inlineStr">
+      <c r="D16" s="305" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E16" s="279" t="inlineStr">
+      <c r="E16" s="304" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F16" s="281" t="n">
+      <c r="F16" s="306" t="n">
         <v>10500</v>
       </c>
-      <c r="G16" s="279" t="inlineStr">
+      <c r="G16" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51773,31 +51791,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="243">
-      <c r="A17" s="279" t="n">
+      <c r="A17" s="304" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="279" t="n">
+      <c r="B17" s="304" t="n">
         <v>6624</v>
       </c>
-      <c r="C17" s="280" t="inlineStr">
+      <c r="C17" s="305" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D17" s="280" t="inlineStr">
+      <c r="D17" s="305" t="inlineStr">
         <is>
           <t>S-45 DIA 19MM</t>
         </is>
       </c>
-      <c r="E17" s="279" t="inlineStr">
+      <c r="E17" s="304" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F17" s="281" t="n">
+      <c r="F17" s="306" t="n">
         <v>15288</v>
       </c>
-      <c r="G17" s="279" t="inlineStr">
+      <c r="G17" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51813,31 +51831,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="243">
-      <c r="A18" s="279" t="n">
+      <c r="A18" s="304" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="279" t="n">
+      <c r="B18" s="304" t="n">
         <v>5731</v>
       </c>
-      <c r="C18" s="280" t="inlineStr">
+      <c r="C18" s="305" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="280" t="inlineStr">
+      <c r="D18" s="305" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E18" s="279" t="inlineStr">
+      <c r="E18" s="304" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F18" s="281" t="n">
+      <c r="F18" s="306" t="n">
         <v>37030</v>
       </c>
-      <c r="G18" s="279" t="inlineStr">
+      <c r="G18" s="304" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>

</xml_diff>

<commit_message>
Add daily.py master script and Daily_Update.bat launcher
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -816,7 +816,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="21"/>
   </cellStyleXfs>
-  <cellXfs count="307">
+  <cellXfs count="313">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1616,6 +1616,24 @@
     <xf numFmtId="3" fontId="47" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -51271,31 +51289,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="243">
-      <c r="A4" s="301" t="n">
+      <c r="A4" s="307" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="301" t="n">
+      <c r="B4" s="307" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="302" t="inlineStr">
+      <c r="C4" s="308" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="302" t="inlineStr">
+      <c r="D4" s="308" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="301" t="inlineStr">
+      <c r="E4" s="307" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="303" t="n">
+      <c r="F4" s="309" t="n">
         <v>18860</v>
       </c>
-      <c r="G4" s="301" t="inlineStr">
+      <c r="G4" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51311,31 +51329,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="243">
-      <c r="A5" s="301" t="n">
+      <c r="A5" s="307" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="301" t="n">
+      <c r="B5" s="307" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="302" t="inlineStr">
+      <c r="C5" s="308" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="302" t="inlineStr">
+      <c r="D5" s="308" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="301" t="inlineStr">
+      <c r="E5" s="307" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="303" t="n">
+      <c r="F5" s="309" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="301" t="inlineStr">
+      <c r="G5" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51351,31 +51369,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="243">
-      <c r="A6" s="301" t="n">
+      <c r="A6" s="307" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="301" t="n">
+      <c r="B6" s="307" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="302" t="inlineStr">
+      <c r="C6" s="308" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="302" t="inlineStr">
+      <c r="D6" s="308" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="301" t="inlineStr">
+      <c r="E6" s="307" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="303" t="n">
+      <c r="F6" s="309" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="301" t="inlineStr">
+      <c r="G6" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51391,31 +51409,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="243">
-      <c r="A7" s="301" t="n">
+      <c r="A7" s="307" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="301" t="n">
+      <c r="B7" s="307" t="n">
         <v>5389</v>
       </c>
-      <c r="C7" s="302" t="inlineStr">
+      <c r="C7" s="308" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D7" s="302" t="inlineStr">
+      <c r="D7" s="308" t="inlineStr">
         <is>
           <t>S-45</t>
         </is>
       </c>
-      <c r="E7" s="301" t="inlineStr">
+      <c r="E7" s="307" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F7" s="303" t="n">
+      <c r="F7" s="309" t="n">
         <v>11088</v>
       </c>
-      <c r="G7" s="301" t="inlineStr">
+      <c r="G7" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51431,31 +51449,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="243">
-      <c r="A8" s="301" t="n">
+      <c r="A8" s="307" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="301" t="n">
+      <c r="B8" s="307" t="n">
         <v>4050</v>
       </c>
-      <c r="C8" s="302" t="inlineStr">
+      <c r="C8" s="308" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D8" s="302" t="inlineStr">
+      <c r="D8" s="308" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E8" s="301" t="inlineStr">
+      <c r="E8" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="303" t="n">
+      <c r="F8" s="309" t="n">
         <v>9450</v>
       </c>
-      <c r="G8" s="301" t="inlineStr">
+      <c r="G8" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51471,31 +51489,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="243">
-      <c r="A9" s="301" t="n">
+      <c r="A9" s="307" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="301" t="n">
+      <c r="B9" s="307" t="n">
         <v>6337</v>
       </c>
-      <c r="C9" s="302" t="inlineStr">
+      <c r="C9" s="308" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="302" t="inlineStr">
+      <c r="D9" s="308" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="301" t="inlineStr">
+      <c r="E9" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="303" t="n">
+      <c r="F9" s="309" t="n">
         <v>15680</v>
       </c>
-      <c r="G9" s="301" t="inlineStr">
+      <c r="G9" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51511,31 +51529,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="243">
-      <c r="A10" s="301" t="n">
+      <c r="A10" s="307" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="301" t="n">
+      <c r="B10" s="307" t="n">
         <v>6416</v>
       </c>
-      <c r="C10" s="302" t="inlineStr">
+      <c r="C10" s="308" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D10" s="302" t="inlineStr">
+      <c r="D10" s="308" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E10" s="301" t="inlineStr">
+      <c r="E10" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F10" s="303" t="n">
+      <c r="F10" s="309" t="n">
         <v>15435</v>
       </c>
-      <c r="G10" s="301" t="inlineStr">
+      <c r="G10" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51551,31 +51569,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="243">
-      <c r="A11" s="301" t="n">
+      <c r="A11" s="307" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="301" t="n">
+      <c r="B11" s="307" t="n">
         <v>5782</v>
       </c>
-      <c r="C11" s="302" t="inlineStr">
+      <c r="C11" s="308" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D11" s="302" t="inlineStr">
+      <c r="D11" s="308" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E11" s="301" t="inlineStr">
+      <c r="E11" s="307" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F11" s="303" t="n">
+      <c r="F11" s="309" t="n">
         <v>63648</v>
       </c>
-      <c r="G11" s="301" t="inlineStr">
+      <c r="G11" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51591,31 +51609,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="243">
-      <c r="A12" s="301" t="n">
+      <c r="A12" s="307" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="301" t="n">
+      <c r="B12" s="307" t="n">
         <v>6531</v>
       </c>
-      <c r="C12" s="302" t="inlineStr">
+      <c r="C12" s="308" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D12" s="302" t="inlineStr">
+      <c r="D12" s="308" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E12" s="301" t="inlineStr">
+      <c r="E12" s="307" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F12" s="303" t="n">
+      <c r="F12" s="309" t="n">
         <v>4380</v>
       </c>
-      <c r="G12" s="301" t="inlineStr">
+      <c r="G12" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51631,31 +51649,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="243">
-      <c r="A13" s="301" t="n">
+      <c r="A13" s="307" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="301" t="n">
+      <c r="B13" s="307" t="n">
         <v>6206</v>
       </c>
-      <c r="C13" s="302" t="inlineStr">
+      <c r="C13" s="308" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D13" s="302" t="inlineStr">
+      <c r="D13" s="308" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E13" s="301" t="inlineStr">
+      <c r="E13" s="307" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F13" s="303" t="n">
+      <c r="F13" s="309" t="n">
         <v>100674</v>
       </c>
-      <c r="G13" s="301" t="inlineStr">
+      <c r="G13" s="307" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51671,31 +51689,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="243">
-      <c r="A14" s="304" t="n">
+      <c r="A14" s="310" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="304" t="n">
+      <c r="B14" s="310" t="n">
         <v>6515</v>
       </c>
-      <c r="C14" s="305" t="inlineStr">
+      <c r="C14" s="311" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D14" s="305" t="inlineStr">
+      <c r="D14" s="311" t="inlineStr">
         <is>
           <t>H.H 100GM</t>
         </is>
       </c>
-      <c r="E14" s="304" t="inlineStr">
+      <c r="E14" s="310" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F14" s="306" t="n">
+      <c r="F14" s="312" t="n">
         <v>38896</v>
       </c>
-      <c r="G14" s="304" t="inlineStr">
+      <c r="G14" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51711,31 +51729,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="243">
-      <c r="A15" s="304" t="n">
+      <c r="A15" s="310" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="304" t="n">
+      <c r="B15" s="310" t="n">
         <v>6530</v>
       </c>
-      <c r="C15" s="305" t="inlineStr">
+      <c r="C15" s="311" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D15" s="305" t="inlineStr">
+      <c r="D15" s="311" t="inlineStr">
         <is>
           <t>V- HC BROWN</t>
         </is>
       </c>
-      <c r="E15" s="304" t="inlineStr">
+      <c r="E15" s="310" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F15" s="306" t="n">
+      <c r="F15" s="312" t="n">
         <v>15000</v>
       </c>
-      <c r="G15" s="304" t="inlineStr">
+      <c r="G15" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51751,31 +51769,31 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="243">
-      <c r="A16" s="304" t="n">
+      <c r="A16" s="310" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="304" t="n">
+      <c r="B16" s="310" t="n">
         <v>5782</v>
       </c>
-      <c r="C16" s="305" t="inlineStr">
+      <c r="C16" s="311" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D16" s="305" t="inlineStr">
+      <c r="D16" s="311" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E16" s="304" t="inlineStr">
+      <c r="E16" s="310" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F16" s="306" t="n">
+      <c r="F16" s="312" t="n">
         <v>10500</v>
       </c>
-      <c r="G16" s="304" t="inlineStr">
+      <c r="G16" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51791,31 +51809,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="243">
-      <c r="A17" s="304" t="n">
+      <c r="A17" s="310" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="304" t="n">
+      <c r="B17" s="310" t="n">
         <v>6624</v>
       </c>
-      <c r="C17" s="305" t="inlineStr">
+      <c r="C17" s="311" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D17" s="305" t="inlineStr">
+      <c r="D17" s="311" t="inlineStr">
         <is>
           <t>S-45 DIA 19MM</t>
         </is>
       </c>
-      <c r="E17" s="304" t="inlineStr">
+      <c r="E17" s="310" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F17" s="306" t="n">
+      <c r="F17" s="312" t="n">
         <v>15288</v>
       </c>
-      <c r="G17" s="304" t="inlineStr">
+      <c r="G17" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51831,31 +51849,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="243">
-      <c r="A18" s="304" t="n">
+      <c r="A18" s="310" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="304" t="n">
+      <c r="B18" s="310" t="n">
         <v>5731</v>
       </c>
-      <c r="C18" s="305" t="inlineStr">
+      <c r="C18" s="311" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="305" t="inlineStr">
+      <c r="D18" s="311" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E18" s="304" t="inlineStr">
+      <c r="E18" s="310" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F18" s="306" t="n">
+      <c r="F18" s="312" t="n">
         <v>37030</v>
       </c>
-      <c r="G18" s="304" t="inlineStr">
+      <c r="G18" s="310" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>

</xml_diff>

<commit_message>
Configure WIP prompt to timeout and skip after 2 seconds of inactivity
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -816,7 +816,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="21"/>
   </cellStyleXfs>
-  <cellXfs count="319">
+  <cellXfs count="325">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1652,6 +1652,24 @@
     <xf numFmtId="3" fontId="47" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="10" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="11" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -51307,31 +51325,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="243">
-      <c r="A4" s="313" t="n">
+      <c r="A4" s="319" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="313" t="n">
+      <c r="B4" s="319" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="314" t="inlineStr">
+      <c r="C4" s="320" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="314" t="inlineStr">
+      <c r="D4" s="320" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="313" t="inlineStr">
+      <c r="E4" s="319" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="315" t="n">
+      <c r="F4" s="321" t="n">
         <v>18860</v>
       </c>
-      <c r="G4" s="313" t="inlineStr">
+      <c r="G4" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51347,31 +51365,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="243">
-      <c r="A5" s="313" t="n">
+      <c r="A5" s="319" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="313" t="n">
+      <c r="B5" s="319" t="n">
         <v>5699</v>
       </c>
-      <c r="C5" s="314" t="inlineStr">
+      <c r="C5" s="320" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="314" t="inlineStr">
+      <c r="D5" s="320" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E5" s="313" t="inlineStr">
+      <c r="E5" s="319" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F5" s="315" t="n">
+      <c r="F5" s="321" t="n">
         <v>14790</v>
       </c>
-      <c r="G5" s="313" t="inlineStr">
+      <c r="G5" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51387,31 +51405,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="243">
-      <c r="A6" s="313" t="n">
+      <c r="A6" s="319" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="313" t="n">
+      <c r="B6" s="319" t="n">
         <v>5731</v>
       </c>
-      <c r="C6" s="314" t="inlineStr">
+      <c r="C6" s="320" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="314" t="inlineStr">
+      <c r="D6" s="320" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E6" s="313" t="inlineStr">
+      <c r="E6" s="319" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F6" s="315" t="n">
+      <c r="F6" s="321" t="n">
         <v>13770</v>
       </c>
-      <c r="G6" s="313" t="inlineStr">
+      <c r="G6" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51427,31 +51445,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="243">
-      <c r="A7" s="313" t="n">
+      <c r="A7" s="319" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="313" t="n">
+      <c r="B7" s="319" t="n">
         <v>5389</v>
       </c>
-      <c r="C7" s="314" t="inlineStr">
+      <c r="C7" s="320" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D7" s="314" t="inlineStr">
+      <c r="D7" s="320" t="inlineStr">
         <is>
           <t>S-45</t>
         </is>
       </c>
-      <c r="E7" s="313" t="inlineStr">
+      <c r="E7" s="319" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F7" s="315" t="n">
+      <c r="F7" s="321" t="n">
         <v>11088</v>
       </c>
-      <c r="G7" s="313" t="inlineStr">
+      <c r="G7" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51467,31 +51485,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="243">
-      <c r="A8" s="313" t="n">
+      <c r="A8" s="319" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="313" t="n">
+      <c r="B8" s="319" t="n">
         <v>4050</v>
       </c>
-      <c r="C8" s="314" t="inlineStr">
+      <c r="C8" s="320" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D8" s="314" t="inlineStr">
+      <c r="D8" s="320" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E8" s="313" t="inlineStr">
+      <c r="E8" s="319" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="315" t="n">
+      <c r="F8" s="321" t="n">
         <v>9450</v>
       </c>
-      <c r="G8" s="313" t="inlineStr">
+      <c r="G8" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51507,31 +51525,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="243">
-      <c r="A9" s="313" t="n">
+      <c r="A9" s="319" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="313" t="n">
+      <c r="B9" s="319" t="n">
         <v>6337</v>
       </c>
-      <c r="C9" s="314" t="inlineStr">
+      <c r="C9" s="320" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="314" t="inlineStr">
+      <c r="D9" s="320" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="313" t="inlineStr">
+      <c r="E9" s="319" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="315" t="n">
+      <c r="F9" s="321" t="n">
         <v>15680</v>
       </c>
-      <c r="G9" s="313" t="inlineStr">
+      <c r="G9" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51547,31 +51565,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="243">
-      <c r="A10" s="313" t="n">
+      <c r="A10" s="319" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="313" t="n">
+      <c r="B10" s="319" t="n">
         <v>6416</v>
       </c>
-      <c r="C10" s="314" t="inlineStr">
+      <c r="C10" s="320" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D10" s="314" t="inlineStr">
+      <c r="D10" s="320" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E10" s="313" t="inlineStr">
+      <c r="E10" s="319" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F10" s="315" t="n">
+      <c r="F10" s="321" t="n">
         <v>15435</v>
       </c>
-      <c r="G10" s="313" t="inlineStr">
+      <c r="G10" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51587,31 +51605,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="243">
-      <c r="A11" s="313" t="n">
+      <c r="A11" s="319" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="313" t="n">
+      <c r="B11" s="319" t="n">
         <v>5782</v>
       </c>
-      <c r="C11" s="314" t="inlineStr">
+      <c r="C11" s="320" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D11" s="314" t="inlineStr">
+      <c r="D11" s="320" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E11" s="313" t="inlineStr">
+      <c r="E11" s="319" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F11" s="315" t="n">
+      <c r="F11" s="321" t="n">
         <v>63648</v>
       </c>
-      <c r="G11" s="313" t="inlineStr">
+      <c r="G11" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51627,31 +51645,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="243">
-      <c r="A12" s="313" t="n">
+      <c r="A12" s="319" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="313" t="n">
+      <c r="B12" s="319" t="n">
         <v>6531</v>
       </c>
-      <c r="C12" s="314" t="inlineStr">
+      <c r="C12" s="320" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D12" s="314" t="inlineStr">
+      <c r="D12" s="320" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E12" s="313" t="inlineStr">
+      <c r="E12" s="319" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F12" s="315" t="n">
+      <c r="F12" s="321" t="n">
         <v>4380</v>
       </c>
-      <c r="G12" s="313" t="inlineStr">
+      <c r="G12" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51667,31 +51685,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="243">
-      <c r="A13" s="313" t="n">
+      <c r="A13" s="319" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="313" t="n">
+      <c r="B13" s="319" t="n">
         <v>6206</v>
       </c>
-      <c r="C13" s="314" t="inlineStr">
+      <c r="C13" s="320" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D13" s="314" t="inlineStr">
+      <c r="D13" s="320" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E13" s="313" t="inlineStr">
+      <c r="E13" s="319" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F13" s="315" t="n">
+      <c r="F13" s="321" t="n">
         <v>100674</v>
       </c>
-      <c r="G13" s="313" t="inlineStr">
+      <c r="G13" s="319" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -51707,31 +51725,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="243">
-      <c r="A14" s="316" t="n">
+      <c r="A14" s="322" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="316" t="n">
+      <c r="B14" s="322" t="n">
         <v>6515</v>
       </c>
-      <c r="C14" s="317" t="inlineStr">
+      <c r="C14" s="323" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D14" s="317" t="inlineStr">
+      <c r="D14" s="323" t="inlineStr">
         <is>
           <t>H.H 100GM</t>
         </is>
       </c>
-      <c r="E14" s="316" t="inlineStr">
+      <c r="E14" s="322" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F14" s="318" t="n">
+      <c r="F14" s="324" t="n">
         <v>38896</v>
       </c>
-      <c r="G14" s="316" t="inlineStr">
+      <c r="G14" s="322" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51747,31 +51765,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="243">
-      <c r="A15" s="316" t="n">
+      <c r="A15" s="322" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="316" t="n">
+      <c r="B15" s="322" t="n">
         <v>6530</v>
       </c>
-      <c r="C15" s="317" t="inlineStr">
+      <c r="C15" s="323" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D15" s="317" t="inlineStr">
+      <c r="D15" s="323" t="inlineStr">
         <is>
           <t>V- HC BROWN</t>
         </is>
       </c>
-      <c r="E15" s="316" t="inlineStr">
+      <c r="E15" s="322" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F15" s="318" t="n">
+      <c r="F15" s="324" t="n">
         <v>15000</v>
       </c>
-      <c r="G15" s="316" t="inlineStr">
+      <c r="G15" s="322" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51787,31 +51805,31 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="243">
-      <c r="A16" s="316" t="n">
+      <c r="A16" s="322" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="316" t="n">
+      <c r="B16" s="322" t="n">
         <v>5782</v>
       </c>
-      <c r="C16" s="317" t="inlineStr">
+      <c r="C16" s="323" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D16" s="317" t="inlineStr">
+      <c r="D16" s="323" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E16" s="316" t="inlineStr">
+      <c r="E16" s="322" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F16" s="318" t="n">
+      <c r="F16" s="324" t="n">
         <v>10500</v>
       </c>
-      <c r="G16" s="316" t="inlineStr">
+      <c r="G16" s="322" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51827,31 +51845,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="243">
-      <c r="A17" s="316" t="n">
+      <c r="A17" s="322" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="316" t="n">
+      <c r="B17" s="322" t="n">
         <v>6624</v>
       </c>
-      <c r="C17" s="317" t="inlineStr">
+      <c r="C17" s="323" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D17" s="317" t="inlineStr">
+      <c r="D17" s="323" t="inlineStr">
         <is>
           <t>S-45 DIA 19MM</t>
         </is>
       </c>
-      <c r="E17" s="316" t="inlineStr">
+      <c r="E17" s="322" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F17" s="318" t="n">
+      <c r="F17" s="324" t="n">
         <v>15288</v>
       </c>
-      <c r="G17" s="316" t="inlineStr">
+      <c r="G17" s="322" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -51867,31 +51885,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="243">
-      <c r="A18" s="316" t="n">
+      <c r="A18" s="322" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="316" t="n">
+      <c r="B18" s="322" t="n">
         <v>5731</v>
       </c>
-      <c r="C18" s="317" t="inlineStr">
+      <c r="C18" s="323" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="317" t="inlineStr">
+      <c r="D18" s="323" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E18" s="316" t="inlineStr">
+      <c r="E18" s="322" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F18" s="318" t="n">
+      <c r="F18" s="324" t="n">
         <v>37030</v>
       </c>
-      <c r="G18" s="316" t="inlineStr">
+      <c r="G18" s="322" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>

</xml_diff>

<commit_message>
Reorganize: move Aerosol files to dedicated subfolder
</commit_message>
<xml_diff>
--- a/Tubex_v10_30.xlsx
+++ b/Tubex_v10_30.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Alpha\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_2FD118E5273BD980398C52F038A5143670CB433C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEE6CE1-2821-47C2-88EA-1FDA8EEC944E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4166,12 +4166,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="36" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="36" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="36" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4181,19 +4194,6 @@
     <xf numFmtId="0" fontId="42" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="36" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4215,6 +4215,9 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="21" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -4222,9 +4225,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4708,22 +4708,22 @@
     </row>
     <row r="2" spans="1:29" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="135"/>
-      <c r="B2" s="238" t="s">
+      <c r="B2" s="232" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="231"/>
-      <c r="D2" s="231"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="231"/>
-      <c r="G2" s="233"/>
-      <c r="H2" s="231"/>
-      <c r="I2" s="231"/>
-      <c r="J2" s="231"/>
-      <c r="K2" s="231"/>
-      <c r="L2" s="231"/>
-      <c r="M2" s="231"/>
-      <c r="N2" s="231"/>
-      <c r="O2" s="231"/>
+      <c r="C2" s="233"/>
+      <c r="D2" s="233"/>
+      <c r="E2" s="234"/>
+      <c r="F2" s="233"/>
+      <c r="G2" s="235"/>
+      <c r="H2" s="233"/>
+      <c r="I2" s="233"/>
+      <c r="J2" s="233"/>
+      <c r="K2" s="233"/>
+      <c r="L2" s="233"/>
+      <c r="M2" s="233"/>
+      <c r="N2" s="233"/>
+      <c r="O2" s="233"/>
       <c r="P2" s="135"/>
       <c r="Q2" s="135"/>
       <c r="R2" s="135"/>
@@ -4741,25 +4741,25 @@
     </row>
     <row r="3" spans="1:29" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="135"/>
-      <c r="B3" s="230" t="s">
+      <c r="B3" s="238" t="s">
         <v>196</v>
       </c>
-      <c r="C3" s="231"/>
-      <c r="D3" s="231"/>
-      <c r="E3" s="232"/>
-      <c r="F3" s="231"/>
-      <c r="G3" s="233"/>
-      <c r="H3" s="235">
+      <c r="C3" s="233"/>
+      <c r="D3" s="233"/>
+      <c r="E3" s="234"/>
+      <c r="F3" s="233"/>
+      <c r="G3" s="235"/>
+      <c r="H3" s="240">
         <f ca="1">TODAY()-1</f>
         <v>46196</v>
       </c>
-      <c r="I3" s="231"/>
-      <c r="J3" s="231"/>
-      <c r="K3" s="231"/>
-      <c r="L3" s="231"/>
-      <c r="M3" s="231"/>
-      <c r="N3" s="231"/>
-      <c r="O3" s="231"/>
+      <c r="I3" s="233"/>
+      <c r="J3" s="233"/>
+      <c r="K3" s="233"/>
+      <c r="L3" s="233"/>
+      <c r="M3" s="233"/>
+      <c r="N3" s="233"/>
+      <c r="O3" s="233"/>
       <c r="P3" s="135"/>
       <c r="Q3" s="135"/>
       <c r="R3" s="135"/>
@@ -4807,24 +4807,24 @@
     </row>
     <row r="5" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="135"/>
-      <c r="B5" s="237" t="s">
+      <c r="B5" s="236" t="s">
         <v>197</v>
       </c>
-      <c r="C5" s="231"/>
+      <c r="C5" s="233"/>
       <c r="D5" s="140" t="s">
         <v>198</v>
       </c>
       <c r="E5" s="140"/>
       <c r="F5" s="141"/>
-      <c r="G5" s="237" t="s">
+      <c r="G5" s="236" t="s">
         <v>199</v>
       </c>
-      <c r="H5" s="231"/>
+      <c r="H5" s="233"/>
       <c r="I5" s="142"/>
-      <c r="J5" s="237" t="s">
+      <c r="J5" s="236" t="s">
         <v>200</v>
       </c>
-      <c r="K5" s="231"/>
+      <c r="K5" s="233"/>
       <c r="L5" s="172"/>
       <c r="M5" s="143" t="s">
         <v>201</v>
@@ -4848,28 +4848,28 @@
     </row>
     <row r="6" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="135"/>
-      <c r="B6" s="234">
+      <c r="B6" s="239">
         <f>SUMPRODUCT((Production_Log!$A$3:$A$8963=MAX(Production_Log!$A$3:$A$8963))*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$H$3:$H$8963)</f>
         <v>18480</v>
       </c>
-      <c r="C6" s="231"/>
+      <c r="C6" s="233"/>
       <c r="D6" s="144">
         <f>SUMIF($B$11:$B$63,"TUBE",$H$11:$H$63)</f>
         <v>258034</v>
       </c>
-      <c r="E6" s="234"/>
-      <c r="F6" s="231"/>
+      <c r="E6" s="239"/>
+      <c r="F6" s="233"/>
       <c r="G6" s="145">
         <f t="array" ref="G6">IFERROR(SUMPRODUCT((Production_Log!$F$3:$F$8963&lt;&gt;0)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*Production_Log!$I$3:$I$8963)/SUMPRODUCT((Production_Log!$F$3:$F$8963&lt;&gt;0)*(LEFT(Production_Log!$B$3:$B$8963,5)="Print")*(ISERROR(SEARCH("(Varnish)",Production_Log!$D$3:$D$8963)))*(Production_Log!$H$3:$H$8963+Production_Log!$I$3:$I$8963)),"-")</f>
         <v>2.469686432221584E-2</v>
       </c>
       <c r="H6" s="145"/>
       <c r="I6" s="142"/>
-      <c r="J6" s="234">
+      <c r="J6" s="239">
         <f>SUMIF($B$11:$B$63,"TUBE",$K$11:$K$63)</f>
         <v>384118</v>
       </c>
-      <c r="K6" s="231"/>
+      <c r="K6" s="233"/>
       <c r="L6" s="146"/>
       <c r="M6" s="177" t="s">
         <v>31</v>
@@ -4897,19 +4897,19 @@
     </row>
     <row r="7" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="135"/>
-      <c r="B7" s="236" t="s">
+      <c r="B7" s="241" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="231"/>
+      <c r="C7" s="233"/>
       <c r="D7" s="147" t="s">
         <v>205</v>
       </c>
       <c r="E7" s="147"/>
       <c r="F7" s="148"/>
-      <c r="G7" s="236" t="s">
+      <c r="G7" s="241" t="s">
         <v>206</v>
       </c>
-      <c r="H7" s="231"/>
+      <c r="H7" s="233"/>
       <c r="I7" s="149"/>
       <c r="J7" s="148" t="s">
         <v>200</v>
@@ -4945,28 +4945,28 @@
     </row>
     <row r="8" spans="1:29" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="135"/>
-      <c r="B8" s="239">
+      <c r="B8" s="237">
         <f>SUMPRODUCT((Production_Log!$A$3:$A$8963=MAX(Production_Log!$A$3:$A$8963))*(Production_Log!$B$3:$B$8963="PF Machine")*Production_Log!$H$3:$H$8963)</f>
         <v>7705</v>
       </c>
-      <c r="C8" s="231"/>
+      <c r="C8" s="233"/>
       <c r="D8" s="150">
         <f>SUMIF($B$11:$B$63,"PET",$H$11:$H$63)</f>
         <v>108790</v>
       </c>
-      <c r="E8" s="239"/>
-      <c r="F8" s="231"/>
+      <c r="E8" s="237"/>
+      <c r="F8" s="233"/>
       <c r="G8" s="151">
         <f t="array" ref="G8">IFERROR(SUMPRODUCT((Production_Log!$B$3:$B$8963="PF Machine")*Production_Log!$I$3:$I$8963)/SUMPRODUCT((Production_Log!$B$3:$B$8963="PF Machine")*(Production_Log!$H$3:$H$8963+Production_Log!$I$3:$I$8963)),0)</f>
         <v>6.8658505264960187E-2</v>
       </c>
       <c r="H8" s="151"/>
       <c r="I8" s="149"/>
-      <c r="J8" s="239">
+      <c r="J8" s="237">
         <f>SUMIF($B$11:$B$63,"PET",$K$11:$K$63)</f>
         <v>133480</v>
       </c>
-      <c r="K8" s="231"/>
+      <c r="K8" s="233"/>
       <c r="L8" s="152"/>
       <c r="M8" s="156" t="str">
         <f>IFERROR(INDEX($S$9:$S$23,MATCH(LARGE($U$9:$U$23,2),$U$9:$U$23,0)),"")</f>
@@ -4997,19 +4997,19 @@
     </row>
     <row r="9" spans="1:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="135"/>
-      <c r="B9" s="240" t="s">
+      <c r="B9" s="230" t="s">
         <v>207</v>
       </c>
-      <c r="C9" s="241"/>
-      <c r="D9" s="241"/>
-      <c r="E9" s="241"/>
-      <c r="F9" s="241"/>
-      <c r="G9" s="241"/>
-      <c r="H9" s="241"/>
-      <c r="I9" s="241"/>
-      <c r="J9" s="241"/>
-      <c r="K9" s="241"/>
-      <c r="L9" s="241"/>
+      <c r="C9" s="231"/>
+      <c r="D9" s="231"/>
+      <c r="E9" s="231"/>
+      <c r="F9" s="231"/>
+      <c r="G9" s="231"/>
+      <c r="H9" s="231"/>
+      <c r="I9" s="231"/>
+      <c r="J9" s="231"/>
+      <c r="K9" s="231"/>
+      <c r="L9" s="231"/>
       <c r="M9" s="156" t="str">
         <f>IFERROR(INDEX($S$9:$S$23,MATCH(LARGE($U$9:$U$23,3),$U$9:$U$23,0)),"")</f>
         <v>Changeover</v>
@@ -8787,11 +8787,11 @@
       </c>
       <c r="F21" s="27">
         <f>IFERROR(INDEX(TableInventory[Store Balance],MATCH(A21,TableInventory[Item ID],0)),0)+IFERROR(INDEX(TableInventory[Work In Process],MATCH(A21,TableInventory[Item ID],0)),0)</f>
-        <v>385</v>
+        <v>325</v>
       </c>
       <c r="G21" s="31">
         <f t="shared" si="1"/>
-        <v>-827.70098400000006</v>
+        <v>-887.70098400000006</v>
       </c>
       <c r="H21" s="28" t="str">
         <f>IF(LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A21)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A21)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A21)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A21)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A21)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A21)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A21)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A21)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))&gt;1,LEFT(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A21)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A21)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A21)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A21)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A21)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A21)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A21)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A21)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""),LEN(IF((COUNTIFS(TableBOM[Product ID],$D$3,TableBOM[Item ID],$A21)&gt;0)*($H$3&gt;0),$C$3&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$4,TableBOM[Item ID],$A21)&gt;0)*($H$4&gt;0),$C$4&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$5,TableBOM[Item ID],$A21)&gt;0)*($H$5&gt;0),$C$5&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$6,TableBOM[Item ID],$A21)&gt;0)*($H$6&gt;0),$C$6&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$7,TableBOM[Item ID],$A21)&gt;0)*($H$7&gt;0),$C$7&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$8,TableBOM[Item ID],$A21)&gt;0)*($H$8&gt;0),$C$8&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$9,TableBOM[Item ID],$A21)&gt;0)*($H$9&gt;0),$C$9&amp;", ","") &amp; IF((COUNTIFS(TableBOM[Product ID],$D$10,TableBOM[Item ID],$A21)&gt;0)*($H$10&gt;0),$C$10&amp;", ",""))-2),"")</f>
@@ -10904,7 +10904,7 @@
         <v>525</v>
       </c>
       <c r="G78" s="31">
-        <f t="shared" ref="G78:G109" si="7">F78-E78</f>
+        <f t="shared" ref="G78:G95" si="7">F78-E78</f>
         <v>18.252281600000003</v>
       </c>
       <c r="H78" s="28" t="str">
@@ -18745,7 +18745,7 @@
         <v>0</v>
       </c>
       <c r="J131" s="203" t="str">
-        <f t="shared" ref="J131:J162" si="4">IFERROR(I131/(H131+I131),"")</f>
+        <f t="shared" ref="J131:J161" si="4">IFERROR(I131/(H131+I131),"")</f>
         <v/>
       </c>
       <c r="K131" s="201"/>
@@ -35380,7 +35380,7 @@
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="15.28515625" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
     <col min="5" max="5" width="8.5703125" style="66" customWidth="1"/>
     <col min="6" max="6" width="8.85546875" style="66" customWidth="1"/>
@@ -35395,13 +35395,13 @@
       <c r="A1" s="247" t="s">
         <v>365</v>
       </c>
-      <c r="B1" s="241"/>
-      <c r="C1" s="241"/>
-      <c r="D1" s="241"/>
-      <c r="E1" s="241"/>
-      <c r="F1" s="241"/>
-      <c r="G1" s="241"/>
-      <c r="H1" s="241"/>
+      <c r="B1" s="231"/>
+      <c r="C1" s="231"/>
+      <c r="D1" s="231"/>
+      <c r="E1" s="231"/>
+      <c r="F1" s="231"/>
+      <c r="G1" s="231"/>
+      <c r="H1" s="231"/>
       <c r="I1" s="68" t="s">
         <v>1</v>
       </c>
@@ -35596,12 +35596,10 @@
         <f t="shared" si="0"/>
         <v>325</v>
       </c>
-      <c r="I7" s="37">
-        <v>60</v>
-      </c>
+      <c r="I7" s="37"/>
       <c r="J7" s="37">
         <f>IFERROR(IF(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])=0,"-",ROUND((H7+I7)/(AVERAGEIF(TableBOM[Item ID],A7,TableBOM[Per 1000 Units])/1000),0)),"-")</f>
-        <v>64994</v>
+        <v>54865</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -38117,7 +38115,7 @@
         <v>1</v>
       </c>
       <c r="H78" s="38">
-        <f t="shared" ref="H78:H109" si="3">E78+F78-G78</f>
+        <f t="shared" ref="H78:H94" si="3">E78+F78-G78</f>
         <v>5</v>
       </c>
       <c r="I78" s="37"/>
@@ -45844,15 +45842,15 @@
     </sortState>
   </autoFilter>
   <mergeCells count="9">
+    <mergeCell ref="A92:K92"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A81:K81"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A75:K75"/>
     <mergeCell ref="A34:K34"/>
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A92:K92"/>
-    <mergeCell ref="A23:K23"/>
-    <mergeCell ref="A65:K65"/>
-    <mergeCell ref="A81:K81"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -47566,7 +47564,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="254" t="s">
+      <c r="A1" s="251" t="s">
         <v>618</v>
       </c>
       <c r="B1" s="243"/>
@@ -47576,7 +47574,7 @@
       <c r="F1" s="243"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="253" t="s">
+      <c r="A2" s="254" t="s">
         <v>619</v>
       </c>
       <c r="B2" s="243"/>
@@ -47604,7 +47602,7 @@
       <c r="F4" s="243"/>
     </row>
     <row r="5" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="251" t="s">
+      <c r="A5" s="252" t="s">
         <v>621</v>
       </c>
       <c r="B5" s="243"/>
@@ -47830,34 +47828,34 @@
       <c r="F17" s="124"/>
     </row>
     <row r="18" spans="1:6" s="92" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="251" t="s">
+      <c r="A18" s="252" t="s">
         <v>678</v>
       </c>
-      <c r="B18" s="252"/>
-      <c r="C18" s="252"/>
-      <c r="D18" s="252"/>
-      <c r="E18" s="252"/>
-      <c r="F18" s="252"/>
+      <c r="B18" s="253"/>
+      <c r="C18" s="253"/>
+      <c r="D18" s="253"/>
+      <c r="E18" s="253"/>
+      <c r="F18" s="253"/>
     </row>
     <row r="19" spans="1:6" s="92" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="251" t="s">
+      <c r="A19" s="252" t="s">
         <v>679</v>
       </c>
-      <c r="B19" s="252"/>
-      <c r="C19" s="252"/>
-      <c r="D19" s="252"/>
-      <c r="E19" s="252"/>
-      <c r="F19" s="252"/>
+      <c r="B19" s="253"/>
+      <c r="C19" s="253"/>
+      <c r="D19" s="253"/>
+      <c r="E19" s="253"/>
+      <c r="F19" s="253"/>
     </row>
     <row r="20" spans="1:6" s="92" customFormat="1" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="251" t="s">
+      <c r="A20" s="252" t="s">
         <v>680</v>
       </c>
-      <c r="B20" s="252"/>
-      <c r="C20" s="252"/>
-      <c r="D20" s="252"/>
-      <c r="E20" s="252"/>
-      <c r="F20" s="252"/>
+      <c r="B20" s="253"/>
+      <c r="C20" s="253"/>
+      <c r="D20" s="253"/>
+      <c r="E20" s="253"/>
+      <c r="F20" s="253"/>
     </row>
     <row r="21" spans="1:6" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="129"/>
@@ -49066,7 +49064,7 @@
       <c r="F118" s="243"/>
     </row>
     <row r="119" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="251" t="s">
+      <c r="A119" s="252" t="s">
         <v>850</v>
       </c>
       <c r="B119" s="243"/>
@@ -49691,6 +49689,10 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="A118:F118"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A110:F110"/>
@@ -49707,10 +49709,6 @@
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A128:F128"/>
-    <mergeCell ref="A80:F80"/>
-    <mergeCell ref="A118:F118"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>